<commit_message>
Sync exhaustive PestFlow QA audit tracker
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ref60d392c6b24edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R525eb3c68f1747e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R5ab92722715946f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R493c128e8e3a45c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rb7546f81ff384bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7ecbb78d0b2b4ea8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R5b589089a73b45fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Rf1d7c97691014230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R89a3365ffea14cfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R4eb4f6750f0c4825"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1312,7 +1312,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskTrackerTable" displayName="TaskTrackerTable" ref="A5:Q20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskTrackerTable" displayName="TaskTrackerTable" ref="A5:Q21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Task ID"/>
     <x:tableColumn id="2" name="Phase"/>
@@ -1337,7 +1337,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N86" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1359,7 +1359,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K75" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1378,7 +1378,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Gap ID"/>
     <x:tableColumn id="2" name="Found During Task"/>
@@ -1693,22 +1693,22 @@
     <x:row r="5">
       <x:c r="A5" s="134" t="n">
         <x:f>COUNTA('Task Tracker'!$A$6:$A$200)</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B5" s="135"/>
       <x:c r="C5" s="136" t="n">
         <x:f>COUNTIF('Task Tracker'!$E$6:$E$200,"Done")</x:f>
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D5" s="137"/>
       <x:c r="E5" s="138" t="n">
         <x:f>COUNTIF('Task Tracker'!$E$6:$E$200,"In Progress")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F5" s="139"/>
       <x:c r="G5" s="140" t="n">
         <x:f>COUNTIF('Task Tracker'!$E$6:$E$200,"Blocked")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H5" s="141"/>
     </x:row>
@@ -1761,22 +1761,22 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>62</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>44</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Failed")</x:f>
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F9" s="141"/>
       <x:c r="G9" s="138" t="n">
         <x:f>COUNTIFS('Product Gaps'!$A$6:$A$200,"&lt;&gt;",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Closed",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Resolved",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Mitigated")</x:f>
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H9" s="139"/>
     </x:row>
@@ -1930,30 +1930,30 @@
         <x:v>Product failures and infrastructure failures stay separate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="98" customHeight="1">
+    <x:row r="17" ht="112" customHeight="1">
       <x:c r="A17" s="120" t="str">
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>New runs self-clean 5/5; historical scope is 55 users and 22 companies, read-only inventoried.</x:v>
+        <x:v>Production owner audit is 69/78; branch fixes pass focused 12/12 and full rendered 194/194.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
-        <x:v>Branch</x:v>
+        <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>codex/desktop-qa-guardian @ addd1a6</x:v>
+        <x:v>PestFlow PR #89 plus Browser-Base-QA @ eb251f2 shared with yawbtng.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Activation</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>Approve/decline historical deletion; restore GitHub Actions; then exact-head Checkly, Browserbase, and candidate deploy.</x:v>
+        <x:v>Deploy reviewed fixes; restore Actions; add Browserbase secrets/context; require exact-SHA external gate.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>Draft PR #89 mergeable; cloud jobs remain zero-step blocked and promotion is unclaimed.</x:v>
+        <x:v>No production fix claimed until deployment and a new 78/78 live certification.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2791,7 +2791,7 @@
         <x:v>Critical workflows pass and owner desk renders without fatal drift at 1440, 1280, and 1024 widths.</x:v>
       </x:c>
       <x:c r="E12" s="166" t="str">
-        <x:v>Done</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="F12" s="166" t="str">
         <x:v>Critical</x:v>
@@ -2800,7 +2800,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H12" s="166" t="str">
-        <x:v>Run eight serial Playwright workflows against new.pestflow.org and api.pestflow.org.</x:v>
+        <x:v>Run all 26 owner routes across 1440, 1280, and 1024; preserve complete failure evidence; after fixes deploy and require a 78/78 production rerun.</x:v>
       </x:c>
       <x:c r="I12" s="166" t="str">
         <x:v>Passed</x:v>
@@ -2815,17 +2815,19 @@
         <x:v>1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M12" s="166" t="str">
-        <x:v>https://new.pestflow.org</x:v>
+        <x:v>69/78 production; 12/12 branch focus; owner-route-matrix.json</x:v>
       </x:c>
       <x:c r="N12" s="166" t="str">
-        <x:v>codex/desktop-qa-guardian</x:v>
-      </x:c>
-      <x:c r="O12" s="166"/>
+        <x:v>Pending PestFlow commit; PR #89</x:v>
+      </x:c>
+      <x:c r="O12" s="166" t="str">
+        <x:v>Requires reviewed deploy for final live certification.</x:v>
+      </x:c>
       <x:c r="P12" s="166" t="str">
-        <x:v>8/8 production desktop scenarios passed in 1.9 minutes.</x:v>
+        <x:v>Coverage is implemented and the audit completed. Three production surfaces remain open until the branch fix is deployed and retested.</x:v>
       </x:c>
       <x:c r="Q12" s="167" t="n">
-        <x:v>46215.27099571759</x:v>
+        <x:v>46215.90625</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -3019,14 +3021,16 @@
         <x:v>Risk-selected + full production</x:v>
       </x:c>
       <x:c r="M16" s="166" t="str">
-        <x:v>/private/tmp/pestflow-desktop-qa-guardian/.github/workflows/desktop-qa-release-gate.yml</x:v>
-      </x:c>
-      <x:c r="N16" s="166"/>
+        <x:v>gicheru214/Browser-Base-QA @ eb251f2; PR #89</x:v>
+      </x:c>
+      <x:c r="N16" s="166" t="str">
+        <x:v>Standalone gate is published; PestFlow exact-head release wiring remains pending.</x:v>
+      </x:c>
       <x:c r="O16" s="166" t="str">
-        <x:v>Needs repository/deploy ownership, Browserbase activation, restored GitHub Actions capacity, and exact-head cloud reruns.</x:v>
+        <x:v>Needs Browserbase secrets/context, deploy ownership, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P16" s="166" t="str">
-        <x:v>Reusable exact-SHA gate exists. Current PR and Checkly jobs still finish with zero steps, so promotion remains blocked.</x:v>
+        <x:v>External control plane is real and shared with yawbtng; current production health still lacks deployment.commitSha.</x:v>
       </x:c>
       <x:c r="Q16" s="167" t="n">
         <x:v>46215.27099571759</x:v>
@@ -3240,24 +3244,58 @@
         <x:v>46215.854166666664</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="133"/>
-      <x:c r="B21" s="133"/>
-      <x:c r="C21" s="133"/>
-      <x:c r="D21" s="133"/>
-      <x:c r="E21" s="133"/>
-      <x:c r="F21" s="133"/>
-      <x:c r="G21" s="133"/>
-      <x:c r="H21" s="133"/>
-      <x:c r="I21" s="133"/>
-      <x:c r="J21" s="133"/>
-      <x:c r="K21" s="133"/>
-      <x:c r="L21" s="133"/>
-      <x:c r="M21" s="133"/>
-      <x:c r="N21" s="133"/>
-      <x:c r="O21" s="133"/>
-      <x:c r="P21" s="133"/>
-      <x:c r="Q21" s="165"/>
+    <x:row r="21" ht="118" customHeight="1">
+      <x:c r="A21" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="B21" s="170" t="str">
+        <x:v>Production Fix</x:v>
+      </x:c>
+      <x:c r="C21" s="170" t="str">
+        <x:v>Deploy and certify exhaustive desktop bug fixes</x:v>
+      </x:c>
+      <x:c r="D21" s="170" t="str">
+        <x:v>The reviewed fixes are deployed, all 26 owner routes pass at 1440×900, 1280×800, and 1024×768, Settings branch API has no 5xx, and evidence is tied to the deployed SHA.</x:v>
+      </x:c>
+      <x:c r="E21" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="F21" s="170" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G21" s="170" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="H21" s="170" t="str">
+        <x:v>Review and deploy PR #89, verify deployed commit identity, rerun the 78-check production matrix plus outcome oracles, and require 78/78 before closure.</x:v>
+      </x:c>
+      <x:c r="I21" s="170" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="J21" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="K21" s="170" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="L21" s="170" t="str">
+        <x:v>1440×900; 1280×800; 1024×768</x:v>
+      </x:c>
+      <x:c r="M21" s="170" t="str">
+        <x:v>G-013; G-014; G-015; PR #89</x:v>
+      </x:c>
+      <x:c r="N21" s="170" t="str">
+        <x:v>Pending PestFlow commit; PR #89</x:v>
+      </x:c>
+      <x:c r="O21" s="170" t="str">
+        <x:v>Needs merge/deploy authority, deployed commit identity, and restored GitHub Actions capacity.</x:v>
+      </x:c>
+      <x:c r="P21" s="170" t="str">
+        <x:v>Branch proof is green; current production is deliberately not certified.</x:v>
+      </x:c>
+      <x:c r="Q21" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="133"/>
@@ -5210,7 +5248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11b053891ea4408b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5162b9b440fd4ba5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8615,117 +8653,313 @@
         <x:v>The draft PR remains mergeable and unstable; production inventory success is not a cloud browser certification.</x:v>
       </x:c>
     </x:row>
-    <x:row r="80">
-      <x:c r="A80" s="133"/>
-      <x:c r="B80" s="165"/>
-      <x:c r="C80" s="133"/>
-      <x:c r="D80" s="133"/>
-      <x:c r="E80" s="133"/>
-      <x:c r="F80" s="133"/>
-      <x:c r="G80" s="133"/>
-      <x:c r="H80" s="133"/>
-      <x:c r="I80" s="133"/>
-      <x:c r="J80" s="133"/>
-      <x:c r="K80" s="133"/>
-      <x:c r="L80" s="133"/>
-      <x:c r="M80" s="133"/>
-      <x:c r="N80" s="133"/>
-    </x:row>
-    <x:row r="81">
-      <x:c r="A81" s="133"/>
-      <x:c r="B81" s="165"/>
-      <x:c r="C81" s="133"/>
-      <x:c r="D81" s="133"/>
-      <x:c r="E81" s="133"/>
-      <x:c r="F81" s="133"/>
-      <x:c r="G81" s="133"/>
-      <x:c r="H81" s="133"/>
-      <x:c r="I81" s="133"/>
-      <x:c r="J81" s="133"/>
-      <x:c r="K81" s="133"/>
-      <x:c r="L81" s="133"/>
-      <x:c r="M81" s="133"/>
-      <x:c r="N81" s="133"/>
-    </x:row>
-    <x:row r="82">
-      <x:c r="A82" s="133"/>
-      <x:c r="B82" s="165"/>
-      <x:c r="C82" s="133"/>
-      <x:c r="D82" s="133"/>
-      <x:c r="E82" s="133"/>
-      <x:c r="F82" s="133"/>
-      <x:c r="G82" s="133"/>
-      <x:c r="H82" s="133"/>
-      <x:c r="I82" s="133"/>
-      <x:c r="J82" s="133"/>
-      <x:c r="K82" s="133"/>
-      <x:c r="L82" s="133"/>
-      <x:c r="M82" s="133"/>
-      <x:c r="N82" s="133"/>
-    </x:row>
-    <x:row r="83">
-      <x:c r="A83" s="133"/>
-      <x:c r="B83" s="165"/>
-      <x:c r="C83" s="133"/>
-      <x:c r="D83" s="133"/>
-      <x:c r="E83" s="133"/>
-      <x:c r="F83" s="133"/>
-      <x:c r="G83" s="133"/>
-      <x:c r="H83" s="133"/>
-      <x:c r="I83" s="133"/>
-      <x:c r="J83" s="133"/>
-      <x:c r="K83" s="133"/>
-      <x:c r="L83" s="133"/>
-      <x:c r="M83" s="133"/>
-      <x:c r="N83" s="133"/>
-    </x:row>
-    <x:row r="84">
-      <x:c r="A84" s="133"/>
-      <x:c r="B84" s="165"/>
-      <x:c r="C84" s="133"/>
-      <x:c r="D84" s="133"/>
-      <x:c r="E84" s="133"/>
-      <x:c r="F84" s="133"/>
-      <x:c r="G84" s="133"/>
-      <x:c r="H84" s="133"/>
-      <x:c r="I84" s="133"/>
-      <x:c r="J84" s="133"/>
-      <x:c r="K84" s="133"/>
-      <x:c r="L84" s="133"/>
-      <x:c r="M84" s="133"/>
-      <x:c r="N84" s="133"/>
-    </x:row>
-    <x:row r="85">
-      <x:c r="A85" s="133"/>
-      <x:c r="B85" s="165"/>
-      <x:c r="C85" s="133"/>
-      <x:c r="D85" s="133"/>
-      <x:c r="E85" s="133"/>
-      <x:c r="F85" s="133"/>
-      <x:c r="G85" s="133"/>
-      <x:c r="H85" s="133"/>
-      <x:c r="I85" s="133"/>
-      <x:c r="J85" s="133"/>
-      <x:c r="K85" s="133"/>
-      <x:c r="L85" s="133"/>
-      <x:c r="M85" s="133"/>
-      <x:c r="N85" s="133"/>
-    </x:row>
-    <x:row r="86">
-      <x:c r="A86" s="133"/>
-      <x:c r="B86" s="165"/>
-      <x:c r="C86" s="133"/>
-      <x:c r="D86" s="133"/>
-      <x:c r="E86" s="133"/>
-      <x:c r="F86" s="133"/>
-      <x:c r="G86" s="133"/>
-      <x:c r="H86" s="133"/>
-      <x:c r="I86" s="133"/>
-      <x:c r="J86" s="133"/>
-      <x:c r="K86" s="133"/>
-      <x:c r="L86" s="133"/>
-      <x:c r="M86" s="133"/>
-      <x:c r="N86" s="133"/>
+    <x:row r="80" ht="112" customHeight="1">
+      <x:c r="A80" s="170" t="str">
+        <x:v>AL-075</x:v>
+      </x:c>
+      <x:c r="B80" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="C80" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D80" s="170" t="str">
+        <x:v>Centralize complete owner-route coverage</x:v>
+      </x:c>
+      <x:c r="E80" s="170" t="str">
+        <x:v>Created one 26-route readiness catalog and made both the deterministic production suite and Checkly owner fallback consume it; added policy parity enforcement.</x:v>
+      </x:c>
+      <x:c r="F80" s="170" t="str">
+        <x:v>Playwright + Checkly</x:v>
+      </x:c>
+      <x:c r="G80" s="170" t="str">
+        <x:v>78 deterministic route/width checks defined</x:v>
+      </x:c>
+      <x:c r="H80" s="170" t="str">
+        <x:v>26 owner routes at 1440×900, 1280×800, and 1024×768; failures aggregate so later security, business, and cleanup checks still run.</x:v>
+      </x:c>
+      <x:c r="I80" s="170" t="str">
+        <x:v>Three desktop widths</x:v>
+      </x:c>
+      <x:c r="J80" s="170" t="str">
+        <x:v>qa/guardian/desktop-owner-route-catalog.json</x:v>
+      </x:c>
+      <x:c r="K80" s="170" t="str">
+        <x:v>Pending PestFlow commit; PR #89</x:v>
+      </x:c>
+      <x:c r="L80" s="170" t="str">
+        <x:v>Run the complete live production matrix and classify every failure.</x:v>
+      </x:c>
+      <x:c r="M80" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N80" s="170" t="str">
+        <x:v>The catalog is shared instead of duplicating route lists across two browser systems.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="112" customHeight="1">
+      <x:c r="A81" s="170" t="str">
+        <x:v>AL-076</x:v>
+      </x:c>
+      <x:c r="B81" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="C81" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D81" s="170" t="str">
+        <x:v>Audit all production owner routes</x:v>
+      </x:c>
+      <x:c r="E81" s="170" t="str">
+        <x:v>Executed the expanded deterministic suite against live PestFlow and preserved the complete route matrix plus the remaining business/security and fixture-cleanup evidence.</x:v>
+      </x:c>
+      <x:c r="F81" s="170" t="str">
+        <x:v>Production Playwright</x:v>
+      </x:c>
+      <x:c r="G81" s="170" t="str">
+        <x:v>69/78 route/width contracts passed</x:v>
+      </x:c>
+      <x:c r="H81" s="170" t="str">
+        <x:v>Services, SMS Contacts, and Common Replies failed at all three widths; Settings also emitted first-party GET /companies/branches 500. All later business/security tests passed and cleanup deleted 5/5 accounts.</x:v>
+      </x:c>
+      <x:c r="I81" s="170" t="str">
+        <x:v>1440×900; 1280×800; 1024×768</x:v>
+      </x:c>
+      <x:c r="J81" s="170" t="str">
+        <x:v>artifacts/desktop-critical/owner-route-matrix.json</x:v>
+      </x:c>
+      <x:c r="K81" s="170" t="str">
+        <x:v>PR #89</x:v>
+      </x:c>
+      <x:c r="L81" s="170" t="str">
+        <x:v>Fix the four customer-visible contracts and prove them on the exact branch.</x:v>
+      </x:c>
+      <x:c r="M81" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N81" s="170" t="str">
+        <x:v>Nine failed combinations were three surfaces repeated across three required widths, not nine unrelated bugs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="112" customHeight="1">
+      <x:c r="A82" s="170" t="str">
+        <x:v>AL-077</x:v>
+      </x:c>
+      <x:c r="B82" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="C82" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="D82" s="170" t="str">
+        <x:v>Repair production bugs found by the exhaustive audit</x:v>
+      </x:c>
+      <x:c r="E82" s="170" t="str">
+        <x:v>Added missing layout titles for SMS Contacts/Common Replies, a defensive AppLayout/help-center title contract, and company-scoped branch CRUD routes before the dynamic /companies/:id route.</x:v>
+      </x:c>
+      <x:c r="F82" s="170" t="str">
+        <x:v>PestFlow UI + API</x:v>
+      </x:c>
+      <x:c r="G82" s="170" t="str">
+        <x:v>Root causes fixed on branch</x:v>
+      </x:c>
+      <x:c r="H82" s="170" t="str">
+        <x:v>The undefined title caused both error-boundary screens; the missing literal API route interpreted branches as a company UUID and returned 500. Services readiness was already corrected by the branch version.</x:v>
+      </x:c>
+      <x:c r="I82" s="170" t="str">
+        <x:v>Desktop application</x:v>
+      </x:c>
+      <x:c r="J82" s="170" t="str">
+        <x:v>src/components/AppLayout.tsx; server/routes/companies.ts</x:v>
+      </x:c>
+      <x:c r="K82" s="170" t="str">
+        <x:v>Pending PestFlow commit; PR #89</x:v>
+      </x:c>
+      <x:c r="L82" s="170" t="str">
+        <x:v>Run focused rendered and unit regressions, then the complete desktop suite.</x:v>
+      </x:c>
+      <x:c r="M82" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N82" s="170" t="str">
+        <x:v>Production is not claimed fixed until the reviewed commit is deployed and audited 78/78.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="112" customHeight="1">
+      <x:c r="A83" s="170" t="str">
+        <x:v>AL-078</x:v>
+      </x:c>
+      <x:c r="B83" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="C83" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="D83" s="170" t="str">
+        <x:v>Prove repaired surfaces on the exact branch</x:v>
+      </x:c>
+      <x:c r="E83" s="170" t="str">
+        <x:v>Added contract tests for branch route ordering/isolation and layout-title protection, then rendered Services, SMS Contacts, Common Replies, and Settings at all three required widths.</x:v>
+      </x:c>
+      <x:c r="F83" s="170" t="str">
+        <x:v>Vitest + local Playwright</x:v>
+      </x:c>
+      <x:c r="G83" s="170" t="str">
+        <x:v>Focused regression passed</x:v>
+      </x:c>
+      <x:c r="H83" s="170" t="str">
+        <x:v>7/7 focused unit contracts and 12/12 route/width renders passed with no fatal UI, console error, or horizontal overflow.</x:v>
+      </x:c>
+      <x:c r="I83" s="170" t="str">
+        <x:v>1440×900; 1280×800; 1024×768</x:v>
+      </x:c>
+      <x:c r="J83" s="170" t="str">
+        <x:v>src/test/companyBranchesRoute.test.ts; e2e/staging-feature-pages.spec.ts</x:v>
+      </x:c>
+      <x:c r="K83" s="170" t="str">
+        <x:v>Pending PestFlow commit; PR #89</x:v>
+      </x:c>
+      <x:c r="L83" s="170" t="str">
+        <x:v>Run every broad branch gate because AppLayout is shared across the product.</x:v>
+      </x:c>
+      <x:c r="M83" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N83" s="170" t="str">
+        <x:v>The local server used a strict dedicated port, so another worktree could not supply false evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="112" customHeight="1">
+      <x:c r="A84" s="170" t="str">
+        <x:v>AL-079</x:v>
+      </x:c>
+      <x:c r="B84" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="C84" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D84" s="170" t="str">
+        <x:v>Complete exhaustive branch regression</x:v>
+      </x:c>
+      <x:c r="E84" s="170" t="str">
+        <x:v>Ran the full unit, policy, incident, type, focused lint, build, Checkly bundle, and delegated rendered desktop suites after the shared-layout and API changes.</x:v>
+      </x:c>
+      <x:c r="F84" s="170" t="str">
+        <x:v>Local verification</x:v>
+      </x:c>
+      <x:c r="G84" s="170" t="str">
+        <x:v>All branch gates passed</x:v>
+      </x:c>
+      <x:c r="H84" s="170" t="str">
+        <x:v>760/760 unit, 44/44 policy, 16/16 incident, tsc, focused ESLint, production build, Checkly bundle, and 194/194 rendered desktop tests passed.</x:v>
+      </x:c>
+      <x:c r="I84" s="170" t="str">
+        <x:v>Full desktop catalog</x:v>
+      </x:c>
+      <x:c r="J84" s="170" t="str">
+        <x:v>Local command evidence; PR #89</x:v>
+      </x:c>
+      <x:c r="K84" s="170" t="str">
+        <x:v>Pending PestFlow commit</x:v>
+      </x:c>
+      <x:c r="L84" s="170" t="str">
+        <x:v>Update PRD, code guide, tracker, commit, push, and retry exact-head cloud gates.</x:v>
+      </x:c>
+      <x:c r="M84" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N84" s="170" t="str">
+        <x:v>Build warnings remain separately tracked; no failing branch regression was hidden or quarantined.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="112" customHeight="1">
+      <x:c r="A85" s="170" t="str">
+        <x:v>AL-080</x:v>
+      </x:c>
+      <x:c r="B85" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="C85" s="170" t="str">
+        <x:v>T-003</x:v>
+      </x:c>
+      <x:c r="D85" s="170" t="str">
+        <x:v>Publish standalone Browser Base QA control plane</x:v>
+      </x:c>
+      <x:c r="E85" s="170" t="str">
+        <x:v>Corrected the repository split by publishing the reusable runner, policies, route registry, outcome oracles, workflows, PRD, code guide, and tracker in Browser-Base-QA; verified collaborator access and active workflows.</x:v>
+      </x:c>
+      <x:c r="F85" s="170" t="str">
+        <x:v>GitHub + standalone Node</x:v>
+      </x:c>
+      <x:c r="G85" s="170" t="str">
+        <x:v>Shared repository is operational</x:v>
+      </x:c>
+      <x:c r="H85" s="170" t="str">
+        <x:v>Commit eb251f2 pushed to main; yawbtng has write access and both accounts are CODEOWNERS. 4/4 contracts and 12-entry dry-run matrix passed; workflows parse and are active.</x:v>
+      </x:c>
+      <x:c r="I85" s="170" t="str">
+        <x:v>External PestFlow QA</x:v>
+      </x:c>
+      <x:c r="J85" s="170" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA</x:v>
+      </x:c>
+      <x:c r="K85" s="170" t="str">
+        <x:v>eb251f2</x:v>
+      </x:c>
+      <x:c r="L85" s="170" t="str">
+        <x:v>Add Browserbase secrets/context and deploy PestFlow commit identity before requiring the external gate.</x:v>
+      </x:c>
+      <x:c r="M85" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N85" s="170" t="str">
+        <x:v>Live public oracles passed DB/schema 2/4 and correctly failed missing deployment.commitSha on current production.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="112" customHeight="1">
+      <x:c r="A86" s="170" t="str">
+        <x:v>AL-081</x:v>
+      </x:c>
+      <x:c r="B86" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="C86" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D86" s="170" t="str">
+        <x:v>Document audit results and repository boundary</x:v>
+      </x:c>
+      <x:c r="E86" s="170" t="str">
+        <x:v>Updated the PestFlow Guardian guide, two-part PRD, codebase map, tracker, and activation boundary with exact production, branch, and standalone-repository evidence.</x:v>
+      </x:c>
+      <x:c r="F86" s="170" t="str">
+        <x:v>Documentation + Excel</x:v>
+      </x:c>
+      <x:c r="G86" s="170" t="str">
+        <x:v>Review trail current before publish</x:v>
+      </x:c>
+      <x:c r="H86" s="170" t="str">
+        <x:v>All five workbook tabs rendered and inspected; formula errors are scanned after export. Production remains 69/78 until deploy and rerun despite local branch greens.</x:v>
+      </x:c>
+      <x:c r="I86" s="170" t="str">
+        <x:v>Desktop review</x:v>
+      </x:c>
+      <x:c r="J86" s="170" t="str">
+        <x:v>docs/reliability-command-center; activity workbook</x:v>
+      </x:c>
+      <x:c r="K86" s="170" t="str">
+        <x:v>Pending PestFlow commit</x:v>
+      </x:c>
+      <x:c r="L86" s="170" t="str">
+        <x:v>Commit and push the verified PestFlow branch, then record exact cloud state.</x:v>
+      </x:c>
+      <x:c r="M86" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N86" s="170" t="str">
+        <x:v>This prevents the standalone repository, branch result, and live PestFlow state from being confused again.</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="133"/>
@@ -9341,7 +9575,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ca414e8712d4ee3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf31eace995144a79"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11644,109 +11878,285 @@
         <x:v>Same GitHub payment/spending refusal; exact-head owner proof remains mandatory and unclaimed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="68">
-      <x:c r="A68" s="133"/>
-      <x:c r="B68" s="133"/>
-      <x:c r="C68" s="133"/>
-      <x:c r="D68" s="133"/>
-      <x:c r="E68" s="133"/>
-      <x:c r="F68" s="133"/>
-      <x:c r="G68" s="133"/>
-      <x:c r="H68" s="133"/>
-      <x:c r="I68" s="165"/>
-      <x:c r="J68" s="133"/>
-      <x:c r="K68" s="133"/>
-    </x:row>
-    <x:row r="69">
-      <x:c r="A69" s="133"/>
-      <x:c r="B69" s="133"/>
-      <x:c r="C69" s="133"/>
-      <x:c r="D69" s="133"/>
-      <x:c r="E69" s="133"/>
-      <x:c r="F69" s="133"/>
-      <x:c r="G69" s="133"/>
-      <x:c r="H69" s="133"/>
-      <x:c r="I69" s="165"/>
-      <x:c r="J69" s="133"/>
-      <x:c r="K69" s="133"/>
-    </x:row>
-    <x:row r="70">
-      <x:c r="A70" s="133"/>
-      <x:c r="B70" s="133"/>
-      <x:c r="C70" s="133"/>
-      <x:c r="D70" s="133"/>
-      <x:c r="E70" s="133"/>
-      <x:c r="F70" s="133"/>
-      <x:c r="G70" s="133"/>
-      <x:c r="H70" s="133"/>
-      <x:c r="I70" s="165"/>
-      <x:c r="J70" s="133"/>
-      <x:c r="K70" s="133"/>
-    </x:row>
-    <x:row r="71">
-      <x:c r="A71" s="133"/>
-      <x:c r="B71" s="133"/>
-      <x:c r="C71" s="133"/>
-      <x:c r="D71" s="133"/>
-      <x:c r="E71" s="133"/>
-      <x:c r="F71" s="133"/>
-      <x:c r="G71" s="133"/>
-      <x:c r="H71" s="133"/>
-      <x:c r="I71" s="165"/>
-      <x:c r="J71" s="133"/>
-      <x:c r="K71" s="133"/>
-    </x:row>
-    <x:row r="72">
-      <x:c r="A72" s="133"/>
-      <x:c r="B72" s="133"/>
-      <x:c r="C72" s="133"/>
-      <x:c r="D72" s="133"/>
-      <x:c r="E72" s="133"/>
-      <x:c r="F72" s="133"/>
-      <x:c r="G72" s="133"/>
-      <x:c r="H72" s="133"/>
-      <x:c r="I72" s="165"/>
-      <x:c r="J72" s="133"/>
-      <x:c r="K72" s="133"/>
-    </x:row>
-    <x:row r="73">
-      <x:c r="A73" s="133"/>
-      <x:c r="B73" s="133"/>
-      <x:c r="C73" s="133"/>
-      <x:c r="D73" s="133"/>
-      <x:c r="E73" s="133"/>
-      <x:c r="F73" s="133"/>
-      <x:c r="G73" s="133"/>
-      <x:c r="H73" s="133"/>
-      <x:c r="I73" s="165"/>
-      <x:c r="J73" s="133"/>
-      <x:c r="K73" s="133"/>
-    </x:row>
-    <x:row r="74">
-      <x:c r="A74" s="133"/>
-      <x:c r="B74" s="133"/>
-      <x:c r="C74" s="133"/>
-      <x:c r="D74" s="133"/>
-      <x:c r="E74" s="133"/>
-      <x:c r="F74" s="133"/>
-      <x:c r="G74" s="133"/>
-      <x:c r="H74" s="133"/>
-      <x:c r="I74" s="165"/>
-      <x:c r="J74" s="133"/>
-      <x:c r="K74" s="133"/>
-    </x:row>
-    <x:row r="75">
-      <x:c r="A75" s="133"/>
-      <x:c r="B75" s="133"/>
-      <x:c r="C75" s="133"/>
-      <x:c r="D75" s="133"/>
-      <x:c r="E75" s="133"/>
-      <x:c r="F75" s="133"/>
-      <x:c r="G75" s="133"/>
-      <x:c r="H75" s="133"/>
-      <x:c r="I75" s="165"/>
-      <x:c r="J75" s="133"/>
-      <x:c r="K75" s="133"/>
+    <x:row r="68" ht="80" customHeight="1">
+      <x:c r="A68" s="170" t="str">
+        <x:v>QA-063</x:v>
+      </x:c>
+      <x:c r="B68" s="170" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="C68" s="170" t="str">
+        <x:v>Shared 26-route catalog parity</x:v>
+      </x:c>
+      <x:c r="D68" s="170" t="str">
+        <x:v>26 owner routes</x:v>
+      </x:c>
+      <x:c r="E68" s="170" t="str">
+        <x:v>Node policy</x:v>
+      </x:c>
+      <x:c r="F68" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G68" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H68" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I68" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="J68" s="170" t="str">
+        <x:v>44/44 Guardian policy tests</x:v>
+      </x:c>
+      <x:c r="K68" s="170" t="str">
+        <x:v>Deterministic and Checkly consumers cannot drift from the shared static owner catalog.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="80" customHeight="1">
+      <x:c r="A69" s="170" t="str">
+        <x:v>QA-064</x:v>
+      </x:c>
+      <x:c r="B69" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C69" s="170" t="str">
+        <x:v>Complete owner route/viewport audit</x:v>
+      </x:c>
+      <x:c r="D69" s="170" t="str">
+        <x:v>3 widths × 26 routes</x:v>
+      </x:c>
+      <x:c r="E69" s="170" t="str">
+        <x:v>Playwright Chromium</x:v>
+      </x:c>
+      <x:c r="F69" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G69" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H69" s="170" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="I69" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="J69" s="170" t="str">
+        <x:v>69/78 passed</x:v>
+      </x:c>
+      <x:c r="K69" s="170" t="str">
+        <x:v>Services, SMS Contacts, and Common Replies failed at each width; Settings branch API returned 500.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="80" customHeight="1">
+      <x:c r="A70" s="170" t="str">
+        <x:v>QA-065</x:v>
+      </x:c>
+      <x:c r="B70" s="170" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C70" s="170" t="str">
+        <x:v>Exact repaired desktop surfaces</x:v>
+      </x:c>
+      <x:c r="D70" s="170" t="str">
+        <x:v>4 routes × 3 widths</x:v>
+      </x:c>
+      <x:c r="E70" s="170" t="str">
+        <x:v>Local Playwright Chromium</x:v>
+      </x:c>
+      <x:c r="F70" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G70" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H70" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I70" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="J70" s="170" t="str">
+        <x:v>12/12 passed</x:v>
+      </x:c>
+      <x:c r="K70" s="170" t="str">
+        <x:v>No fatal UI, console error, or horizontal overflow on Services, SMS Contacts, Common Replies, or Settings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="80" customHeight="1">
+      <x:c r="A71" s="170" t="str">
+        <x:v>QA-066</x:v>
+      </x:c>
+      <x:c r="B71" s="170" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C71" s="170" t="str">
+        <x:v>Layout and company-branch contracts</x:v>
+      </x:c>
+      <x:c r="D71" s="170" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="E71" s="170" t="str">
+        <x:v>Vitest</x:v>
+      </x:c>
+      <x:c r="F71" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G71" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H71" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I71" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="J71" s="170" t="str">
+        <x:v>7/7 focused tests</x:v>
+      </x:c>
+      <x:c r="K71" s="170" t="str">
+        <x:v>Route ordering/isolation, validation, primary protection, title fallback, and feature titles are locked.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="80" customHeight="1">
+      <x:c r="A72" s="170" t="str">
+        <x:v>QA-067</x:v>
+      </x:c>
+      <x:c r="B72" s="170" t="str">
+        <x:v>Quality</x:v>
+      </x:c>
+      <x:c r="C72" s="170" t="str">
+        <x:v>Complete branch code gates</x:v>
+      </x:c>
+      <x:c r="D72" s="170" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="E72" s="170" t="str">
+        <x:v>Vitest + Node + tsc + ESLint + Vite</x:v>
+      </x:c>
+      <x:c r="F72" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G72" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="H72" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I72" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="J72" s="170" t="str">
+        <x:v>760 unit; 44 policy; 16 incident</x:v>
+      </x:c>
+      <x:c r="K72" s="170" t="str">
+        <x:v>TypeScript, focused lint, production build, and Checkly bundle also exited 0.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="80" customHeight="1">
+      <x:c r="A73" s="170" t="str">
+        <x:v>QA-068</x:v>
+      </x:c>
+      <x:c r="B73" s="170" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C73" s="170" t="str">
+        <x:v>Complete rendered desktop catalog</x:v>
+      </x:c>
+      <x:c r="D73" s="170" t="str">
+        <x:v>194 behaviors</x:v>
+      </x:c>
+      <x:c r="E73" s="170" t="str">
+        <x:v>Local Playwright Chromium</x:v>
+      </x:c>
+      <x:c r="F73" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G73" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="H73" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I73" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="J73" s="170" t="str">
+        <x:v>194/194 passed in 6.7m</x:v>
+      </x:c>
+      <x:c r="K73" s="170" t="str">
+        <x:v>Shared AppLayout changes did not regress the delegated feature catalog.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="80" customHeight="1">
+      <x:c r="A74" s="170" t="str">
+        <x:v>QA-069</x:v>
+      </x:c>
+      <x:c r="B74" s="170" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="C74" s="170" t="str">
+        <x:v>Standalone Browser Base QA foundation</x:v>
+      </x:c>
+      <x:c r="D74" s="170" t="str">
+        <x:v>12 journey/device entries</x:v>
+      </x:c>
+      <x:c r="E74" s="170" t="str">
+        <x:v>Node + YAML</x:v>
+      </x:c>
+      <x:c r="F74" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G74" s="170" t="str">
+        <x:v>T-003</x:v>
+      </x:c>
+      <x:c r="H74" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I74" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="J74" s="170" t="str">
+        <x:v>4/4 contracts; 12-entry dry run</x:v>
+      </x:c>
+      <x:c r="K74" s="170" t="str">
+        <x:v>Commit eb251f2 is on main; yawbtng has write access; scheduled and reusable workflows are active.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="80" customHeight="1">
+      <x:c r="A75" s="170" t="str">
+        <x:v>QA-070</x:v>
+      </x:c>
+      <x:c r="B75" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C75" s="170" t="str">
+        <x:v>Standalone public PestFlow oracles</x:v>
+      </x:c>
+      <x:c r="D75" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="E75" s="170" t="str">
+        <x:v>Read-only HTTP</x:v>
+      </x:c>
+      <x:c r="F75" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G75" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H75" s="170" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="I75" s="171" t="n">
+        <x:v>46215.90625</x:v>
+      </x:c>
+      <x:c r="J75" s="170" t="str">
+        <x:v>2/4 passed</x:v>
+      </x:c>
+      <x:c r="K75" s="170" t="str">
+        <x:v>DB/schema pass; currently deployed frontend/API health omit deployment.commitSha and therefore fail closed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="133"/>
@@ -12451,7 +12861,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca459fdbd85a4d52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra14041bb4ca04694"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13078,6 +13488,120 @@
       </x:c>
       <x:c r="L18" s="174" t="str">
         <x:v>Scope is now quantified. Deletion remains blocked on explicit authority; new runs already self-clean 5/5.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="116" customHeight="1">
+      <x:c r="A19" s="174" t="str">
+        <x:v>G-013</x:v>
+      </x:c>
+      <x:c r="B19" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="C19" s="174" t="str">
+        <x:v>Desktop Runtime</x:v>
+      </x:c>
+      <x:c r="D19" s="174" t="str">
+        <x:v>SMS Contacts and Common Replies crash in current production because they omit the AppLayout title expected by the shared help center.</x:v>
+      </x:c>
+      <x:c r="E19" s="174" t="str">
+        <x:v>Owners see an error boundary instead of messaging tools at every required desktop width.</x:v>
+      </x:c>
+      <x:c r="F19" s="174" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G19" s="174" t="str">
+        <x:v>Deploy the feature titles and defensive AppLayout/help-center contract, then prove both routes at three widths.</x:v>
+      </x:c>
+      <x:c r="H19" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I19" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="J19" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K19" s="174" t="str">
+        <x:v>Branch fixed; 12/12 focused renders and 194/194 full suite pass.</x:v>
+      </x:c>
+      <x:c r="L19" s="174" t="str">
+        <x:v>Production certification pending deploy and 78/78 rerun.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="116" customHeight="1">
+      <x:c r="A20" s="174" t="str">
+        <x:v>G-014</x:v>
+      </x:c>
+      <x:c r="B20" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="C20" s="174" t="str">
+        <x:v>Desktop API</x:v>
+      </x:c>
+      <x:c r="D20" s="174" t="str">
+        <x:v>Settings GET /companies/branches returns 500 because the literal route is missing and /companies/:id interprets branches as a UUID.</x:v>
+      </x:c>
+      <x:c r="E20" s="174" t="str">
+        <x:v>Branch management cannot load reliably and the production audit records a first-party server failure.</x:v>
+      </x:c>
+      <x:c r="F20" s="174" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G20" s="174" t="str">
+        <x:v>Deploy company-scoped branch CRUD routes before /:id and verify no Settings 5xx in the live matrix.</x:v>
+      </x:c>
+      <x:c r="H20" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I20" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="J20" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K20" s="174" t="str">
+        <x:v>Branch route contract tests pass 5/5.</x:v>
+      </x:c>
+      <x:c r="L20" s="174" t="str">
+        <x:v>Production certification pending deploy and exact-SHA oracle proof.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="116" customHeight="1">
+      <x:c r="A21" s="174" t="str">
+        <x:v>G-015</x:v>
+      </x:c>
+      <x:c r="B21" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="C21" s="174" t="str">
+        <x:v>Desktop Accessibility</x:v>
+      </x:c>
+      <x:c r="D21" s="174" t="str">
+        <x:v>The currently served Services screen does not expose the readiness heading required by its route contract.</x:v>
+      </x:c>
+      <x:c r="E21" s="174" t="str">
+        <x:v>Users and assistive/browser automation lack a stable page identity; production fails this surface at all three widths.</x:v>
+      </x:c>
+      <x:c r="F21" s="174" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="G21" s="174" t="str">
+        <x:v>Deploy the branch Services heading and keep the shared readiness catalog assertion.</x:v>
+      </x:c>
+      <x:c r="H21" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I21" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="J21" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K21" s="174" t="str">
+        <x:v>Branch Services render passes at all three widths.</x:v>
+      </x:c>
+      <x:c r="L21" s="174" t="str">
+        <x:v>Production certification pending deploy and 78/78 rerun.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13114,7 +13638,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9b98b176f7940bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R306ce1f4fa194eb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Sync final PestFlow QA evidence
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7ecbb78d0b2b4ea8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R5b589089a73b45fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Rf1d7c97691014230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R89a3365ffea14cfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R4eb4f6750f0c4825"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4c05d42b95a247ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R65e91ff8202940c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R79a04e22a7b64b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R33b7bd7df07a496a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R3c4c14f1d0264eca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1337,7 +1337,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N86" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N88" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1359,7 +1359,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K75" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1761,7 +1761,7 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>70</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
@@ -1930,30 +1930,30 @@
         <x:v>Product failures and infrastructure failures stay separate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="112" customHeight="1">
+    <x:row r="17" ht="118" customHeight="1">
       <x:c r="A17" s="120" t="str">
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Production owner audit is 69/78; branch fixes pass focused 12/12 and full rendered 194/194.</x:v>
+        <x:v>Historical production audit 69/78; merged head has 27 routes/81 checks and passes focused 15/15 plus full 194/194.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 plus Browser-Base-QA @ eb251f2 shared with yawbtng.</x:v>
+        <x:v>PestFlow PR #89 @ b10e176; Browser-Base-QA @ a468b1a shared with yawbtng.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Activation</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>Deploy reviewed fixes; restore Actions; add Browserbase secrets/context; require exact-SHA external gate.</x:v>
+        <x:v>Restore Actions; deploy reviewed fixes; add Browserbase secrets/context; require exact-SHA external gate and 81/81.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>No production fix claimed until deployment and a new 78/78 live certification.</x:v>
+        <x:v>Draft PR mergeable/unstable; exact-head runs 29210282667 and 29210311515 were zero-step billing blocked.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2070,12 +2070,12 @@
         <x:v>The reviewer can understand what changed and why.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="42" customHeight="1">
+    <x:row r="23" ht="62" customHeight="1">
       <x:c r="A23" s="117" t="str">
         <x:v>Note</x:v>
       </x:c>
       <x:c r="B23" s="118" t="str">
-        <x:v>Production deterministic baseline is green.</x:v>
+        <x:v>Original critical workflows are green; the exhaustive live owner matrix remains red at 69/78 until the reviewed fixes deploy.</x:v>
       </x:c>
       <x:c r="C23" s="118" t="str">
         <x:v>Note</x:v>
@@ -2788,7 +2788,7 @@
         <x:v>Expand deterministic desktop production coverage</x:v>
       </x:c>
       <x:c r="D12" s="166" t="str">
-        <x:v>Critical workflows pass and owner desk renders without fatal drift at 1440, 1280, and 1024 widths.</x:v>
+        <x:v>All static owner routes are audited at three widths, complete failure evidence is preserved, and the deployed reviewed head passes the current dynamic matrix.</x:v>
       </x:c>
       <x:c r="E12" s="166" t="str">
         <x:v>In Progress</x:v>
@@ -2800,7 +2800,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H12" s="166" t="str">
-        <x:v>Run all 26 owner routes across 1440, 1280, and 1024; preserve complete failure evidence; after fixes deploy and require a 78/78 production rerun.</x:v>
+        <x:v>Run all 27 owner routes across 1440, 1280, and 1024; preserve complete failure evidence; after fixes deploy and require an 81/81 production rerun.</x:v>
       </x:c>
       <x:c r="I12" s="166" t="str">
         <x:v>Passed</x:v>
@@ -2815,19 +2815,19 @@
         <x:v>1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M12" s="166" t="str">
-        <x:v>69/78 production; 12/12 branch focus; owner-route-matrix.json</x:v>
+        <x:v>69/78 historical production; 15/15 merged-branch focus; current target 81/81</x:v>
       </x:c>
       <x:c r="N12" s="166" t="str">
-        <x:v>Pending PestFlow commit; PR #89</x:v>
+        <x:v>b10e176; PR #89</x:v>
       </x:c>
       <x:c r="O12" s="166" t="str">
         <x:v>Requires reviewed deploy for final live certification.</x:v>
       </x:c>
       <x:c r="P12" s="166" t="str">
-        <x:v>Coverage is implemented and the audit completed. Three production surfaces remain open until the branch fix is deployed and retested.</x:v>
+        <x:v>Coverage automatically absorbed Move-In Assistant from current main. Historical audit remains red until deploy and all 81 checks pass.</x:v>
       </x:c>
       <x:c r="Q12" s="167" t="n">
-        <x:v>46215.90625</x:v>
+        <x:v>46215.913194444445</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2922,14 +2922,14 @@
         <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/pull/89</x:v>
       </x:c>
       <x:c r="N14" s="166" t="str">
-        <x:v>All Guardian checkpoints through addd1a6 pushed; PR #89</x:v>
+        <x:v>b10e176; PR #89</x:v>
       </x:c>
       <x:c r="O14" s="166"/>
       <x:c r="P14" s="166" t="str">
-        <x:v>753/753 unit, 44/44 policy, 16/16 incident, 8/8 production workflows, 5/5 new-fixture cleanup, and read-only historical inventory pass. Cloud jobs remain zero-step blocked.</x:v>
+        <x:v>769/769 unit, 44/44 policy, 16/16 incident, 15/15 focused renders, 194/194 full desktop, build/type/lint/Checkly green; cloud zero-step blocked.</x:v>
       </x:c>
       <x:c r="Q14" s="167" t="n">
-        <x:v>46215.28418983796</x:v>
+        <x:v>46215.913194444445</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -3021,16 +3021,16 @@
         <x:v>Risk-selected + full production</x:v>
       </x:c>
       <x:c r="M16" s="166" t="str">
-        <x:v>gicheru214/Browser-Base-QA @ eb251f2; PR #89</x:v>
+        <x:v>Browser-Base-QA @ a468b1a; PR #89 @ b10e176</x:v>
       </x:c>
       <x:c r="N16" s="166" t="str">
-        <x:v>Standalone gate is published; PestFlow exact-head release wiring remains pending.</x:v>
+        <x:v>Standalone gate and merged PestFlow head are published; production promotion wiring remains pending.</x:v>
       </x:c>
       <x:c r="O16" s="166" t="str">
         <x:v>Needs Browserbase secrets/context, deploy ownership, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P16" s="166" t="str">
-        <x:v>External control plane is real and shared with yawbtng; current production health still lacks deployment.commitSha.</x:v>
+        <x:v>Current catalog has 27 routes. Production health still lacks deployment.commitSha until reviewed PestFlow work is deployed.</x:v>
       </x:c>
       <x:c r="Q16" s="167" t="n">
         <x:v>46215.27099571759</x:v>
@@ -3161,7 +3161,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H19" s="170" t="str">
-        <x:v>Restore GitHub runner access, then execute the expanded 26-path owner proof and complete Checkly catalog at the exact final SHA; inspect route timings and first-party network evidence.</x:v>
+        <x:v>Restore GitHub runner access, then execute the expanded 27-path owner proof and complete Checkly catalog at the exact final SHA; inspect route timings and first-party network evidence.</x:v>
       </x:c>
       <x:c r="I19" s="170" t="str">
         <x:v>Passed</x:v>
@@ -3176,16 +3176,16 @@
         <x:v>1366×900 cloud; 1440/1280/1024 local</x:v>
       </x:c>
       <x:c r="M19" s="170" t="str">
-        <x:v>44/44 policy; 8/8 production with cleanup 5/5; runs 29207823858 and 29207830428</x:v>
+        <x:v>44/44 policy; 27-path parity; runs 29210282667 and 29210311515</x:v>
       </x:c>
       <x:c r="N19" s="170" t="str">
-        <x:v>addd1a6; PR #89</x:v>
+        <x:v>b10e176; PR #89</x:v>
       </x:c>
       <x:c r="O19" s="170" t="str">
         <x:v>GitHub Actions payment/spending limit prevents cloud job steps from starting.</x:v>
       </x:c>
       <x:c r="P19" s="170" t="str">
-        <x:v>All 26 static owner paths retain fallback parity; exact-head cloud proof is still deliberately unclaimed.</x:v>
+        <x:v>The final head includes Move-In Assistant and requires a 27-route cloud confirmation after runner access returns.</x:v>
       </x:c>
       <x:c r="Q19" s="171" t="n">
         <x:v>46215.82638888889</x:v>
@@ -3255,7 +3255,7 @@
         <x:v>Deploy and certify exhaustive desktop bug fixes</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
-        <x:v>The reviewed fixes are deployed, all 26 owner routes pass at 1440×900, 1280×800, and 1024×768, Settings branch API has no 5xx, and evidence is tied to the deployed SHA.</x:v>
+        <x:v>The reviewed fixes are deployed, all 27 owner routes pass at 1440×900, 1280×800, and 1024×768, Settings branch API has no 5xx, and evidence is tied to the deployed SHA.</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
         <x:v>Blocked</x:v>
@@ -3267,7 +3267,7 @@
         <x:v>Trevor + Codex</x:v>
       </x:c>
       <x:c r="H21" s="170" t="str">
-        <x:v>Review and deploy PR #89, verify deployed commit identity, rerun the 78-check production matrix plus outcome oracles, and require 78/78 before closure.</x:v>
+        <x:v>Review and deploy PR #89, verify deployed commit identity, rerun the 81-check production matrix plus outcome oracles, and require 81/81 before closure.</x:v>
       </x:c>
       <x:c r="I21" s="170" t="str">
         <x:v>Pending</x:v>
@@ -3282,19 +3282,19 @@
         <x:v>1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M21" s="170" t="str">
-        <x:v>G-013; G-014; G-015; PR #89</x:v>
+        <x:v>G-013; G-014; G-015; PR #89 @ b10e176</x:v>
       </x:c>
       <x:c r="N21" s="170" t="str">
-        <x:v>Pending PestFlow commit; PR #89</x:v>
+        <x:v>b10e176; PR #89</x:v>
       </x:c>
       <x:c r="O21" s="170" t="str">
         <x:v>Needs merge/deploy authority, deployed commit identity, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P21" s="170" t="str">
-        <x:v>Branch proof is green; current production is deliberately not certified.</x:v>
+        <x:v>Merged branch proof is green; current production is deliberately not certified. Move-In Assistant is included in the 81-check target.</x:v>
       </x:c>
       <x:c r="Q21" s="171" t="n">
-        <x:v>46215.90625</x:v>
+        <x:v>46215.913194444445</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -5248,7 +5248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5162b9b440fd4ba5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde96a1f3366a454c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8808,7 +8808,7 @@
         <x:v>Focused regression passed</x:v>
       </x:c>
       <x:c r="H83" s="170" t="str">
-        <x:v>7/7 focused unit contracts and 12/12 route/width renders passed with no fatal UI, console error, or horizontal overflow.</x:v>
+        <x:v>10/10 focused unit contracts and 15/15 route/width renders passed across Services, SMS Contacts, Common Replies, Settings, and the newer Move-In Assistant.</x:v>
       </x:c>
       <x:c r="I83" s="170" t="str">
         <x:v>1440×900; 1280×800; 1024×768</x:v>
@@ -8817,7 +8817,7 @@
         <x:v>src/test/companyBranchesRoute.test.ts; e2e/staging-feature-pages.spec.ts</x:v>
       </x:c>
       <x:c r="K83" s="170" t="str">
-        <x:v>Pending PestFlow commit; PR #89</x:v>
+        <x:v>b10e176; PR #89</x:v>
       </x:c>
       <x:c r="L83" s="170" t="str">
         <x:v>Run every broad branch gate because AppLayout is shared across the product.</x:v>
@@ -8852,7 +8852,7 @@
         <x:v>All branch gates passed</x:v>
       </x:c>
       <x:c r="H84" s="170" t="str">
-        <x:v>760/760 unit, 44/44 policy, 16/16 incident, tsc, focused ESLint, production build, Checkly bundle, and 194/194 rendered desktop tests passed.</x:v>
+        <x:v>769/769 unit, 44/44 policy, 16/16 incident, TypeScript, focused ESLint, production build, Checkly bundle, and an uncontended 194/194 rendered desktop rerun passed.</x:v>
       </x:c>
       <x:c r="I84" s="170" t="str">
         <x:v>Full desktop catalog</x:v>
@@ -8861,7 +8861,7 @@
         <x:v>Local command evidence; PR #89</x:v>
       </x:c>
       <x:c r="K84" s="170" t="str">
-        <x:v>Pending PestFlow commit</x:v>
+        <x:v>b10e176; PR #89</x:v>
       </x:c>
       <x:c r="L84" s="170" t="str">
         <x:v>Update PRD, code guide, tracker, commit, push, and retry exact-head cloud gates.</x:v>
@@ -8896,7 +8896,7 @@
         <x:v>Shared repository is operational</x:v>
       </x:c>
       <x:c r="H85" s="170" t="str">
-        <x:v>Commit eb251f2 pushed to main; yawbtng has write access and both accounts are CODEOWNERS. 4/4 contracts and 12-entry dry-run matrix passed; workflows parse and are active.</x:v>
+        <x:v>Browser-Base-QA commits eb251f2, 7284800, and a468b1a are on main; yawbtng has write access and both accounts are CODEOWNERS.</x:v>
       </x:c>
       <x:c r="I85" s="170" t="str">
         <x:v>External PestFlow QA</x:v>
@@ -8905,7 +8905,7 @@
         <x:v>https://github.com/gicheru214/Browser-Base-QA</x:v>
       </x:c>
       <x:c r="K85" s="170" t="str">
-        <x:v>eb251f2</x:v>
+        <x:v>a468b1a</x:v>
       </x:c>
       <x:c r="L85" s="170" t="str">
         <x:v>Add Browserbase secrets/context and deploy PestFlow commit identity before requiring the external gate.</x:v>
@@ -8940,7 +8940,7 @@
         <x:v>Review trail current before publish</x:v>
       </x:c>
       <x:c r="H86" s="170" t="str">
-        <x:v>All five workbook tabs rendered and inspected; formula errors are scanned after export. Production remains 69/78 until deploy and rerun despite local branch greens.</x:v>
+        <x:v>All five workbook tabs rendered and inspected with no formula errors. Current catalog is 27 routes/81 width checks; historical live evidence remains 69/78 until deploy and rerun.</x:v>
       </x:c>
       <x:c r="I86" s="170" t="str">
         <x:v>Desktop review</x:v>
@@ -8949,7 +8949,7 @@
         <x:v>docs/reliability-command-center; activity workbook</x:v>
       </x:c>
       <x:c r="K86" s="170" t="str">
-        <x:v>Pending PestFlow commit</x:v>
+        <x:v>b10e176; PR #89</x:v>
       </x:c>
       <x:c r="L86" s="170" t="str">
         <x:v>Commit and push the verified PestFlow branch, then record exact cloud state.</x:v>
@@ -8961,37 +8961,93 @@
         <x:v>This prevents the standalone repository, branch result, and live PestFlow state from being confused again.</x:v>
       </x:c>
     </x:row>
-    <x:row r="87">
-      <x:c r="A87" s="133"/>
-      <x:c r="B87" s="165"/>
-      <x:c r="C87" s="133"/>
-      <x:c r="D87" s="133"/>
-      <x:c r="E87" s="133"/>
-      <x:c r="F87" s="133"/>
-      <x:c r="G87" s="133"/>
-      <x:c r="H87" s="133"/>
-      <x:c r="I87" s="133"/>
-      <x:c r="J87" s="133"/>
-      <x:c r="K87" s="133"/>
-      <x:c r="L87" s="133"/>
-      <x:c r="M87" s="133"/>
-      <x:c r="N87" s="133"/>
-    </x:row>
-    <x:row r="88">
-      <x:c r="A88" s="133"/>
-      <x:c r="B88" s="165"/>
-      <x:c r="C88" s="133"/>
-      <x:c r="D88" s="133"/>
-      <x:c r="E88" s="133"/>
-      <x:c r="F88" s="133"/>
-      <x:c r="G88" s="133"/>
-      <x:c r="H88" s="133"/>
-      <x:c r="I88" s="133"/>
-      <x:c r="J88" s="133"/>
-      <x:c r="K88" s="133"/>
-      <x:c r="L88" s="133"/>
-      <x:c r="M88" s="133"/>
-      <x:c r="N88" s="133"/>
+    <x:row r="87" ht="116" customHeight="1">
+      <x:c r="A87" s="170" t="str">
+        <x:v>AL-082</x:v>
+      </x:c>
+      <x:c r="B87" s="171" t="n">
+        <x:v>46215.913194444445</x:v>
+      </x:c>
+      <x:c r="C87" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D87" s="170" t="str">
+        <x:v>Integrate latest PestFlow main without losing QA fixes</x:v>
+      </x:c>
+      <x:c r="E87" s="170" t="str">
+        <x:v>Fetched seven newer main commits, merged them into the QA branch, combined the AppLayout setup-prompt behavior with the title fallback, and detected the new Move-In Assistant route through the parity contract.</x:v>
+      </x:c>
+      <x:c r="F87" s="170" t="str">
+        <x:v>Git merge + complete local gates</x:v>
+      </x:c>
+      <x:c r="G87" s="170" t="str">
+        <x:v>Current main integrated and coverage expanded</x:v>
+      </x:c>
+      <x:c r="H87" s="170" t="str">
+        <x:v>Catalog grew dynamically from 26 routes/78 checks to 27 routes/81 checks. 769/769 unit, 44/44 policy, 16/16 incident, build, tsc, lint, Checkly bundle, 15/15 focused renders, and 194/194 uncontended behaviors passed.</x:v>
+      </x:c>
+      <x:c r="I87" s="170" t="str">
+        <x:v>1440×900; 1280×800; 1024×768</x:v>
+      </x:c>
+      <x:c r="J87" s="170" t="str">
+        <x:v>b10e176; PR #89</x:v>
+      </x:c>
+      <x:c r="K87" s="170" t="str">
+        <x:v>b10e176</x:v>
+      </x:c>
+      <x:c r="L87" s="170" t="str">
+        <x:v>Deploy reviewed head and rerun all 81 production contracts.</x:v>
+      </x:c>
+      <x:c r="M87" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N87" s="170" t="str">
+        <x:v>One parallel local run timed out 1/194 under unit/build contention; exact case passed 1/1 and uncontended complete rerun passed 194/194.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="116" customHeight="1">
+      <x:c r="A88" s="170" t="str">
+        <x:v>AL-083</x:v>
+      </x:c>
+      <x:c r="B88" s="171" t="n">
+        <x:v>46215.913194444445</x:v>
+      </x:c>
+      <x:c r="C88" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="D88" s="170" t="str">
+        <x:v>Publish and verify exact merged head</x:v>
+      </x:c>
+      <x:c r="E88" s="170" t="str">
+        <x:v>Pushed merge commit b10e176, refreshed draft PR #89, verified it is mergeable, and ran the automatic PR gate plus an isolated owner proof on the exact SHA.</x:v>
+      </x:c>
+      <x:c r="F88" s="170" t="str">
+        <x:v>GitHub + Checkly workflow</x:v>
+      </x:c>
+      <x:c r="G88" s="170" t="str">
+        <x:v>Branch current; cloud proof blocked before execution</x:v>
+      </x:c>
+      <x:c r="H88" s="170" t="str">
+        <x:v>PR gate 29210282667 and owner proof 29210311515 each had zero steps. Check-run annotations explicitly report failed recent payments or exceeded spending limit.</x:v>
+      </x:c>
+      <x:c r="I88" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="J88" s="170" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/actions/runs/29210311515</x:v>
+      </x:c>
+      <x:c r="K88" s="170" t="str">
+        <x:v>b10e176; PR #89</x:v>
+      </x:c>
+      <x:c r="L88" s="170" t="str">
+        <x:v>Restore GitHub Actions capacity, rerun exact-head cloud proof, then deploy and require 81/81 production certification.</x:v>
+      </x:c>
+      <x:c r="M88" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="N88" s="170" t="str">
+        <x:v>PR is mergeable/unstable. Billing is infrastructure evidence, not a PestFlow product verdict.</x:v>
+      </x:c>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="133"/>
@@ -9575,7 +9631,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf31eace995144a79"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb303945e30a4f2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11886,10 +11942,10 @@
         <x:v>Automation</x:v>
       </x:c>
       <x:c r="C68" s="170" t="str">
-        <x:v>Shared 26-route catalog parity</x:v>
+        <x:v>Shared static owner-route catalog parity</x:v>
       </x:c>
       <x:c r="D68" s="170" t="str">
-        <x:v>26 owner routes</x:v>
+        <x:v>27 owner routes</x:v>
       </x:c>
       <x:c r="E68" s="170" t="str">
         <x:v>Node policy</x:v>
@@ -11904,13 +11960,13 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="I68" s="171" t="n">
-        <x:v>46215.90625</x:v>
+        <x:v>46215.913194444445</x:v>
       </x:c>
       <x:c r="J68" s="170" t="str">
         <x:v>44/44 Guardian policy tests</x:v>
       </x:c>
       <x:c r="K68" s="170" t="str">
-        <x:v>Deterministic and Checkly consumers cannot drift from the shared static owner catalog.</x:v>
+        <x:v>Deterministic and Checkly consumers cannot drift; Move-In Assistant was added when main introduced the route.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="80" customHeight="1">
@@ -11924,7 +11980,7 @@
         <x:v>Complete owner route/viewport audit</x:v>
       </x:c>
       <x:c r="D69" s="170" t="str">
-        <x:v>3 widths × 26 routes</x:v>
+        <x:v>3 widths × 26 historical routes</x:v>
       </x:c>
       <x:c r="E69" s="170" t="str">
         <x:v>Playwright Chromium</x:v>
@@ -11939,13 +11995,13 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="I69" s="171" t="n">
-        <x:v>46215.90625</x:v>
+        <x:v>46215.913194444445</x:v>
       </x:c>
       <x:c r="J69" s="170" t="str">
         <x:v>69/78 passed</x:v>
       </x:c>
       <x:c r="K69" s="170" t="str">
-        <x:v>Services, SMS Contacts, and Common Replies failed at each width; Settings branch API returned 500.</x:v>
+        <x:v>Historical live audit predates Move-In Assistant; current required matrix is 27×3=81.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="80" customHeight="1">
@@ -11959,7 +12015,7 @@
         <x:v>Exact repaired desktop surfaces</x:v>
       </x:c>
       <x:c r="D70" s="170" t="str">
-        <x:v>4 routes × 3 widths</x:v>
+        <x:v>5 routes × 3 widths</x:v>
       </x:c>
       <x:c r="E70" s="170" t="str">
         <x:v>Local Playwright Chromium</x:v>
@@ -11974,13 +12030,13 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="I70" s="171" t="n">
-        <x:v>46215.90625</x:v>
+        <x:v>46215.913194444445</x:v>
       </x:c>
       <x:c r="J70" s="170" t="str">
-        <x:v>12/12 passed</x:v>
+        <x:v>15/15 passed</x:v>
       </x:c>
       <x:c r="K70" s="170" t="str">
-        <x:v>No fatal UI, console error, or horizontal overflow on Services, SMS Contacts, Common Replies, or Settings.</x:v>
+        <x:v>Services, SMS Contacts, Common Replies, Settings, and Move-In Assistant render without fatal UI, console error, or overflow.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="80" customHeight="1">
@@ -12009,13 +12065,13 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="I71" s="171" t="n">
-        <x:v>46215.90625</x:v>
+        <x:v>46215.913194444445</x:v>
       </x:c>
       <x:c r="J71" s="170" t="str">
-        <x:v>7/7 focused tests</x:v>
+        <x:v>10/10 focused tests</x:v>
       </x:c>
       <x:c r="K71" s="170" t="str">
-        <x:v>Route ordering/isolation, validation, primary protection, title fallback, and feature titles are locked.</x:v>
+        <x:v>Branch CRUD invariants plus AppLayout and feature-title contracts passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="80" customHeight="1">
@@ -12044,13 +12100,13 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="I72" s="171" t="n">
-        <x:v>46215.90625</x:v>
+        <x:v>46215.913194444445</x:v>
       </x:c>
       <x:c r="J72" s="170" t="str">
-        <x:v>760 unit; 44 policy; 16 incident</x:v>
+        <x:v>769 unit; 44 policy; 16 incident</x:v>
       </x:c>
       <x:c r="K72" s="170" t="str">
-        <x:v>TypeScript, focused lint, production build, and Checkly bundle also exited 0.</x:v>
+        <x:v>TypeScript, focused lint, production build, and Checkly bundle also exited 0 after merging current main.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="80" customHeight="1">
@@ -12079,13 +12135,13 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="I73" s="171" t="n">
-        <x:v>46215.90625</x:v>
+        <x:v>46215.913194444445</x:v>
       </x:c>
       <x:c r="J73" s="170" t="str">
-        <x:v>194/194 passed in 6.7m</x:v>
+        <x:v>194/194 passed in 2.7m</x:v>
       </x:c>
       <x:c r="K73" s="170" t="str">
-        <x:v>Shared AppLayout changes did not regress the delegated feature catalog.</x:v>
+        <x:v>Uncontended final rerun passed. Prior parallel resource-contention timeout remains recorded separately.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="80" customHeight="1">
@@ -12117,10 +12173,10 @@
         <x:v>46215.90625</x:v>
       </x:c>
       <x:c r="J74" s="170" t="str">
-        <x:v>4/4 contracts; 12-entry dry run</x:v>
+        <x:v>4/4 contracts; 12-entry dry run; a468b1a</x:v>
       </x:c>
       <x:c r="K74" s="170" t="str">
-        <x:v>Commit eb251f2 is on main; yawbtng has write access; scheduled and reusable workflows are active.</x:v>
+        <x:v>Standalone registry now includes all 27 owner routes including Move-In Assistant.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="80" customHeight="1">
@@ -12158,31 +12214,75 @@
         <x:v>DB/schema pass; currently deployed frontend/API health omit deployment.commitSha and therefore fail closed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="76">
-      <x:c r="A76" s="133"/>
-      <x:c r="B76" s="133"/>
-      <x:c r="C76" s="133"/>
-      <x:c r="D76" s="133"/>
-      <x:c r="E76" s="133"/>
-      <x:c r="F76" s="133"/>
-      <x:c r="G76" s="133"/>
-      <x:c r="H76" s="133"/>
-      <x:c r="I76" s="165"/>
-      <x:c r="J76" s="133"/>
-      <x:c r="K76" s="133"/>
-    </x:row>
-    <x:row r="77">
-      <x:c r="A77" s="133"/>
-      <x:c r="B77" s="133"/>
-      <x:c r="C77" s="133"/>
-      <x:c r="D77" s="133"/>
-      <x:c r="E77" s="133"/>
-      <x:c r="F77" s="133"/>
-      <x:c r="G77" s="133"/>
-      <x:c r="H77" s="133"/>
-      <x:c r="I77" s="165"/>
-      <x:c r="J77" s="133"/>
-      <x:c r="K77" s="133"/>
+    <x:row r="76" ht="82" customHeight="1">
+      <x:c r="A76" s="170" t="str">
+        <x:v>QA-071</x:v>
+      </x:c>
+      <x:c r="B76" s="170" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C76" s="170" t="str">
+        <x:v>Exact merged-head PR release gate</x:v>
+      </x:c>
+      <x:c r="D76" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="E76" s="170" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F76" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G76" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H76" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I76" s="171" t="n">
+        <x:v>46215.913194444445</x:v>
+      </x:c>
+      <x:c r="J76" s="170" t="str">
+        <x:v>Run 29210282667: zero steps</x:v>
+      </x:c>
+      <x:c r="K76" s="170" t="str">
+        <x:v>Verified billing/spending refusal; no product or QA command started.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="82" customHeight="1">
+      <x:c r="A77" s="170" t="str">
+        <x:v>QA-072</x:v>
+      </x:c>
+      <x:c r="B77" s="170" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C77" s="170" t="str">
+        <x:v>Exact merged-head 27-route owner proof</x:v>
+      </x:c>
+      <x:c r="D77" s="170" t="str">
+        <x:v>1366×900</x:v>
+      </x:c>
+      <x:c r="E77" s="170" t="str">
+        <x:v>GitHub Actions + Checkly</x:v>
+      </x:c>
+      <x:c r="F77" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G77" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H77" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I77" s="171" t="n">
+        <x:v>46215.913194444445</x:v>
+      </x:c>
+      <x:c r="J77" s="170" t="str">
+        <x:v>Run 29210311515: zero steps</x:v>
+      </x:c>
+      <x:c r="K77" s="170" t="str">
+        <x:v>Same verified billing/spending refusal; no final-head cloud pass is claimed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="133"/>
@@ -12861,7 +12961,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra14041bb4ca04694"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56d40376222540a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13522,10 +13622,10 @@
         <x:v>Trevor + Codex</x:v>
       </x:c>
       <x:c r="K19" s="174" t="str">
-        <x:v>Branch fixed; 12/12 focused renders and 194/194 full suite pass.</x:v>
+        <x:v>Branch fixed; 15/15 focused renders and 194/194 uncontended full suite pass at b10e176.</x:v>
       </x:c>
       <x:c r="L19" s="174" t="str">
-        <x:v>Production certification pending deploy and 78/78 rerun.</x:v>
+        <x:v>Production certification pending deploy and 81/81 rerun.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="116" customHeight="1">
@@ -13560,7 +13660,7 @@
         <x:v>Trevor + Codex</x:v>
       </x:c>
       <x:c r="K20" s="174" t="str">
-        <x:v>Branch route contract tests pass 5/5.</x:v>
+        <x:v>Branch route contract tests pass 8/8 at b10e176.</x:v>
       </x:c>
       <x:c r="L20" s="174" t="str">
         <x:v>Production certification pending deploy and exact-SHA oracle proof.</x:v>
@@ -13598,10 +13698,10 @@
         <x:v>Trevor + Codex</x:v>
       </x:c>
       <x:c r="K21" s="174" t="str">
-        <x:v>Branch Services render passes at all three widths.</x:v>
+        <x:v>Branch Services and Move-In Assistant renders pass at all three widths.</x:v>
       </x:c>
       <x:c r="L21" s="174" t="str">
-        <x:v>Production certification pending deploy and 78/78 rerun.</x:v>
+        <x:v>Production certification pending deploy and 81/81 rerun.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13638,7 +13738,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R306ce1f4fa194eb7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R086e95feb64d4fe7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: sync owner API contract activity tracker
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4c05d42b95a247ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R65e91ff8202940c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R79a04e22a7b64b31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R33b7bd7df07a496a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R3c4c14f1d0264eca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R42ad6909ac7a4ae7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R7c036d9defff4e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R4cf4609e7f524405"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R06806b6b9df74aae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R9255dd6e22d24db6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1337,7 +1337,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N88" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N93" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1359,7 +1359,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1761,17 +1761,17 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>72</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>50</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Failed")</x:f>
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F9" s="141"/>
       <x:c r="G9" s="138" t="n">
@@ -1930,30 +1930,30 @@
         <x:v>Product failures and infrastructure failures stay separate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="118" customHeight="1">
+    <x:row r="17" ht="126" customHeight="1">
       <x:c r="A17" s="120" t="str">
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Historical production audit 69/78; merged head has 27 routes/81 checks and passes focused 15/15 plus full 194/194.</x:v>
+        <x:v>Live owner APIs pass 31/32; historical route audit is 69/78. Branch 7a8d746 fixes the only API failure and retains 15/15 focused plus 194/194 broad route proof.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ b10e176; Browser-Base-QA @ a468b1a shared with yawbtng.</x:v>
+        <x:v>PestFlow PR #89 @ 7a8d746; Browser-Base-QA @ 17795cb shared with yawbtng.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Activation</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>Restore Actions; deploy reviewed fixes; add Browserbase secrets/context; require exact-SHA external gate and 81/81.</x:v>
+        <x:v>Restore Actions; deploy reviewed fixes; add Browserbase secrets/context; require exact-SHA 32/32 API and 81/81 route gates.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>Draft PR mergeable/unstable; exact-head runs 29210282667 and 29210311515 were zero-step billing blocked.</x:v>
+        <x:v>Draft PR mergeable/unstable; run 29211160983 was zero-step billing blocked.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2075,7 +2075,7 @@
         <x:v>Note</x:v>
       </x:c>
       <x:c r="B23" s="118" t="str">
-        <x:v>Original critical workflows are green; the exhaustive live owner matrix remains red at 69/78 until the reviewed fixes deploy.</x:v>
+        <x:v>Original critical workflows are green; live owner evidence remains red at 31/32 APIs and 69/78 historical routes until the reviewed fixes deploy.</x:v>
       </x:c>
       <x:c r="C23" s="118" t="str">
         <x:v>Note</x:v>
@@ -2614,11 +2614,11 @@
         <x:v>/private/tmp/pestflow-desktop-qa-guardian/qa/guardian/desktop-journeys.json</x:v>
       </x:c>
       <x:c r="N8" s="113" t="str">
-        <x:v>d3c3dcb; PR #89</x:v>
+        <x:v>7a8d746 + Browser-Base-QA 17795cb; PR #89</x:v>
       </x:c>
       <x:c r="O8" s="113"/>
       <x:c r="P8" s="113" t="str">
-        <x:v>Production journeys are read-only. Results now include sanitized first-party network failures and uncaught page errors.</x:v>
+        <x:v>The standalone recorded owner session now executes all 32 PestFlow API contracts once, in addition to semantic route journeys.</x:v>
       </x:c>
       <x:c r="Q8" s="163" t="n">
         <x:v>46215.27099571759</x:v>
@@ -2788,7 +2788,7 @@
         <x:v>Expand deterministic desktop production coverage</x:v>
       </x:c>
       <x:c r="D12" s="166" t="str">
-        <x:v>All static owner routes are audited at three widths, complete failure evidence is preserved, and the deployed reviewed head passes the current dynamic matrix.</x:v>
+        <x:v>All 32 registered owner APIs and all static owner routes are audited; complete evidence is preserved; the deployed reviewed head passes 32/32 APIs and the current 81-route matrix.</x:v>
       </x:c>
       <x:c r="E12" s="166" t="str">
         <x:v>In Progress</x:v>
@@ -2800,7 +2800,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H12" s="166" t="str">
-        <x:v>Run all 27 owner routes across 1440, 1280, and 1024; preserve complete failure evidence; after fixes deploy and require an 81/81 production rerun.</x:v>
+        <x:v>Run all 32 authenticated GET contracts, then all 27 routes across 1440, 1280, and 1024; preserve complete failure and cleanup evidence; require 32/32 plus 81/81 after deploy.</x:v>
       </x:c>
       <x:c r="I12" s="166" t="str">
         <x:v>Passed</x:v>
@@ -2812,22 +2812,22 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="L12" s="166" t="str">
-        <x:v>1440×900; 1280×800; 1024×768</x:v>
+        <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M12" s="166" t="str">
-        <x:v>69/78 historical production; 15/15 merged-branch focus; current target 81/81</x:v>
+        <x:v>31/32 live APIs; 69/78 historical routes; 15/15 merged-branch focus; targets 32/32 and 81/81</x:v>
       </x:c>
       <x:c r="N12" s="166" t="str">
-        <x:v>b10e176; PR #89</x:v>
+        <x:v>7a8d746; PR #89</x:v>
       </x:c>
       <x:c r="O12" s="166" t="str">
-        <x:v>Requires reviewed deploy for final live certification.</x:v>
+        <x:v>Requires reviewed deploy and restored GitHub Actions capacity for final live certification.</x:v>
       </x:c>
       <x:c r="P12" s="166" t="str">
-        <x:v>Coverage automatically absorbed Move-In Assistant from current main. Historical audit remains red until deploy and all 81 checks pass.</x:v>
+        <x:v>Only current production /companies/branches remains red in the API sweep; the exact branch repair and lifecycle regression are green.</x:v>
       </x:c>
       <x:c r="Q12" s="167" t="n">
-        <x:v>46215.913194444445</x:v>
+        <x:v>46215.92916666667</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2922,11 +2922,11 @@
         <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/pull/89</x:v>
       </x:c>
       <x:c r="N14" s="166" t="str">
-        <x:v>b10e176; PR #89</x:v>
+        <x:v>7a8d746; PR #89</x:v>
       </x:c>
       <x:c r="O14" s="166"/>
       <x:c r="P14" s="166" t="str">
-        <x:v>769/769 unit, 44/44 policy, 16/16 incident, 15/15 focused renders, 194/194 full desktop, build/type/lint/Checkly green; cloud zero-step blocked.</x:v>
+        <x:v>769/769 unit, 45/45 policy, 16/16 incident, build/type/lint green; production API audit 31/32 with verified 5/5 cleanup; run 29211160983 zero-step billing blocked.</x:v>
       </x:c>
       <x:c r="Q14" s="167" t="n">
         <x:v>46215.913194444445</x:v>
@@ -3021,16 +3021,16 @@
         <x:v>Risk-selected + full production</x:v>
       </x:c>
       <x:c r="M16" s="166" t="str">
-        <x:v>Browser-Base-QA @ a468b1a; PR #89 @ b10e176</x:v>
+        <x:v>Browser-Base-QA @ 17795cb; PR #89 @ 7a8d746</x:v>
       </x:c>
       <x:c r="N16" s="166" t="str">
-        <x:v>Standalone gate and merged PestFlow head are published; production promotion wiring remains pending.</x:v>
+        <x:v>The standalone owner session now executes the shared 32-endpoint contract; production promotion wiring remains pending.</x:v>
       </x:c>
       <x:c r="O16" s="166" t="str">
         <x:v>Needs Browserbase secrets/context, deploy ownership, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P16" s="166" t="str">
-        <x:v>Current catalog has 27 routes. Production health still lacks deployment.commitSha until reviewed PestFlow work is deployed.</x:v>
+        <x:v>Current production is 31/32 owner APIs and still lacks deployment.commitSha; deploy reviewed PestFlow head, then require 32/32 plus 81/81.</x:v>
       </x:c>
       <x:c r="Q16" s="167" t="n">
         <x:v>46215.27099571759</x:v>
@@ -3255,7 +3255,7 @@
         <x:v>Deploy and certify exhaustive desktop bug fixes</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
-        <x:v>The reviewed fixes are deployed, all 27 owner routes pass at 1440×900, 1280×800, and 1024×768, Settings branch API has no 5xx, and evidence is tied to the deployed SHA.</x:v>
+        <x:v>The reviewed fixes are deployed, all 32 owner API contracts pass, all 27 owner routes pass at 1440×900, 1280×800, and 1024×768, and evidence is tied to the deployed SHA.</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
         <x:v>Blocked</x:v>
@@ -3267,7 +3267,7 @@
         <x:v>Trevor + Codex</x:v>
       </x:c>
       <x:c r="H21" s="170" t="str">
-        <x:v>Review and deploy PR #89, verify deployed commit identity, rerun the 81-check production matrix plus outcome oracles, and require 81/81 before closure.</x:v>
+        <x:v>Review and deploy PR #89, verify deployed commit identity, rerun the 32-API contract plus 81-route matrix and public oracles, and require every check before closure.</x:v>
       </x:c>
       <x:c r="I21" s="170" t="str">
         <x:v>Pending</x:v>
@@ -3279,22 +3279,22 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="L21" s="170" t="str">
-        <x:v>1440×900; 1280×800; 1024×768</x:v>
+        <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M21" s="170" t="str">
-        <x:v>G-013; G-014; G-015; PR #89 @ b10e176</x:v>
+        <x:v>31/32 production APIs; G-013; G-014; G-015; PR #89 @ 7a8d746</x:v>
       </x:c>
       <x:c r="N21" s="170" t="str">
-        <x:v>b10e176; PR #89</x:v>
+        <x:v>7a8d746; PR #89</x:v>
       </x:c>
       <x:c r="O21" s="170" t="str">
         <x:v>Needs merge/deploy authority, deployed commit identity, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P21" s="170" t="str">
-        <x:v>Merged branch proof is green; current production is deliberately not certified. Move-In Assistant is included in the 81-check target.</x:v>
+        <x:v>Branch proof is green; current production is deliberately not certified. Final target is 32/32 APIs plus 81/81 route/width checks.</x:v>
       </x:c>
       <x:c r="Q21" s="171" t="n">
-        <x:v>46215.913194444445</x:v>
+        <x:v>46215.92916666667</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -5248,7 +5248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde96a1f3366a454c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea35987a55ab4568"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9049,85 +9049,225 @@
         <x:v>PR is mergeable/unstable. Billing is infrastructure evidence, not a PestFlow product verdict.</x:v>
       </x:c>
     </x:row>
-    <x:row r="89">
-      <x:c r="A89" s="133"/>
-      <x:c r="B89" s="165"/>
-      <x:c r="C89" s="133"/>
-      <x:c r="D89" s="133"/>
-      <x:c r="E89" s="133"/>
-      <x:c r="F89" s="133"/>
-      <x:c r="G89" s="133"/>
-      <x:c r="H89" s="133"/>
-      <x:c r="I89" s="133"/>
-      <x:c r="J89" s="133"/>
-      <x:c r="K89" s="133"/>
-      <x:c r="L89" s="133"/>
-      <x:c r="M89" s="133"/>
-      <x:c r="N89" s="133"/>
-    </x:row>
-    <x:row r="90">
-      <x:c r="A90" s="133"/>
-      <x:c r="B90" s="165"/>
-      <x:c r="C90" s="133"/>
-      <x:c r="D90" s="133"/>
-      <x:c r="E90" s="133"/>
-      <x:c r="F90" s="133"/>
-      <x:c r="G90" s="133"/>
-      <x:c r="H90" s="133"/>
-      <x:c r="I90" s="133"/>
-      <x:c r="J90" s="133"/>
-      <x:c r="K90" s="133"/>
-      <x:c r="L90" s="133"/>
-      <x:c r="M90" s="133"/>
-      <x:c r="N90" s="133"/>
-    </x:row>
-    <x:row r="91">
-      <x:c r="A91" s="133"/>
-      <x:c r="B91" s="165"/>
-      <x:c r="C91" s="133"/>
-      <x:c r="D91" s="133"/>
-      <x:c r="E91" s="133"/>
-      <x:c r="F91" s="133"/>
-      <x:c r="G91" s="133"/>
-      <x:c r="H91" s="133"/>
-      <x:c r="I91" s="133"/>
-      <x:c r="J91" s="133"/>
-      <x:c r="K91" s="133"/>
-      <x:c r="L91" s="133"/>
-      <x:c r="M91" s="133"/>
-      <x:c r="N91" s="133"/>
-    </x:row>
-    <x:row r="92">
-      <x:c r="A92" s="133"/>
-      <x:c r="B92" s="165"/>
-      <x:c r="C92" s="133"/>
-      <x:c r="D92" s="133"/>
-      <x:c r="E92" s="133"/>
-      <x:c r="F92" s="133"/>
-      <x:c r="G92" s="133"/>
-      <x:c r="H92" s="133"/>
-      <x:c r="I92" s="133"/>
-      <x:c r="J92" s="133"/>
-      <x:c r="K92" s="133"/>
-      <x:c r="L92" s="133"/>
-      <x:c r="M92" s="133"/>
-      <x:c r="N92" s="133"/>
-    </x:row>
-    <x:row r="93">
-      <x:c r="A93" s="133"/>
-      <x:c r="B93" s="165"/>
-      <x:c r="C93" s="133"/>
-      <x:c r="D93" s="133"/>
-      <x:c r="E93" s="133"/>
-      <x:c r="F93" s="133"/>
-      <x:c r="G93" s="133"/>
-      <x:c r="H93" s="133"/>
-      <x:c r="I93" s="133"/>
-      <x:c r="J93" s="133"/>
-      <x:c r="K93" s="133"/>
-      <x:c r="L93" s="133"/>
-      <x:c r="M93" s="133"/>
-      <x:c r="N93" s="133"/>
+    <x:row r="89" ht="116" customHeight="1">
+      <x:c r="A89" s="170" t="str">
+        <x:v>AL-084</x:v>
+      </x:c>
+      <x:c r="B89" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="C89" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D89" s="170" t="str">
+        <x:v>Register the authenticated desktop API surface</x:v>
+      </x:c>
+      <x:c r="E89" s="170" t="str">
+        <x:v>Created one 32-endpoint owner GET registry covering the data behind customers, jobs, invoices, documents, services, equipment, chemicals, messaging, notifications, chat, estimates, migration, reviews, and reports.</x:v>
+      </x:c>
+      <x:c r="F89" s="170" t="str">
+        <x:v>Playwright API + policy</x:v>
+      </x:c>
+      <x:c r="G89" s="170" t="str">
+        <x:v>Complete API contract sweep implemented</x:v>
+      </x:c>
+      <x:c r="H89" s="170" t="str">
+        <x:v>Every contract requires HTTP 200, JSON, named keys, and declared array shapes. Evidence retains status/schema/timing only and attempts all rows before aggregate failure.</x:v>
+      </x:c>
+      <x:c r="I89" s="170" t="str">
+        <x:v>Authenticated desktop owner</x:v>
+      </x:c>
+      <x:c r="J89" s="170" t="str">
+        <x:v>qa/guardian/desktop-owner-api-contracts.json</x:v>
+      </x:c>
+      <x:c r="K89" s="170" t="str">
+        <x:v>7a8d746; PR #89</x:v>
+      </x:c>
+      <x:c r="L89" s="170" t="str">
+        <x:v>Deploy the reviewed company-branches repair, then require 32/32 on the deployed SHA.</x:v>
+      </x:c>
+      <x:c r="M89" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N89" s="170" t="str">
+        <x:v>A synthetic-tenant lifecycle also covers branch creation, one-primary enforcement, tenant denial, promotion, and deactivation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="116" customHeight="1">
+      <x:c r="A90" s="170" t="str">
+        <x:v>AL-085</x:v>
+      </x:c>
+      <x:c r="B90" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="C90" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D90" s="170" t="str">
+        <x:v>Audit all registered owner APIs in production</x:v>
+      </x:c>
+      <x:c r="E90" s="170" t="str">
+        <x:v>Ran the new complete contract sweep with five disposable accounts against the real PestFlow API and retained body-free evidence plus teardown proof.</x:v>
+      </x:c>
+      <x:c r="F90" s="170" t="str">
+        <x:v>Production Playwright API</x:v>
+      </x:c>
+      <x:c r="G90" s="170" t="str">
+        <x:v>31/32 passed; known branch endpoint isolated</x:v>
+      </x:c>
+      <x:c r="H90" s="170" t="str">
+        <x:v>Only GET /companies/branches returned 500. All other 31 contracts passed; 5/5 accounts were deleted, sessions cleared, and credentials rejected.</x:v>
+      </x:c>
+      <x:c r="I90" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="J90" s="170" t="str">
+        <x:v>artifacts/desktop-critical/owner-api-contracts.json</x:v>
+      </x:c>
+      <x:c r="K90" s="170" t="str">
+        <x:v>7a8d746; PR #89</x:v>
+      </x:c>
+      <x:c r="L90" s="170" t="str">
+        <x:v>Deploy commit 7a8d746 and rerun the same 32 contracts before certification.</x:v>
+      </x:c>
+      <x:c r="M90" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N90" s="170" t="str">
+        <x:v>This confirms the production failure is narrow and already repaired on the branch; production remains deliberately red until deploy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="116" customHeight="1">
+      <x:c r="A91" s="170" t="str">
+        <x:v>AL-086</x:v>
+      </x:c>
+      <x:c r="B91" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="C91" s="170" t="str">
+        <x:v>T-003</x:v>
+      </x:c>
+      <x:c r="D91" s="170" t="str">
+        <x:v>Connect Browser Base QA to PestFlow owner APIs</x:v>
+      </x:c>
+      <x:c r="E91" s="170" t="str">
+        <x:v>Copied the shared contract into Browser-Base-QA and made the recorded authenticated Browserbase owner session execute it once per Guardian run without exporting response bodies.</x:v>
+      </x:c>
+      <x:c r="F91" s="170" t="str">
+        <x:v>Browserbase/Stagehand control plane</x:v>
+      </x:c>
+      <x:c r="G91" s="170" t="str">
+        <x:v>Standalone PestFlow contract integration published</x:v>
+      </x:c>
+      <x:c r="H91" s="170" t="str">
+        <x:v>6/6 standalone tests, 12-entry Guardian dry run, 32-contract validation, and moderate audit threshold passed; only 19 known low Stagehand advisories remain.</x:v>
+      </x:c>
+      <x:c r="I91" s="170" t="str">
+        <x:v>1440/1280/1920/1024 registry</x:v>
+      </x:c>
+      <x:c r="J91" s="170" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA/commit/37f199c</x:v>
+      </x:c>
+      <x:c r="K91" s="170" t="str">
+        <x:v>37f199c</x:v>
+      </x:c>
+      <x:c r="L91" s="170" t="str">
+        <x:v>Add Browserbase secrets and isolated owner context before the first managed replay run.</x:v>
+      </x:c>
+      <x:c r="M91" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N91" s="170" t="str">
+        <x:v>This makes the shared repository an executing outside-in control plane rather than a passive copy of PestFlow files.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="116" customHeight="1">
+      <x:c r="A92" s="170" t="str">
+        <x:v>AL-087</x:v>
+      </x:c>
+      <x:c r="B92" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="C92" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="D92" s="170" t="str">
+        <x:v>Publish and classify the API-contract checkpoint</x:v>
+      </x:c>
+      <x:c r="E92" s="170" t="str">
+        <x:v>Pushed both repositories, refreshed draft PR #89, verified the exact PestFlow head, and inspected the automatically triggered release gate.</x:v>
+      </x:c>
+      <x:c r="F92" s="170" t="str">
+        <x:v>GitHub + GitHub Actions</x:v>
+      </x:c>
+      <x:c r="G92" s="170" t="str">
+        <x:v>Both repos current; cloud gate blocked before execution</x:v>
+      </x:c>
+      <x:c r="H92" s="170" t="str">
+        <x:v>PestFlow head 7a8d746 and Browser-Base-QA head 37f199c are remote. Run 29211160983 had zero steps and the same verified payment/spending-limit annotation.</x:v>
+      </x:c>
+      <x:c r="I92" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="J92" s="170" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/actions/runs/29211160983</x:v>
+      </x:c>
+      <x:c r="K92" s="170" t="str">
+        <x:v>7a8d746; 37f199c; PR #89</x:v>
+      </x:c>
+      <x:c r="L92" s="170" t="str">
+        <x:v>Restore Actions capacity, deploy the reviewed PestFlow head, then require 32/32 API and 81/81 route certification.</x:v>
+      </x:c>
+      <x:c r="M92" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="N92" s="170" t="str">
+        <x:v>PR #89 remains mergeable/unstable. No cloud or production-green result is claimed for this exact head.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="116" customHeight="1">
+      <x:c r="A93" s="170" t="str">
+        <x:v>AL-088</x:v>
+      </x:c>
+      <x:c r="B93" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="C93" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D93" s="170" t="str">
+        <x:v>Publish the complete PRD in Browser Base QA</x:v>
+      </x:c>
+      <x:c r="E93" s="170" t="str">
+        <x:v>Replaced the standalone repository's short PRD summary with the complete two-part Reliability Command Center PRD from PestFlow after the repository-boundary gap was identified.</x:v>
+      </x:c>
+      <x:c r="F93" s="170" t="str">
+        <x:v>Documentation + GitHub</x:v>
+      </x:c>
+      <x:c r="G93" s="170" t="str">
+        <x:v>Full canonical PRD published</x:v>
+      </x:c>
+      <x:c r="H93" s="170" t="str">
+        <x:v>Both PRD files are 492 lines with identical SHA-1 content; Browser-Base-QA commit 17795cb is pushed on main.</x:v>
+      </x:c>
+      <x:c r="I93" s="170" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="J93" s="170" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA/blob/main/docs/PRD.md</x:v>
+      </x:c>
+      <x:c r="K93" s="170" t="str">
+        <x:v>17795cb</x:v>
+      </x:c>
+      <x:c r="L93" s="170" t="str">
+        <x:v>Keep the standalone PRD synchronized when product requirements materially change.</x:v>
+      </x:c>
+      <x:c r="M93" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N93" s="170" t="str">
+        <x:v>The shared repository now contains the beginner explanation and the full product, architecture, safety, rollout, evidence, and activation specification.</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="133"/>
@@ -9631,7 +9771,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb303945e30a4f2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95186bdafaf24079"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12284,83 +12424,215 @@
         <x:v>Same verified billing/spending refusal; no final-head cloud pass is claimed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="78">
-      <x:c r="A78" s="133"/>
-      <x:c r="B78" s="133"/>
-      <x:c r="C78" s="133"/>
-      <x:c r="D78" s="133"/>
-      <x:c r="E78" s="133"/>
-      <x:c r="F78" s="133"/>
-      <x:c r="G78" s="133"/>
-      <x:c r="H78" s="133"/>
-      <x:c r="I78" s="165"/>
-      <x:c r="J78" s="133"/>
-      <x:c r="K78" s="133"/>
-    </x:row>
-    <x:row r="79">
-      <x:c r="A79" s="133"/>
-      <x:c r="B79" s="133"/>
-      <x:c r="C79" s="133"/>
-      <x:c r="D79" s="133"/>
-      <x:c r="E79" s="133"/>
-      <x:c r="F79" s="133"/>
-      <x:c r="G79" s="133"/>
-      <x:c r="H79" s="133"/>
-      <x:c r="I79" s="165"/>
-      <x:c r="J79" s="133"/>
-      <x:c r="K79" s="133"/>
-    </x:row>
-    <x:row r="80">
-      <x:c r="A80" s="133"/>
-      <x:c r="B80" s="133"/>
-      <x:c r="C80" s="133"/>
-      <x:c r="D80" s="133"/>
-      <x:c r="E80" s="133"/>
-      <x:c r="F80" s="133"/>
-      <x:c r="G80" s="133"/>
-      <x:c r="H80" s="133"/>
-      <x:c r="I80" s="165"/>
-      <x:c r="J80" s="133"/>
-      <x:c r="K80" s="133"/>
-    </x:row>
-    <x:row r="81">
-      <x:c r="A81" s="133"/>
-      <x:c r="B81" s="133"/>
-      <x:c r="C81" s="133"/>
-      <x:c r="D81" s="133"/>
-      <x:c r="E81" s="133"/>
-      <x:c r="F81" s="133"/>
-      <x:c r="G81" s="133"/>
-      <x:c r="H81" s="133"/>
-      <x:c r="I81" s="165"/>
-      <x:c r="J81" s="133"/>
-      <x:c r="K81" s="133"/>
-    </x:row>
-    <x:row r="82">
-      <x:c r="A82" s="133"/>
-      <x:c r="B82" s="133"/>
-      <x:c r="C82" s="133"/>
-      <x:c r="D82" s="133"/>
-      <x:c r="E82" s="133"/>
-      <x:c r="F82" s="133"/>
-      <x:c r="G82" s="133"/>
-      <x:c r="H82" s="133"/>
-      <x:c r="I82" s="165"/>
-      <x:c r="J82" s="133"/>
-      <x:c r="K82" s="133"/>
-    </x:row>
-    <x:row r="83">
-      <x:c r="A83" s="133"/>
-      <x:c r="B83" s="133"/>
-      <x:c r="C83" s="133"/>
-      <x:c r="D83" s="133"/>
-      <x:c r="E83" s="133"/>
-      <x:c r="F83" s="133"/>
-      <x:c r="G83" s="133"/>
-      <x:c r="H83" s="133"/>
-      <x:c r="I83" s="165"/>
-      <x:c r="J83" s="133"/>
-      <x:c r="K83" s="133"/>
+    <x:row r="78" ht="78" customHeight="1">
+      <x:c r="A78" s="170" t="str">
+        <x:v>QA-073</x:v>
+      </x:c>
+      <x:c r="B78" s="170" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="C78" s="170" t="str">
+        <x:v>Authenticated owner API registry policy</x:v>
+      </x:c>
+      <x:c r="D78" s="170" t="str">
+        <x:v>32 endpoints</x:v>
+      </x:c>
+      <x:c r="E78" s="170" t="str">
+        <x:v>Node + TypeScript + ESLint</x:v>
+      </x:c>
+      <x:c r="F78" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G78" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H78" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I78" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="J78" s="170" t="str">
+        <x:v>45/45 Guardian policy tests</x:v>
+      </x:c>
+      <x:c r="K78" s="170" t="str">
+        <x:v>Paths, ids, schema keys, arrays, GET-only use, complete attempts, and body non-retention are locked.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="78" customHeight="1">
+      <x:c r="A79" s="170" t="str">
+        <x:v>QA-074</x:v>
+      </x:c>
+      <x:c r="B79" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C79" s="170" t="str">
+        <x:v>Authenticated owner API contract audit</x:v>
+      </x:c>
+      <x:c r="D79" s="170" t="str">
+        <x:v>32 endpoints</x:v>
+      </x:c>
+      <x:c r="E79" s="170" t="str">
+        <x:v>Playwright API</x:v>
+      </x:c>
+      <x:c r="F79" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G79" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H79" s="170" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="I79" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="J79" s="170" t="str">
+        <x:v>31/32 passed</x:v>
+      </x:c>
+      <x:c r="K79" s="170" t="str">
+        <x:v>Only /companies/branches returned 500 on current production; all other registered data surfaces passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="78" customHeight="1">
+      <x:c r="A80" s="170" t="str">
+        <x:v>QA-075</x:v>
+      </x:c>
+      <x:c r="B80" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C80" s="170" t="str">
+        <x:v>API-audit fixture teardown</x:v>
+      </x:c>
+      <x:c r="D80" s="170" t="str">
+        <x:v>5 synthetic accounts</x:v>
+      </x:c>
+      <x:c r="E80" s="170" t="str">
+        <x:v>Better Auth + API</x:v>
+      </x:c>
+      <x:c r="F80" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G80" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H80" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I80" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="J80" s="170" t="str">
+        <x:v>5/5 deleted; 5/5 sessions cleared; 5/5 logins rejected</x:v>
+      </x:c>
+      <x:c r="K80" s="170" t="str">
+        <x:v>No reserved-domain account from this run remained usable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="78" customHeight="1">
+      <x:c r="A81" s="170" t="str">
+        <x:v>QA-076</x:v>
+      </x:c>
+      <x:c r="B81" s="170" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="C81" s="170" t="str">
+        <x:v>Standalone Browserbase owner API executor</x:v>
+      </x:c>
+      <x:c r="D81" s="170" t="str">
+        <x:v>32 endpoints; 12 sessions</x:v>
+      </x:c>
+      <x:c r="E81" s="170" t="str">
+        <x:v>Node + Guardian dry run</x:v>
+      </x:c>
+      <x:c r="F81" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G81" s="170" t="str">
+        <x:v>T-003</x:v>
+      </x:c>
+      <x:c r="H81" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I81" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="J81" s="170" t="str">
+        <x:v>6/6 tests; 12-entry dry run; 37f199c</x:v>
+      </x:c>
+      <x:c r="K81" s="170" t="str">
+        <x:v>Browser fetch evidence retains only status, content type, timing, key names, and array counts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="78" customHeight="1">
+      <x:c r="A82" s="170" t="str">
+        <x:v>QA-077</x:v>
+      </x:c>
+      <x:c r="B82" s="170" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C82" s="170" t="str">
+        <x:v>Exact API-contract PR release gate</x:v>
+      </x:c>
+      <x:c r="D82" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="E82" s="170" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F82" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G82" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H82" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I82" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="J82" s="170" t="str">
+        <x:v>Run 29211160983: zero steps</x:v>
+      </x:c>
+      <x:c r="K82" s="170" t="str">
+        <x:v>Verified payment/spending refusal; no product or QA command started.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="78" customHeight="1">
+      <x:c r="A83" s="170" t="str">
+        <x:v>QA-078</x:v>
+      </x:c>
+      <x:c r="B83" s="170" t="str">
+        <x:v>Documentation</x:v>
+      </x:c>
+      <x:c r="C83" s="170" t="str">
+        <x:v>Complete standalone PRD parity</x:v>
+      </x:c>
+      <x:c r="D83" s="170" t="str">
+        <x:v>492 lines</x:v>
+      </x:c>
+      <x:c r="E83" s="170" t="str">
+        <x:v>File hash + GitHub</x:v>
+      </x:c>
+      <x:c r="F83" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G83" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="H83" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I83" s="171" t="n">
+        <x:v>46215.92916666667</x:v>
+      </x:c>
+      <x:c r="J83" s="170" t="str">
+        <x:v>Both PRDs have identical SHA-1; 17795cb</x:v>
+      </x:c>
+      <x:c r="K83" s="170" t="str">
+        <x:v>The complete canonical PRD is published in Browser-Base-QA, not only PestFlow.</x:v>
+      </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="133"/>
@@ -12961,7 +13233,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56d40376222540a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f6d8f6fa70f4c94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13660,10 +13932,10 @@
         <x:v>Trevor + Codex</x:v>
       </x:c>
       <x:c r="K20" s="174" t="str">
-        <x:v>Branch route contract tests pass 8/8 at b10e176.</x:v>
+        <x:v>Live contract audit reproduces only this endpoint: 31/32 passed. Branch unit and lifecycle coverage are green at 7a8d746.</x:v>
       </x:c>
       <x:c r="L20" s="174" t="str">
-        <x:v>Production certification pending deploy and exact-SHA oracle proof.</x:v>
+        <x:v>Production certification pending deploy, 32/32 rerun, and exact-SHA oracle proof.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="116" customHeight="1">
@@ -13738,7 +14010,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R086e95feb64d4fe7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red45dcc80d9a44cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: log owner resource lifecycle proof
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R42ad6909ac7a4ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R7c036d9defff4e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R4cf4609e7f524405"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R06806b6b9df74aae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R9255dd6e22d24db6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb96cb2fe9a5f475f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R4d470a01ba0d496b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Re0c4a40a379f4163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Ra0f248e069594d32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R0c548527944e499d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1337,7 +1337,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N93" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N96" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1359,7 +1359,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K86" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1761,12 +1761,12 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>78</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
@@ -1935,13 +1935,13 @@
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Live owner APIs pass 31/32; historical route audit is 69/78. Branch 7a8d746 fixes the only API failure and retains 15/15 focused plus 194/194 broad route proof.</x:v>
+        <x:v>Live owner APIs pass 31/32 and all three Settings/Inventory resource lifecycles pass; historical route audit remains 69/78 until deploy.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ 7a8d746; Browser-Base-QA @ 17795cb shared with yawbtng.</x:v>
+        <x:v>PestFlow PR #89 @ 2aae98e; Browser-Base-QA @ 7788b30 shared with yawbtng.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Activation</x:v>
@@ -1953,7 +1953,7 @@
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>Draft PR mergeable/unstable; run 29211160983 was zero-step billing blocked.</x:v>
+        <x:v>Draft PR mergeable/unstable; run 29211489437 was zero-step billing blocked.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2614,11 +2614,11 @@
         <x:v>/private/tmp/pestflow-desktop-qa-guardian/qa/guardian/desktop-journeys.json</x:v>
       </x:c>
       <x:c r="N8" s="113" t="str">
-        <x:v>7a8d746 + Browser-Base-QA 17795cb; PR #89</x:v>
+        <x:v>2aae98e + Browser-Base-QA 7788b30; PR #89</x:v>
       </x:c>
       <x:c r="O8" s="113"/>
       <x:c r="P8" s="113" t="str">
-        <x:v>The standalone recorded owner session now executes all 32 PestFlow API contracts once, in addition to semantic route journeys.</x:v>
+        <x:v>The standalone recorded owner session executes all 32 PestFlow API contracts; the complete PRD remains synchronized after resource lifecycle expansion.</x:v>
       </x:c>
       <x:c r="Q8" s="163" t="n">
         <x:v>46215.27099571759</x:v>
@@ -2815,19 +2815,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M12" s="166" t="str">
-        <x:v>31/32 live APIs; 69/78 historical routes; 15/15 merged-branch focus; targets 32/32 and 81/81</x:v>
+        <x:v>31/32 live APIs; 3/3 resource lifecycles; 69/78 historical routes; 15/15 merged-branch focus</x:v>
       </x:c>
       <x:c r="N12" s="166" t="str">
-        <x:v>7a8d746; PR #89</x:v>
+        <x:v>2aae98e; PR #89</x:v>
       </x:c>
       <x:c r="O12" s="166" t="str">
         <x:v>Requires reviewed deploy and restored GitHub Actions capacity for final live certification.</x:v>
       </x:c>
       <x:c r="P12" s="166" t="str">
-        <x:v>Only current production /companies/branches remains red in the API sweep; the exact branch repair and lifecycle regression are green.</x:v>
+        <x:v>Equipment, preset notes, and chemical products now have full production-safe CRUD/isolation proof. Current production /companies/branches remains the only API contract failure.</x:v>
       </x:c>
       <x:c r="Q12" s="167" t="n">
-        <x:v>46215.92916666667</x:v>
+        <x:v>46215.93541666667</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2922,11 +2922,11 @@
         <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/pull/89</x:v>
       </x:c>
       <x:c r="N14" s="166" t="str">
-        <x:v>7a8d746; PR #89</x:v>
+        <x:v>2aae98e; PR #89</x:v>
       </x:c>
       <x:c r="O14" s="166"/>
       <x:c r="P14" s="166" t="str">
-        <x:v>769/769 unit, 45/45 policy, 16/16 incident, build/type/lint green; production API audit 31/32 with verified 5/5 cleanup; run 29211160983 zero-step billing blocked.</x:v>
+        <x:v>Latest focused live resource run passed 1/1 with verified 5/5 cleanup; exact-head cloud run 29211489437 was zero-step billing blocked.</x:v>
       </x:c>
       <x:c r="Q14" s="167" t="n">
         <x:v>46215.913194444445</x:v>
@@ -3021,16 +3021,16 @@
         <x:v>Risk-selected + full production</x:v>
       </x:c>
       <x:c r="M16" s="166" t="str">
-        <x:v>Browser-Base-QA @ 17795cb; PR #89 @ 7a8d746</x:v>
+        <x:v>Browser-Base-QA @ 7788b30; PR #89 @ 2aae98e</x:v>
       </x:c>
       <x:c r="N16" s="166" t="str">
-        <x:v>The standalone owner session now executes the shared 32-endpoint contract; production promotion wiring remains pending.</x:v>
+        <x:v>Standalone API executor and complete PRD are current; production promotion wiring remains pending.</x:v>
       </x:c>
       <x:c r="O16" s="166" t="str">
         <x:v>Needs Browserbase secrets/context, deploy ownership, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P16" s="166" t="str">
-        <x:v>Current production is 31/32 owner APIs and still lacks deployment.commitSha; deploy reviewed PestFlow head, then require 32/32 plus 81/81.</x:v>
+        <x:v>Live read contracts are 31/32; owner equipment/preset/chemical lifecycles pass. Deploy reviewed PestFlow head, then require 32/32 plus 81/81.</x:v>
       </x:c>
       <x:c r="Q16" s="167" t="n">
         <x:v>46215.27099571759</x:v>
@@ -3282,19 +3282,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M21" s="170" t="str">
-        <x:v>31/32 production APIs; G-013; G-014; G-015; PR #89 @ 7a8d746</x:v>
+        <x:v>31/32 production APIs; 3/3 resource lifecycles; G-013; G-014; G-015; PR #89 @ 2aae98e</x:v>
       </x:c>
       <x:c r="N21" s="170" t="str">
-        <x:v>7a8d746; PR #89</x:v>
+        <x:v>2aae98e; PR #89</x:v>
       </x:c>
       <x:c r="O21" s="170" t="str">
         <x:v>Needs merge/deploy authority, deployed commit identity, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P21" s="170" t="str">
-        <x:v>Branch proof is green; current production is deliberately not certified. Final target is 32/32 APIs plus 81/81 route/width checks.</x:v>
+        <x:v>Branch proof includes full resource lifecycles; current production is deliberately not certified. Final target remains 32/32 APIs plus 81/81 route/width checks.</x:v>
       </x:c>
       <x:c r="Q21" s="171" t="n">
-        <x:v>46215.92916666667</x:v>
+        <x:v>46215.93541666667</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -5248,7 +5248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea35987a55ab4568"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb4c3acc587a4002"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9269,53 +9269,137 @@
         <x:v>The shared repository now contains the beginner explanation and the full product, architecture, safety, rollout, evidence, and activation specification.</x:v>
       </x:c>
     </x:row>
-    <x:row r="94">
-      <x:c r="A94" s="133"/>
-      <x:c r="B94" s="165"/>
-      <x:c r="C94" s="133"/>
-      <x:c r="D94" s="133"/>
-      <x:c r="E94" s="133"/>
-      <x:c r="F94" s="133"/>
-      <x:c r="G94" s="133"/>
-      <x:c r="H94" s="133"/>
-      <x:c r="I94" s="133"/>
-      <x:c r="J94" s="133"/>
-      <x:c r="K94" s="133"/>
-      <x:c r="L94" s="133"/>
-      <x:c r="M94" s="133"/>
-      <x:c r="N94" s="133"/>
-    </x:row>
-    <x:row r="95">
-      <x:c r="A95" s="133"/>
-      <x:c r="B95" s="165"/>
-      <x:c r="C95" s="133"/>
-      <x:c r="D95" s="133"/>
-      <x:c r="E95" s="133"/>
-      <x:c r="F95" s="133"/>
-      <x:c r="G95" s="133"/>
-      <x:c r="H95" s="133"/>
-      <x:c r="I95" s="133"/>
-      <x:c r="J95" s="133"/>
-      <x:c r="K95" s="133"/>
-      <x:c r="L95" s="133"/>
-      <x:c r="M95" s="133"/>
-      <x:c r="N95" s="133"/>
-    </x:row>
-    <x:row r="96">
-      <x:c r="A96" s="133"/>
-      <x:c r="B96" s="165"/>
-      <x:c r="C96" s="133"/>
-      <x:c r="D96" s="133"/>
-      <x:c r="E96" s="133"/>
-      <x:c r="F96" s="133"/>
-      <x:c r="G96" s="133"/>
-      <x:c r="H96" s="133"/>
-      <x:c r="I96" s="133"/>
-      <x:c r="J96" s="133"/>
-      <x:c r="K96" s="133"/>
-      <x:c r="L96" s="133"/>
-      <x:c r="M96" s="133"/>
-      <x:c r="N96" s="133"/>
+    <x:row r="94" ht="116" customHeight="1">
+      <x:c r="A94" s="170" t="str">
+        <x:v>AL-089</x:v>
+      </x:c>
+      <x:c r="B94" s="171" t="n">
+        <x:v>46215.93541666667</x:v>
+      </x:c>
+      <x:c r="C94" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D94" s="170" t="str">
+        <x:v>Prove Settings and Inventory resource lifecycles</x:v>
+      </x:c>
+      <x:c r="E94" s="170" t="str">
+        <x:v>Added one synthetic-owner scenario that creates, lists, tenant-isolates, updates, explicitly deletes, and proves absence for equipment, preset notes, and chemical products.</x:v>
+      </x:c>
+      <x:c r="F94" s="170" t="str">
+        <x:v>Production Playwright API</x:v>
+      </x:c>
+      <x:c r="G94" s="170" t="str">
+        <x:v>All three owner resource lifecycles passed</x:v>
+      </x:c>
+      <x:c r="H94" s="170" t="str">
+        <x:v>Focused production run passed 1/1 in 2.4m. Every resource was removed before teardown; unrelated-owner update/delete attempts returned 404.</x:v>
+      </x:c>
+      <x:c r="I94" s="170" t="str">
+        <x:v>Authenticated production owner</x:v>
+      </x:c>
+      <x:c r="J94" s="170" t="str">
+        <x:v>e2e/desktop-critical-workflows.spec.ts</x:v>
+      </x:c>
+      <x:c r="K94" s="170" t="str">
+        <x:v>2aae98e; PR #89</x:v>
+      </x:c>
+      <x:c r="L94" s="170" t="str">
+        <x:v>Extend the same outcome depth to service documents, notifications, messaging, and inventory application logs.</x:v>
+      </x:c>
+      <x:c r="M94" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N94" s="170" t="str">
+        <x:v>No message, payment, provider, or customer-facing action ran; all writes stayed inside reserved synthetic companies.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="116" customHeight="1">
+      <x:c r="A95" s="170" t="str">
+        <x:v>AL-090</x:v>
+      </x:c>
+      <x:c r="B95" s="171" t="n">
+        <x:v>46215.93541666667</x:v>
+      </x:c>
+      <x:c r="C95" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D95" s="170" t="str">
+        <x:v>Publish resource lifecycle and synchronized PRD</x:v>
+      </x:c>
+      <x:c r="E95" s="170" t="str">
+        <x:v>Pushed PestFlow lifecycle commit 2aae98e, updated draft PR #89, and synchronized the complete 499-line PRD into Browser-Base-QA main.</x:v>
+      </x:c>
+      <x:c r="F95" s="170" t="str">
+        <x:v>Git + GitHub</x:v>
+      </x:c>
+      <x:c r="G95" s="170" t="str">
+        <x:v>Product test and canonical documentation published</x:v>
+      </x:c>
+      <x:c r="H95" s="170" t="str">
+        <x:v>PestFlow remote head matches 2aae98e. Browser-Base-QA commit 7788b30 has byte-identical PRD content to the PestFlow source.</x:v>
+      </x:c>
+      <x:c r="I95" s="170" t="str">
+        <x:v>Documentation + test code</x:v>
+      </x:c>
+      <x:c r="J95" s="170" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA/blob/main/docs/PRD.md</x:v>
+      </x:c>
+      <x:c r="K95" s="170" t="str">
+        <x:v>2aae98e; 7788b30; PR #89</x:v>
+      </x:c>
+      <x:c r="L95" s="170" t="str">
+        <x:v>Keep the standalone PRD synchronized as the next outcome layers are added.</x:v>
+      </x:c>
+      <x:c r="M95" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N95" s="170" t="str">
+        <x:v>This directly resolves the earlier repository-boundary mistake instead of letting the full PRD drift back into PestFlow only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="116" customHeight="1">
+      <x:c r="A96" s="170" t="str">
+        <x:v>AL-091</x:v>
+      </x:c>
+      <x:c r="B96" s="171" t="n">
+        <x:v>46215.93541666667</x:v>
+      </x:c>
+      <x:c r="C96" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="D96" s="170" t="str">
+        <x:v>Classify exact resource-lifecycle PR gate</x:v>
+      </x:c>
+      <x:c r="E96" s="170" t="str">
+        <x:v>Inspected the automatic PR release gate for exact PestFlow head 2aae98e and verified whether any QA command actually started.</x:v>
+      </x:c>
+      <x:c r="F96" s="170" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="G96" s="170" t="str">
+        <x:v>Cloud gate blocked before execution</x:v>
+      </x:c>
+      <x:c r="H96" s="170" t="str">
+        <x:v>Run 29211489437 had zero steps. Its annotation again reports failed recent payments or an exceeded spending limit.</x:v>
+      </x:c>
+      <x:c r="I96" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="J96" s="170" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/actions/runs/29211489437</x:v>
+      </x:c>
+      <x:c r="K96" s="170" t="str">
+        <x:v>2aae98e; PR #89</x:v>
+      </x:c>
+      <x:c r="L96" s="170" t="str">
+        <x:v>Restore Actions capacity and rerun exact-head gates; do not replace this with a product pass.</x:v>
+      </x:c>
+      <x:c r="M96" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="N96" s="170" t="str">
+        <x:v>PR remains mergeable/unstable. Local/live focused proof is real; cloud exact-head proof remains unavailable.</x:v>
+      </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="133"/>
@@ -9771,7 +9855,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95186bdafaf24079"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eb6547649264f94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12634,44 +12718,110 @@
         <x:v>The complete canonical PRD is published in Browser-Base-QA, not only PestFlow.</x:v>
       </x:c>
     </x:row>
-    <x:row r="84">
-      <x:c r="A84" s="133"/>
-      <x:c r="B84" s="133"/>
-      <x:c r="C84" s="133"/>
-      <x:c r="D84" s="133"/>
-      <x:c r="E84" s="133"/>
-      <x:c r="F84" s="133"/>
-      <x:c r="G84" s="133"/>
-      <x:c r="H84" s="133"/>
-      <x:c r="I84" s="165"/>
-      <x:c r="J84" s="133"/>
-      <x:c r="K84" s="133"/>
-    </x:row>
-    <x:row r="85">
-      <x:c r="A85" s="133"/>
-      <x:c r="B85" s="133"/>
-      <x:c r="C85" s="133"/>
-      <x:c r="D85" s="133"/>
-      <x:c r="E85" s="133"/>
-      <x:c r="F85" s="133"/>
-      <x:c r="G85" s="133"/>
-      <x:c r="H85" s="133"/>
-      <x:c r="I85" s="165"/>
-      <x:c r="J85" s="133"/>
-      <x:c r="K85" s="133"/>
-    </x:row>
-    <x:row r="86">
-      <x:c r="A86" s="133"/>
-      <x:c r="B86" s="133"/>
-      <x:c r="C86" s="133"/>
-      <x:c r="D86" s="133"/>
-      <x:c r="E86" s="133"/>
-      <x:c r="F86" s="133"/>
-      <x:c r="G86" s="133"/>
-      <x:c r="H86" s="133"/>
-      <x:c r="I86" s="165"/>
-      <x:c r="J86" s="133"/>
-      <x:c r="K86" s="133"/>
+    <x:row r="84" ht="78" customHeight="1">
+      <x:c r="A84" s="170" t="str">
+        <x:v>QA-079</x:v>
+      </x:c>
+      <x:c r="B84" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C84" s="170" t="str">
+        <x:v>Owner Settings/Inventory resource lifecycles</x:v>
+      </x:c>
+      <x:c r="D84" s="170" t="str">
+        <x:v>3 resources</x:v>
+      </x:c>
+      <x:c r="E84" s="170" t="str">
+        <x:v>Playwright API</x:v>
+      </x:c>
+      <x:c r="F84" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G84" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H84" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I84" s="171" t="n">
+        <x:v>46215.93541666667</x:v>
+      </x:c>
+      <x:c r="J84" s="170" t="str">
+        <x:v>1/1 in 2.4m</x:v>
+      </x:c>
+      <x:c r="K84" s="170" t="str">
+        <x:v>Equipment, preset notes, and chemical products passed create/list/isolate/update/delete/absence proof.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="78" customHeight="1">
+      <x:c r="A85" s="170" t="str">
+        <x:v>QA-080</x:v>
+      </x:c>
+      <x:c r="B85" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C85" s="170" t="str">
+        <x:v>Resource-lifecycle fixture teardown</x:v>
+      </x:c>
+      <x:c r="D85" s="170" t="str">
+        <x:v>5 synthetic accounts</x:v>
+      </x:c>
+      <x:c r="E85" s="170" t="str">
+        <x:v>Better Auth + API</x:v>
+      </x:c>
+      <x:c r="F85" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G85" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H85" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I85" s="171" t="n">
+        <x:v>46215.93541666667</x:v>
+      </x:c>
+      <x:c r="J85" s="170" t="str">
+        <x:v>5/5 deleted; 5/5 sessions cleared; 5/5 logins rejected</x:v>
+      </x:c>
+      <x:c r="K85" s="170" t="str">
+        <x:v>All explicitly created resources were removed before the company/account cascade.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="78" customHeight="1">
+      <x:c r="A86" s="170" t="str">
+        <x:v>QA-081</x:v>
+      </x:c>
+      <x:c r="B86" s="170" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C86" s="170" t="str">
+        <x:v>Exact resource-lifecycle PR release gate</x:v>
+      </x:c>
+      <x:c r="D86" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="E86" s="170" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F86" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G86" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H86" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I86" s="171" t="n">
+        <x:v>46215.93541666667</x:v>
+      </x:c>
+      <x:c r="J86" s="170" t="str">
+        <x:v>Run 29211489437: zero steps</x:v>
+      </x:c>
+      <x:c r="K86" s="170" t="str">
+        <x:v>Verified payment/spending refusal; no product or QA command started.</x:v>
+      </x:c>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="133"/>
@@ -13233,7 +13383,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f6d8f6fa70f4c94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59614015c8c34455"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14010,7 +14160,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red45dcc80d9a44cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd9772c4c38d4e74"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: log provider-safe communications proof
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb96cb2fe9a5f475f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R4d470a01ba0d496b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Re0c4a40a379f4163"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Ra0f248e069594d32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R0c548527944e499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R59e9273e57994242"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R83f79e67d2dd4d4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Rb866cbb68ab44ea5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R6cf6b1dee6b94bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rc5adc464d1f74918"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1337,7 +1337,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N96" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N99" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1359,7 +1359,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K86" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K89" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1761,12 +1761,12 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>81</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>56</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
@@ -1930,18 +1930,18 @@
         <x:v>Product failures and infrastructure failures stay separate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="126" customHeight="1">
+    <x:row r="17" ht="132" customHeight="1">
       <x:c r="A17" s="120" t="str">
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Live owner APIs pass 31/32 and all three Settings/Inventory resource lifecycles pass; historical route audit remains 69/78 until deploy.</x:v>
+        <x:v>Live owner APIs pass 31/32; Settings/Inventory and provider-safe communications lifecycles pass; historical route audit remains 69/78 until deploy.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ 2aae98e; Browser-Base-QA @ 7788b30 shared with yawbtng.</x:v>
+        <x:v>PestFlow PR #89 @ 7f067f4; Browser-Base-QA @ 7e2698f shared with yawbtng.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Activation</x:v>
@@ -1953,7 +1953,7 @@
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>Draft PR mergeable/unstable; run 29211489437 was zero-step billing blocked.</x:v>
+        <x:v>Draft PR mergeable/unstable; run 29211754954 was zero-step billing blocked.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2614,11 +2614,11 @@
         <x:v>/private/tmp/pestflow-desktop-qa-guardian/qa/guardian/desktop-journeys.json</x:v>
       </x:c>
       <x:c r="N8" s="113" t="str">
-        <x:v>2aae98e + Browser-Base-QA 7788b30; PR #89</x:v>
+        <x:v>7f067f4 + Browser-Base-QA 7e2698f; PR #89</x:v>
       </x:c>
       <x:c r="O8" s="113"/>
       <x:c r="P8" s="113" t="str">
-        <x:v>The standalone recorded owner session executes all 32 PestFlow API contracts; the complete PRD remains synchronized after resource lifecycle expansion.</x:v>
+        <x:v>The standalone recorded owner session executes 32 API contracts and the complete 508-line PRD remains synchronized.</x:v>
       </x:c>
       <x:c r="Q8" s="163" t="n">
         <x:v>46215.27099571759</x:v>
@@ -2815,19 +2815,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M12" s="166" t="str">
-        <x:v>31/32 live APIs; 3/3 resource lifecycles; 69/78 historical routes; 15/15 merged-branch focus</x:v>
+        <x:v>31/32 live APIs; 3/3 resource lifecycles; provider-safe communications 1/1; 69/78 historical routes</x:v>
       </x:c>
       <x:c r="N12" s="166" t="str">
-        <x:v>2aae98e; PR #89</x:v>
+        <x:v>7f067f4; PR #89</x:v>
       </x:c>
       <x:c r="O12" s="166" t="str">
         <x:v>Requires reviewed deploy and restored GitHub Actions capacity for final live certification.</x:v>
       </x:c>
       <x:c r="P12" s="166" t="str">
-        <x:v>Equipment, preset notes, and chemical products now have full production-safe CRUD/isolation proof. Current production /companies/branches remains the only API contract failure.</x:v>
+        <x:v>Documents/internal communication now have provider-safe persistence, isolation, cleanup, and preference proof. Current production /companies/branches remains the only API contract failure.</x:v>
       </x:c>
       <x:c r="Q12" s="167" t="n">
-        <x:v>46215.93541666667</x:v>
+        <x:v>46215.94097222222</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2922,11 +2922,11 @@
         <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/pull/89</x:v>
       </x:c>
       <x:c r="N14" s="166" t="str">
-        <x:v>2aae98e; PR #89</x:v>
+        <x:v>7f067f4; PR #89</x:v>
       </x:c>
       <x:c r="O14" s="166"/>
       <x:c r="P14" s="166" t="str">
-        <x:v>Latest focused live resource run passed 1/1 with verified 5/5 cleanup; exact-head cloud run 29211489437 was zero-step billing blocked.</x:v>
+        <x:v>Latest live provider-safe communications run passed 1/1 with 5/5 cleanup; exact-head cloud run 29211754954 was zero-step billing blocked.</x:v>
       </x:c>
       <x:c r="Q14" s="167" t="n">
         <x:v>46215.913194444445</x:v>
@@ -3021,16 +3021,16 @@
         <x:v>Risk-selected + full production</x:v>
       </x:c>
       <x:c r="M16" s="166" t="str">
-        <x:v>Browser-Base-QA @ 7788b30; PR #89 @ 2aae98e</x:v>
+        <x:v>Browser-Base-QA @ 7e2698f; PR #89 @ 7f067f4</x:v>
       </x:c>
       <x:c r="N16" s="166" t="str">
-        <x:v>Standalone API executor and complete PRD are current; production promotion wiring remains pending.</x:v>
+        <x:v>Standalone API executor and complete PRD are current; promotion wiring remains pending.</x:v>
       </x:c>
       <x:c r="O16" s="166" t="str">
         <x:v>Needs Browserbase secrets/context, deploy ownership, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P16" s="166" t="str">
-        <x:v>Live read contracts are 31/32; owner equipment/preset/chemical lifecycles pass. Deploy reviewed PestFlow head, then require 32/32 plus 81/81.</x:v>
+        <x:v>Live reads are 31/32; resource and provider-safe communications lifecycles pass. Deploy reviewed head, then require 32/32 plus 81/81.</x:v>
       </x:c>
       <x:c r="Q16" s="167" t="n">
         <x:v>46215.27099571759</x:v>
@@ -3282,19 +3282,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M21" s="170" t="str">
-        <x:v>31/32 production APIs; 3/3 resource lifecycles; G-013; G-014; G-015; PR #89 @ 2aae98e</x:v>
+        <x:v>31/32 production APIs; resource + communications lifecycles pass; G-013; G-014; G-015; PR #89 @ 7f067f4</x:v>
       </x:c>
       <x:c r="N21" s="170" t="str">
-        <x:v>2aae98e; PR #89</x:v>
+        <x:v>7f067f4; PR #89</x:v>
       </x:c>
       <x:c r="O21" s="170" t="str">
         <x:v>Needs merge/deploy authority, deployed commit identity, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P21" s="170" t="str">
-        <x:v>Branch proof includes full resource lifecycles; current production is deliberately not certified. Final target remains 32/32 APIs plus 81/81 route/width checks.</x:v>
+        <x:v>Branch proof now includes Settings/Inventory and provider-safe communication outcomes; current production is not certified.</x:v>
       </x:c>
       <x:c r="Q21" s="171" t="n">
-        <x:v>46215.93541666667</x:v>
+        <x:v>46215.94097222222</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -5248,7 +5248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb4c3acc587a4002"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a049563ae474e27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9401,53 +9401,137 @@
         <x:v>PR remains mergeable/unstable. Local/live focused proof is real; cloud exact-head proof remains unavailable.</x:v>
       </x:c>
     </x:row>
-    <x:row r="97">
-      <x:c r="A97" s="133"/>
-      <x:c r="B97" s="165"/>
-      <x:c r="C97" s="133"/>
-      <x:c r="D97" s="133"/>
-      <x:c r="E97" s="133"/>
-      <x:c r="F97" s="133"/>
-      <x:c r="G97" s="133"/>
-      <x:c r="H97" s="133"/>
-      <x:c r="I97" s="133"/>
-      <x:c r="J97" s="133"/>
-      <x:c r="K97" s="133"/>
-      <x:c r="L97" s="133"/>
-      <x:c r="M97" s="133"/>
-      <x:c r="N97" s="133"/>
-    </x:row>
-    <x:row r="98">
-      <x:c r="A98" s="133"/>
-      <x:c r="B98" s="165"/>
-      <x:c r="C98" s="133"/>
-      <x:c r="D98" s="133"/>
-      <x:c r="E98" s="133"/>
-      <x:c r="F98" s="133"/>
-      <x:c r="G98" s="133"/>
-      <x:c r="H98" s="133"/>
-      <x:c r="I98" s="133"/>
-      <x:c r="J98" s="133"/>
-      <x:c r="K98" s="133"/>
-      <x:c r="L98" s="133"/>
-      <x:c r="M98" s="133"/>
-      <x:c r="N98" s="133"/>
-    </x:row>
-    <x:row r="99">
-      <x:c r="A99" s="133"/>
-      <x:c r="B99" s="165"/>
-      <x:c r="C99" s="133"/>
-      <x:c r="D99" s="133"/>
-      <x:c r="E99" s="133"/>
-      <x:c r="F99" s="133"/>
-      <x:c r="G99" s="133"/>
-      <x:c r="H99" s="133"/>
-      <x:c r="I99" s="133"/>
-      <x:c r="J99" s="133"/>
-      <x:c r="K99" s="133"/>
-      <x:c r="L99" s="133"/>
-      <x:c r="M99" s="133"/>
-      <x:c r="N99" s="133"/>
+    <x:row r="97" ht="116" customHeight="1">
+      <x:c r="A97" s="170" t="str">
+        <x:v>AL-092</x:v>
+      </x:c>
+      <x:c r="B97" s="171" t="n">
+        <x:v>46215.94097222222</x:v>
+      </x:c>
+      <x:c r="C97" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D97" s="170" t="str">
+        <x:v>Prove provider-safe documents and internal communications</x:v>
+      </x:c>
+      <x:c r="E97" s="170" t="str">
+        <x:v>Added one synthetic-owner scenario for an unsigned recipient-free service document, response-template archive, disabled auto-response rule, teammate message read state, tenant isolation, and notification preference restore.</x:v>
+      </x:c>
+      <x:c r="F97" s="170" t="str">
+        <x:v>Production Playwright API</x:v>
+      </x:c>
+      <x:c r="G97" s="170" t="str">
+        <x:v>Provider-safe communications lifecycle passed</x:v>
+      </x:c>
+      <x:c r="H97" s="170" t="str">
+        <x:v>Focused production run passed 1/1 in 2.4m. It used no signatures, recipient addresses, sends, enabled rules, payments, or external provider calls.</x:v>
+      </x:c>
+      <x:c r="I97" s="170" t="str">
+        <x:v>Authenticated production owner</x:v>
+      </x:c>
+      <x:c r="J97" s="170" t="str">
+        <x:v>e2e/desktop-critical-workflows.spec.ts</x:v>
+      </x:c>
+      <x:c r="K97" s="170" t="str">
+        <x:v>7f067f4; PR #89</x:v>
+      </x:c>
+      <x:c r="L97" s="170" t="str">
+        <x:v>Add the next safe outcome layer for chemical applications, job equipment use, and Website Chat tenant state.</x:v>
+      </x:c>
+      <x:c r="M97" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N97" s="170" t="str">
+        <x:v>Response records were archived/deleted, preferences restored, cross-company access denied, and remaining synthetic rows cascaded with account cleanup.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="116" customHeight="1">
+      <x:c r="A98" s="170" t="str">
+        <x:v>AL-093</x:v>
+      </x:c>
+      <x:c r="B98" s="171" t="n">
+        <x:v>46215.94097222222</x:v>
+      </x:c>
+      <x:c r="C98" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D98" s="170" t="str">
+        <x:v>Publish communications lifecycle and synchronized PRD</x:v>
+      </x:c>
+      <x:c r="E98" s="170" t="str">
+        <x:v>Pushed PestFlow commit 7f067f4, refreshed PR #89, and synchronized the complete 508-line PRD into Browser-Base-QA.</x:v>
+      </x:c>
+      <x:c r="F98" s="170" t="str">
+        <x:v>Git + GitHub</x:v>
+      </x:c>
+      <x:c r="G98" s="170" t="str">
+        <x:v>Test and canonical PRD published</x:v>
+      </x:c>
+      <x:c r="H98" s="170" t="str">
+        <x:v>PestFlow remote head matches 7f067f4. Browser-Base-QA commit 7e2698f has byte-identical PRD content to PestFlow.</x:v>
+      </x:c>
+      <x:c r="I98" s="170" t="str">
+        <x:v>Documentation + test code</x:v>
+      </x:c>
+      <x:c r="J98" s="170" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA/blob/main/docs/PRD.md</x:v>
+      </x:c>
+      <x:c r="K98" s="170" t="str">
+        <x:v>7f067f4; 7e2698f; PR #89</x:v>
+      </x:c>
+      <x:c r="L98" s="170" t="str">
+        <x:v>Keep the shared PRD and tracker current through the next outcome layer.</x:v>
+      </x:c>
+      <x:c r="M98" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N98" s="170" t="str">
+        <x:v>The comprehensive PRD remains in the shared repository after this new PestFlow-only regression was added.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="116" customHeight="1">
+      <x:c r="A99" s="170" t="str">
+        <x:v>AL-094</x:v>
+      </x:c>
+      <x:c r="B99" s="171" t="n">
+        <x:v>46215.94097222222</x:v>
+      </x:c>
+      <x:c r="C99" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="D99" s="170" t="str">
+        <x:v>Classify exact communications-lifecycle PR gate</x:v>
+      </x:c>
+      <x:c r="E99" s="170" t="str">
+        <x:v>Inspected the automatic release gate for exact PestFlow head 7f067f4 and verified whether any command executed.</x:v>
+      </x:c>
+      <x:c r="F99" s="170" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="G99" s="170" t="str">
+        <x:v>Cloud gate blocked before execution</x:v>
+      </x:c>
+      <x:c r="H99" s="170" t="str">
+        <x:v>Run 29211754954 had zero steps and the same failed-payment or spending-limit annotation.</x:v>
+      </x:c>
+      <x:c r="I99" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="J99" s="170" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/actions/runs/29211754954</x:v>
+      </x:c>
+      <x:c r="K99" s="170" t="str">
+        <x:v>7f067f4; PR #89</x:v>
+      </x:c>
+      <x:c r="L99" s="170" t="str">
+        <x:v>Restore Actions capacity and rerun exact-head gates; retain this as infrastructure evidence.</x:v>
+      </x:c>
+      <x:c r="M99" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="N99" s="170" t="str">
+        <x:v>PR remains mergeable/unstable. Live focused proof passed, but exact-head cloud proof is unavailable.</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="133"/>
@@ -9855,7 +9939,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0eb6547649264f94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42e5746b46114bfa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12823,44 +12907,110 @@
         <x:v>Verified payment/spending refusal; no product or QA command started.</x:v>
       </x:c>
     </x:row>
-    <x:row r="87">
-      <x:c r="A87" s="133"/>
-      <x:c r="B87" s="133"/>
-      <x:c r="C87" s="133"/>
-      <x:c r="D87" s="133"/>
-      <x:c r="E87" s="133"/>
-      <x:c r="F87" s="133"/>
-      <x:c r="G87" s="133"/>
-      <x:c r="H87" s="133"/>
-      <x:c r="I87" s="165"/>
-      <x:c r="J87" s="133"/>
-      <x:c r="K87" s="133"/>
-    </x:row>
-    <x:row r="88">
-      <x:c r="A88" s="133"/>
-      <x:c r="B88" s="133"/>
-      <x:c r="C88" s="133"/>
-      <x:c r="D88" s="133"/>
-      <x:c r="E88" s="133"/>
-      <x:c r="F88" s="133"/>
-      <x:c r="G88" s="133"/>
-      <x:c r="H88" s="133"/>
-      <x:c r="I88" s="165"/>
-      <x:c r="J88" s="133"/>
-      <x:c r="K88" s="133"/>
-    </x:row>
-    <x:row r="89">
-      <x:c r="A89" s="133"/>
-      <x:c r="B89" s="133"/>
-      <x:c r="C89" s="133"/>
-      <x:c r="D89" s="133"/>
-      <x:c r="E89" s="133"/>
-      <x:c r="F89" s="133"/>
-      <x:c r="G89" s="133"/>
-      <x:c r="H89" s="133"/>
-      <x:c r="I89" s="165"/>
-      <x:c r="J89" s="133"/>
-      <x:c r="K89" s="133"/>
+    <x:row r="87" ht="78" customHeight="1">
+      <x:c r="A87" s="170" t="str">
+        <x:v>QA-082</x:v>
+      </x:c>
+      <x:c r="B87" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C87" s="170" t="str">
+        <x:v>Provider-safe documents and communications</x:v>
+      </x:c>
+      <x:c r="D87" s="170" t="str">
+        <x:v>5 outcome groups</x:v>
+      </x:c>
+      <x:c r="E87" s="170" t="str">
+        <x:v>Playwright API</x:v>
+      </x:c>
+      <x:c r="F87" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G87" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H87" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I87" s="171" t="n">
+        <x:v>46215.94097222222</x:v>
+      </x:c>
+      <x:c r="J87" s="170" t="str">
+        <x:v>1/1 in 2.4m</x:v>
+      </x:c>
+      <x:c r="K87" s="170" t="str">
+        <x:v>Unsigned document, response template, disabled rule, internal message read, and preference restore passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="78" customHeight="1">
+      <x:c r="A88" s="170" t="str">
+        <x:v>QA-083</x:v>
+      </x:c>
+      <x:c r="B88" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C88" s="170" t="str">
+        <x:v>Communications-lifecycle fixture teardown</x:v>
+      </x:c>
+      <x:c r="D88" s="170" t="str">
+        <x:v>5 synthetic accounts</x:v>
+      </x:c>
+      <x:c r="E88" s="170" t="str">
+        <x:v>Better Auth + API</x:v>
+      </x:c>
+      <x:c r="F88" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G88" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H88" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I88" s="171" t="n">
+        <x:v>46215.94097222222</x:v>
+      </x:c>
+      <x:c r="J88" s="170" t="str">
+        <x:v>5/5 deleted; 5/5 sessions cleared; 5/5 logins rejected</x:v>
+      </x:c>
+      <x:c r="K88" s="170" t="str">
+        <x:v>No provider action ran and no synthetic account remained usable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="78" customHeight="1">
+      <x:c r="A89" s="170" t="str">
+        <x:v>QA-084</x:v>
+      </x:c>
+      <x:c r="B89" s="170" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C89" s="170" t="str">
+        <x:v>Exact communications-lifecycle PR gate</x:v>
+      </x:c>
+      <x:c r="D89" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="E89" s="170" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F89" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G89" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H89" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I89" s="171" t="n">
+        <x:v>46215.94097222222</x:v>
+      </x:c>
+      <x:c r="J89" s="170" t="str">
+        <x:v>Run 29211754954: zero steps</x:v>
+      </x:c>
+      <x:c r="K89" s="170" t="str">
+        <x:v>Verified payment/spending refusal; no product or QA command started.</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="133"/>
@@ -13383,7 +13533,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59614015c8c34455"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5d9ecc38d9a4688"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14160,7 +14310,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd9772c4c38d4e74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R680f6b7dc1ee47e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record operational tenant-boundary QA
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R59e9273e57994242"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R83f79e67d2dd4d4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Rb866cbb68ab44ea5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R6cf6b1dee6b94bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rc5adc464d1f74918"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re95865165f6842f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R061ac27910204b67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Re308fae81fbf4c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R026ec276fc8441c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R07f421a5550f457e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1337,7 +1337,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N99" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1359,7 +1359,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K89" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K94" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1378,7 +1378,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Gap ID"/>
     <x:tableColumn id="2" name="Found During Task"/>
@@ -1761,22 +1761,22 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>84</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>58</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Failed")</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F9" s="141"/>
       <x:c r="G9" s="138" t="n">
         <x:f>COUNTIFS('Product Gaps'!$A$6:$A$200,"&lt;&gt;",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Closed",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Resolved",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Mitigated")</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H9" s="139"/>
     </x:row>
@@ -1930,30 +1930,30 @@
         <x:v>Product failures and infrastructure failures stay separate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="132" customHeight="1">
+    <x:row r="17" ht="148" customHeight="1">
       <x:c r="A17" s="120" t="str">
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Live owner APIs pass 31/32; Settings/Inventory and provider-safe communications lifecycles pass; historical route audit remains 69/78 until deploy.</x:v>
+        <x:v>Live owner APIs pass 31/32 and safe lifecycles pass, but current production accepts both tested cross-company operational writes (200/200).</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ 7f067f4; Browser-Base-QA @ 7e2698f shared with yawbtng.</x:v>
+        <x:v>PestFlow PR #89 @ cad0544; Browser-Base-QA @ 343a154 shared with yawbtng; complete 522-line PRD synchronized.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Activation</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>Restore Actions; deploy reviewed fixes; add Browserbase secrets/context; require exact-SHA 32/32 API and 81/81 route gates.</x:v>
+        <x:v>Restore Actions; deploy cad0544; prove exact-SHA 32/32 APIs, 81/81 routes, and operational tenant isolation 404/404.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>Draft PR mergeable/unstable; run 29211754954 was zero-step billing blocked.</x:v>
+        <x:v>Draft PR mergeable/unstable; run 29212212813 was zero-step billing blocked, while full local branch gates passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2614,11 +2614,11 @@
         <x:v>/private/tmp/pestflow-desktop-qa-guardian/qa/guardian/desktop-journeys.json</x:v>
       </x:c>
       <x:c r="N8" s="113" t="str">
-        <x:v>7f067f4 + Browser-Base-QA 7e2698f; PR #89</x:v>
+        <x:v>cad0544 + Browser-Base-QA 343a154; PR #89</x:v>
       </x:c>
       <x:c r="O8" s="113"/>
       <x:c r="P8" s="113" t="str">
-        <x:v>The standalone recorded owner session executes 32 API contracts and the complete 508-line PRD remains synchronized.</x:v>
+        <x:v>The standalone executor, 32 API contracts, tenant-boundary evidence, and complete 522-line PRD are synchronized.</x:v>
       </x:c>
       <x:c r="Q8" s="163" t="n">
         <x:v>46215.27099571759</x:v>
@@ -2815,19 +2815,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M12" s="166" t="str">
-        <x:v>31/32 live APIs; 3/3 resource lifecycles; provider-safe communications 1/1; 69/78 historical routes</x:v>
+        <x:v>31/32 live APIs; resource + communications pass; operational tenant isolation fails 200/200</x:v>
       </x:c>
       <x:c r="N12" s="166" t="str">
-        <x:v>7f067f4; PR #89</x:v>
+        <x:v>cad0544; PR #89</x:v>
       </x:c>
       <x:c r="O12" s="166" t="str">
-        <x:v>Requires reviewed deploy and restored GitHub Actions capacity for final live certification.</x:v>
+        <x:v>Requires reviewed deploy, 404/404 production rerun, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P12" s="166" t="str">
-        <x:v>Documents/internal communication now have provider-safe persistence, isolation, cleanup, and preference proof. Current production /companies/branches remains the only API contract failure.</x:v>
+        <x:v>Current production is not certified: cross-company operational references are accepted. Branch repair and full local gates pass.</x:v>
       </x:c>
       <x:c r="Q12" s="167" t="n">
-        <x:v>46215.94097222222</x:v>
+        <x:v>46215.95486111111</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2922,11 +2922,11 @@
         <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/pull/89</x:v>
       </x:c>
       <x:c r="N14" s="166" t="str">
-        <x:v>7f067f4; PR #89</x:v>
+        <x:v>cad0544; PR #89</x:v>
       </x:c>
       <x:c r="O14" s="166"/>
       <x:c r="P14" s="166" t="str">
-        <x:v>Latest live provider-safe communications run passed 1/1 with 5/5 cleanup; exact-head cloud run 29211754954 was zero-step billing blocked.</x:v>
+        <x:v>Latest production tenant test failed 200/200 with complete cleanup; exact-head cloud run 29212212813 was zero-step billing blocked.</x:v>
       </x:c>
       <x:c r="Q14" s="167" t="n">
         <x:v>46215.913194444445</x:v>
@@ -3021,7 +3021,7 @@
         <x:v>Risk-selected + full production</x:v>
       </x:c>
       <x:c r="M16" s="166" t="str">
-        <x:v>Browser-Base-QA @ 7e2698f; PR #89 @ 7f067f4</x:v>
+        <x:v>Browser-Base-QA @ 343a154; PR #89 @ cad0544</x:v>
       </x:c>
       <x:c r="N16" s="166" t="str">
         <x:v>Standalone API executor and complete PRD are current; promotion wiring remains pending.</x:v>
@@ -3030,7 +3030,7 @@
         <x:v>Needs Browserbase secrets/context, deploy ownership, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P16" s="166" t="str">
-        <x:v>Live reads are 31/32; resource and provider-safe communications lifecycles pass. Deploy reviewed head, then require 32/32 plus 81/81.</x:v>
+        <x:v>Deploy reviewed head, then require 32/32 APIs, 81/81 routes, and operational isolation 404/404 on the exact SHA.</x:v>
       </x:c>
       <x:c r="Q16" s="167" t="n">
         <x:v>46215.27099571759</x:v>
@@ -3282,19 +3282,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M21" s="170" t="str">
-        <x:v>31/32 production APIs; resource + communications lifecycles pass; G-013; G-014; G-015; PR #89 @ 7f067f4</x:v>
+        <x:v>31/32 production APIs; safe lifecycles pass; G-013–G-016; PR #89 @ cad0544</x:v>
       </x:c>
       <x:c r="N21" s="170" t="str">
-        <x:v>7f067f4; PR #89</x:v>
+        <x:v>cad0544; PR #89</x:v>
       </x:c>
       <x:c r="O21" s="170" t="str">
-        <x:v>Needs merge/deploy authority, deployed commit identity, and restored GitHub Actions capacity.</x:v>
+        <x:v>Needs merge/deploy authority, deployed commit identity, production 404/404, and restored Actions capacity.</x:v>
       </x:c>
       <x:c r="P21" s="170" t="str">
-        <x:v>Branch proof now includes Settings/Inventory and provider-safe communication outcomes; current production is not certified.</x:v>
+        <x:v>Branch proof includes 775 unit tests and the operational tenant repair; current production remains uncertified.</x:v>
       </x:c>
       <x:c r="Q21" s="171" t="n">
-        <x:v>46215.94097222222</x:v>
+        <x:v>46215.95486111111</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -5248,7 +5248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a049563ae474e27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1272a6b6a18e4ad2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9533,85 +9533,225 @@
         <x:v>PR remains mergeable/unstable. Live focused proof passed, but exact-head cloud proof is unavailable.</x:v>
       </x:c>
     </x:row>
-    <x:row r="100">
-      <x:c r="A100" s="133"/>
-      <x:c r="B100" s="165"/>
-      <x:c r="C100" s="133"/>
-      <x:c r="D100" s="133"/>
-      <x:c r="E100" s="133"/>
-      <x:c r="F100" s="133"/>
-      <x:c r="G100" s="133"/>
-      <x:c r="H100" s="133"/>
-      <x:c r="I100" s="133"/>
-      <x:c r="J100" s="133"/>
-      <x:c r="K100" s="133"/>
-      <x:c r="L100" s="133"/>
-      <x:c r="M100" s="133"/>
-      <x:c r="N100" s="133"/>
-    </x:row>
-    <x:row r="101">
-      <x:c r="A101" s="133"/>
-      <x:c r="B101" s="165"/>
-      <x:c r="C101" s="133"/>
-      <x:c r="D101" s="133"/>
-      <x:c r="E101" s="133"/>
-      <x:c r="F101" s="133"/>
-      <x:c r="G101" s="133"/>
-      <x:c r="H101" s="133"/>
-      <x:c r="I101" s="133"/>
-      <x:c r="J101" s="133"/>
-      <x:c r="K101" s="133"/>
-      <x:c r="L101" s="133"/>
-      <x:c r="M101" s="133"/>
-      <x:c r="N101" s="133"/>
-    </x:row>
-    <x:row r="102">
-      <x:c r="A102" s="133"/>
-      <x:c r="B102" s="165"/>
-      <x:c r="C102" s="133"/>
-      <x:c r="D102" s="133"/>
-      <x:c r="E102" s="133"/>
-      <x:c r="F102" s="133"/>
-      <x:c r="G102" s="133"/>
-      <x:c r="H102" s="133"/>
-      <x:c r="I102" s="133"/>
-      <x:c r="J102" s="133"/>
-      <x:c r="K102" s="133"/>
-      <x:c r="L102" s="133"/>
-      <x:c r="M102" s="133"/>
-      <x:c r="N102" s="133"/>
-    </x:row>
-    <x:row r="103">
-      <x:c r="A103" s="133"/>
-      <x:c r="B103" s="165"/>
-      <x:c r="C103" s="133"/>
-      <x:c r="D103" s="133"/>
-      <x:c r="E103" s="133"/>
-      <x:c r="F103" s="133"/>
-      <x:c r="G103" s="133"/>
-      <x:c r="H103" s="133"/>
-      <x:c r="I103" s="133"/>
-      <x:c r="J103" s="133"/>
-      <x:c r="K103" s="133"/>
-      <x:c r="L103" s="133"/>
-      <x:c r="M103" s="133"/>
-      <x:c r="N103" s="133"/>
-    </x:row>
-    <x:row r="104">
-      <x:c r="A104" s="133"/>
-      <x:c r="B104" s="165"/>
-      <x:c r="C104" s="133"/>
-      <x:c r="D104" s="133"/>
-      <x:c r="E104" s="133"/>
-      <x:c r="F104" s="133"/>
-      <x:c r="G104" s="133"/>
-      <x:c r="H104" s="133"/>
-      <x:c r="I104" s="133"/>
-      <x:c r="J104" s="133"/>
-      <x:c r="K104" s="133"/>
-      <x:c r="L104" s="133"/>
-      <x:c r="M104" s="133"/>
-      <x:c r="N104" s="133"/>
+    <x:row r="100" ht="124" customHeight="1">
+      <x:c r="A100" s="170" t="str">
+        <x:v>AL-095</x:v>
+      </x:c>
+      <x:c r="B100" s="171" t="n">
+        <x:v>46215.95486111111</x:v>
+      </x:c>
+      <x:c r="C100" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D100" s="170" t="str">
+        <x:v>Audit operational inventory tenant references</x:v>
+      </x:c>
+      <x:c r="E100" s="170" t="str">
+        <x:v>Traced the create paths for job equipment usage and chemical application logs and found that referenced job, equipment, customer, and technician IDs were not proven to belong to the authenticated company.</x:v>
+      </x:c>
+      <x:c r="F100" s="170" t="str">
+        <x:v>Route and schema inspection</x:v>
+      </x:c>
+      <x:c r="G100" s="170" t="str">
+        <x:v>Critical tenant-boundary gap confirmed</x:v>
+      </x:c>
+      <x:c r="H100" s="170" t="str">
+        <x:v>The insert company_id was scoped, but related record IDs could point at a different company and later appear through joined operational history.</x:v>
+      </x:c>
+      <x:c r="I100" s="170" t="str">
+        <x:v>Desktop operational APIs</x:v>
+      </x:c>
+      <x:c r="J100" s="170" t="str">
+        <x:v>server/routes/job-equipment-used.ts; server/routes/chemical-logs.ts</x:v>
+      </x:c>
+      <x:c r="K100" s="170" t="str">
+        <x:v>G-016; PR #89</x:v>
+      </x:c>
+      <x:c r="L100" s="170" t="str">
+        <x:v>Reproduce with isolated synthetic companies, then repair every referenced-ID boundary.</x:v>
+      </x:c>
+      <x:c r="M100" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N100" s="170" t="str">
+        <x:v>This is an integrity and data-isolation defect, not merely a browser presentation failure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="124" customHeight="1">
+      <x:c r="A101" s="170" t="str">
+        <x:v>AL-096</x:v>
+      </x:c>
+      <x:c r="B101" s="171" t="n">
+        <x:v>46215.95486111111</x:v>
+      </x:c>
+      <x:c r="C101" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D101" s="170" t="str">
+        <x:v>Prove current production accepts cross-company references</x:v>
+      </x:c>
+      <x:c r="E101" s="170" t="str">
+        <x:v>Ran the controlled synthetic-owner scenario twice against production, attempting chemical-log and job-equipment writes with IDs owned by an unrelated synthetic company.</x:v>
+      </x:c>
+      <x:c r="F101" s="170" t="str">
+        <x:v>Production Playwright API</x:v>
+      </x:c>
+      <x:c r="G101" s="170" t="str">
+        <x:v>Current production failed tenant isolation</x:v>
+      </x:c>
+      <x:c r="H101" s="170" t="str">
+        <x:v>Both prohibited writes returned HTTP 200 instead of 404 in both discovery runs.</x:v>
+      </x:c>
+      <x:c r="I101" s="170" t="str">
+        <x:v>Authenticated synthetic owners</x:v>
+      </x:c>
+      <x:c r="J101" s="170" t="str">
+        <x:v>e2e/desktop-critical-workflows.spec.ts</x:v>
+      </x:c>
+      <x:c r="K101" s="170" t="str">
+        <x:v>G-016</x:v>
+      </x:c>
+      <x:c r="L101" s="170" t="str">
+        <x:v>Keep production uncertified until the repaired commit is deployed and both writes return 404.</x:v>
+      </x:c>
+      <x:c r="M101" s="170" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="N101" s="170" t="str">
+        <x:v>Each run deleted 5/5 synthetic accounts, cleared 5/5 sessions, and confirmed 5/5 logins were rejected; explicit usage cleanup also completed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="124" customHeight="1">
+      <x:c r="A102" s="170" t="str">
+        <x:v>AL-097</x:v>
+      </x:c>
+      <x:c r="B102" s="171" t="n">
+        <x:v>46215.95486111111</x:v>
+      </x:c>
+      <x:c r="C102" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="D102" s="170" t="str">
+        <x:v>Enforce operational inventory tenant scope</x:v>
+      </x:c>
+      <x:c r="E102" s="170" t="str">
+        <x:v>Added UUID validation and company-scoped existence checks before job-equipment and chemical-log inserts, plus deterministic regression coverage for invalid, foreign, and valid references.</x:v>
+      </x:c>
+      <x:c r="F102" s="170" t="str">
+        <x:v>PestFlow API + Vitest</x:v>
+      </x:c>
+      <x:c r="G102" s="170" t="str">
+        <x:v>Branch repair implemented and verified</x:v>
+      </x:c>
+      <x:c r="H102" s="170" t="str">
+        <x:v>Focused tenant tests passed 6/6. Full branch gates passed 775/775 unit, 45/45 Guardian policy, 16/16 incident, TypeScript, focused lint, and the 5,699-module production build.</x:v>
+      </x:c>
+      <x:c r="I102" s="170" t="str">
+        <x:v>Desktop operational APIs</x:v>
+      </x:c>
+      <x:c r="J102" s="170" t="str">
+        <x:v>src/test/operationalInventoryTenantScope.test.ts</x:v>
+      </x:c>
+      <x:c r="K102" s="170" t="str">
+        <x:v>cad0544; PR #89</x:v>
+      </x:c>
+      <x:c r="L102" s="170" t="str">
+        <x:v>Deploy the reviewed commit and rerun the exact production isolation scenario.</x:v>
+      </x:c>
+      <x:c r="M102" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N102" s="170" t="str">
+        <x:v>The branch now returns 404 before insertion whenever a supplied related record is not owned by the authenticated company.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="124" customHeight="1">
+      <x:c r="A103" s="170" t="str">
+        <x:v>AL-098</x:v>
+      </x:c>
+      <x:c r="B103" s="171" t="n">
+        <x:v>46215.95486111111</x:v>
+      </x:c>
+      <x:c r="C103" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D103" s="170" t="str">
+        <x:v>Publish tenant-boundary fix and synchronized PRD</x:v>
+      </x:c>
+      <x:c r="E103" s="170" t="str">
+        <x:v>Pushed PestFlow commit cad0544 and synchronized the complete 522-line PRD, including the live failure evidence and certification condition, into Browser-Base-QA.</x:v>
+      </x:c>
+      <x:c r="F103" s="170" t="str">
+        <x:v>Git + GitHub</x:v>
+      </x:c>
+      <x:c r="G103" s="170" t="str">
+        <x:v>Repair and canonical documentation published</x:v>
+      </x:c>
+      <x:c r="H103" s="170" t="str">
+        <x:v>PestFlow PR #89 points at cad0544. Browser-Base-QA commit 343a154 contains a byte-identical PRD.</x:v>
+      </x:c>
+      <x:c r="I103" s="170" t="str">
+        <x:v>Documentation + test code</x:v>
+      </x:c>
+      <x:c r="J103" s="170" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA/blob/main/docs/PRD.md</x:v>
+      </x:c>
+      <x:c r="K103" s="170" t="str">
+        <x:v>cad0544; 343a154; PR #89</x:v>
+      </x:c>
+      <x:c r="L103" s="170" t="str">
+        <x:v>Keep tracker evidence current and require deployed 404/404 proof before closure.</x:v>
+      </x:c>
+      <x:c r="M103" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N103" s="170" t="str">
+        <x:v>The shared repository now explains the defect, repair, safety controls, and remaining production boundary in beginner-friendly and technical terms.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="124" customHeight="1">
+      <x:c r="A104" s="170" t="str">
+        <x:v>AL-099</x:v>
+      </x:c>
+      <x:c r="B104" s="171" t="n">
+        <x:v>46215.95486111111</x:v>
+      </x:c>
+      <x:c r="C104" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="D104" s="170" t="str">
+        <x:v>Classify exact tenant-boundary PR gate</x:v>
+      </x:c>
+      <x:c r="E104" s="170" t="str">
+        <x:v>Inspected the automatic release gate for exact PestFlow head cad0544 and verified whether a validation command executed.</x:v>
+      </x:c>
+      <x:c r="F104" s="170" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="G104" s="170" t="str">
+        <x:v>Cloud gate blocked before execution</x:v>
+      </x:c>
+      <x:c r="H104" s="170" t="str">
+        <x:v>Run 29212212813, job 86701739111 had zero steps; GitHub annotated a failed-payment or spending-limit refusal.</x:v>
+      </x:c>
+      <x:c r="I104" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="J104" s="170" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/actions/runs/29212212813</x:v>
+      </x:c>
+      <x:c r="K104" s="170" t="str">
+        <x:v>cad0544; PR #89</x:v>
+      </x:c>
+      <x:c r="L104" s="170" t="str">
+        <x:v>Restore Actions capacity and rerun exact-head gates; retain the local and live evidence separately.</x:v>
+      </x:c>
+      <x:c r="M104" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="N104" s="170" t="str">
+        <x:v>PR remains mergeable/unstable. The red check is infrastructure evidence and did not execute product tests.</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="133"/>
@@ -9939,7 +10079,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42e5746b46114bfa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceb10aa6f5c24c1c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13012,70 +13152,180 @@
         <x:v>Verified payment/spending refusal; no product or QA command started.</x:v>
       </x:c>
     </x:row>
-    <x:row r="90">
-      <x:c r="A90" s="133"/>
-      <x:c r="B90" s="133"/>
-      <x:c r="C90" s="133"/>
-      <x:c r="D90" s="133"/>
-      <x:c r="E90" s="133"/>
-      <x:c r="F90" s="133"/>
-      <x:c r="G90" s="133"/>
-      <x:c r="H90" s="133"/>
-      <x:c r="I90" s="165"/>
-      <x:c r="J90" s="133"/>
-      <x:c r="K90" s="133"/>
-    </x:row>
-    <x:row r="91">
-      <x:c r="A91" s="133"/>
-      <x:c r="B91" s="133"/>
-      <x:c r="C91" s="133"/>
-      <x:c r="D91" s="133"/>
-      <x:c r="E91" s="133"/>
-      <x:c r="F91" s="133"/>
-      <x:c r="G91" s="133"/>
-      <x:c r="H91" s="133"/>
-      <x:c r="I91" s="165"/>
-      <x:c r="J91" s="133"/>
-      <x:c r="K91" s="133"/>
-    </x:row>
-    <x:row r="92">
-      <x:c r="A92" s="133"/>
-      <x:c r="B92" s="133"/>
-      <x:c r="C92" s="133"/>
-      <x:c r="D92" s="133"/>
-      <x:c r="E92" s="133"/>
-      <x:c r="F92" s="133"/>
-      <x:c r="G92" s="133"/>
-      <x:c r="H92" s="133"/>
-      <x:c r="I92" s="165"/>
-      <x:c r="J92" s="133"/>
-      <x:c r="K92" s="133"/>
-    </x:row>
-    <x:row r="93">
-      <x:c r="A93" s="133"/>
-      <x:c r="B93" s="133"/>
-      <x:c r="C93" s="133"/>
-      <x:c r="D93" s="133"/>
-      <x:c r="E93" s="133"/>
-      <x:c r="F93" s="133"/>
-      <x:c r="G93" s="133"/>
-      <x:c r="H93" s="133"/>
-      <x:c r="I93" s="165"/>
-      <x:c r="J93" s="133"/>
-      <x:c r="K93" s="133"/>
-    </x:row>
-    <x:row r="94">
-      <x:c r="A94" s="133"/>
-      <x:c r="B94" s="133"/>
-      <x:c r="C94" s="133"/>
-      <x:c r="D94" s="133"/>
-      <x:c r="E94" s="133"/>
-      <x:c r="F94" s="133"/>
-      <x:c r="G94" s="133"/>
-      <x:c r="H94" s="133"/>
-      <x:c r="I94" s="165"/>
-      <x:c r="J94" s="133"/>
-      <x:c r="K94" s="133"/>
+    <x:row r="90" ht="84" customHeight="1">
+      <x:c r="A90" s="170" t="str">
+        <x:v>QA-085</x:v>
+      </x:c>
+      <x:c r="B90" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C90" s="170" t="str">
+        <x:v>Operational inventory tenant isolation</x:v>
+      </x:c>
+      <x:c r="D90" s="170" t="str">
+        <x:v>2 prohibited cross-company writes</x:v>
+      </x:c>
+      <x:c r="E90" s="170" t="str">
+        <x:v>Playwright API</x:v>
+      </x:c>
+      <x:c r="F90" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G90" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H90" s="170" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="I90" s="171" t="n">
+        <x:v>46215.95486111111</x:v>
+      </x:c>
+      <x:c r="J90" s="170" t="str">
+        <x:v>HTTP 200/200; expected 404/404</x:v>
+      </x:c>
+      <x:c r="K90" s="170" t="str">
+        <x:v>Current production accepted foreign job/equipment/customer references in two controlled synthetic runs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="84" customHeight="1">
+      <x:c r="A91" s="170" t="str">
+        <x:v>QA-086</x:v>
+      </x:c>
+      <x:c r="B91" s="170" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C91" s="170" t="str">
+        <x:v>Operational inventory tenant-scope route contracts</x:v>
+      </x:c>
+      <x:c r="D91" s="170" t="str">
+        <x:v>Invalid, foreign, and valid references</x:v>
+      </x:c>
+      <x:c r="E91" s="170" t="str">
+        <x:v>Vitest</x:v>
+      </x:c>
+      <x:c r="F91" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G91" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H91" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I91" s="171" t="n">
+        <x:v>46215.95486111111</x:v>
+      </x:c>
+      <x:c r="J91" s="170" t="str">
+        <x:v>6/6 passed</x:v>
+      </x:c>
+      <x:c r="K91" s="170" t="str">
+        <x:v>Both routes reject invalid IDs, reject cross-company references, and preserve valid company-owned inserts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="84" customHeight="1">
+      <x:c r="A92" s="170" t="str">
+        <x:v>QA-087</x:v>
+      </x:c>
+      <x:c r="B92" s="170" t="str">
+        <x:v>Quality</x:v>
+      </x:c>
+      <x:c r="C92" s="170" t="str">
+        <x:v>Full repaired branch validation</x:v>
+      </x:c>
+      <x:c r="D92" s="170" t="str">
+        <x:v>75 unit files + Guardian + incident + build</x:v>
+      </x:c>
+      <x:c r="E92" s="170" t="str">
+        <x:v>Vitest + TypeScript + ESLint + Vite</x:v>
+      </x:c>
+      <x:c r="F92" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G92" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H92" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I92" s="171" t="n">
+        <x:v>46215.95486111111</x:v>
+      </x:c>
+      <x:c r="J92" s="170" t="str">
+        <x:v>775/775; 45/45; 16/16; build passed</x:v>
+      </x:c>
+      <x:c r="K92" s="170" t="str">
+        <x:v>TypeScript and focused lint also passed; production build transformed 5,699 modules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="84" customHeight="1">
+      <x:c r="A93" s="170" t="str">
+        <x:v>QA-088</x:v>
+      </x:c>
+      <x:c r="B93" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C93" s="170" t="str">
+        <x:v>Tenant-isolation discovery teardown</x:v>
+      </x:c>
+      <x:c r="D93" s="170" t="str">
+        <x:v>2 runs × 5 synthetic accounts</x:v>
+      </x:c>
+      <x:c r="E93" s="170" t="str">
+        <x:v>Better Auth + API</x:v>
+      </x:c>
+      <x:c r="F93" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G93" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H93" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I93" s="171" t="n">
+        <x:v>46215.95486111111</x:v>
+      </x:c>
+      <x:c r="J93" s="170" t="str">
+        <x:v>Each run: 5/5 deleted, sessions cleared, logins rejected</x:v>
+      </x:c>
+      <x:c r="K93" s="170" t="str">
+        <x:v>Explicit job-equipment usage was deleted and the synthetic company cascade removed the controlled chemical record.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="84" customHeight="1">
+      <x:c r="A94" s="170" t="str">
+        <x:v>QA-089</x:v>
+      </x:c>
+      <x:c r="B94" s="170" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C94" s="170" t="str">
+        <x:v>Exact tenant-boundary PR gate</x:v>
+      </x:c>
+      <x:c r="D94" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="E94" s="170" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F94" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G94" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H94" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I94" s="171" t="n">
+        <x:v>46215.95486111111</x:v>
+      </x:c>
+      <x:c r="J94" s="170" t="str">
+        <x:v>Run 29212212813: zero steps</x:v>
+      </x:c>
+      <x:c r="K94" s="170" t="str">
+        <x:v>Verified payment/spending refusal; no product or QA command started.</x:v>
+      </x:c>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="133"/>
@@ -13533,7 +13783,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5d9ecc38d9a4688"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc512b8c00e0440cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14274,6 +14524,44 @@
       </x:c>
       <x:c r="L21" s="174" t="str">
         <x:v>Production certification pending deploy and 81/81 rerun.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="132" customHeight="1">
+      <x:c r="A22" s="174" t="str">
+        <x:v>G-016</x:v>
+      </x:c>
+      <x:c r="B22" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="C22" s="174" t="str">
+        <x:v>Tenant Integrity / Security</x:v>
+      </x:c>
+      <x:c r="D22" s="174" t="str">
+        <x:v>Current production accepts another company’s job, equipment, customer, or technician IDs when creating job-equipment usage and chemical application logs.</x:v>
+      </x:c>
+      <x:c r="E22" s="174" t="str">
+        <x:v>A caller can corrupt operational and compliance history and may surface foreign joined names through otherwise company-scoped reads.</x:v>
+      </x:c>
+      <x:c r="F22" s="174" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G22" s="174" t="str">
+        <x:v>Deploy cad0544, require exact production 404/404 proof, and run a read-only mismatch count before considering any historical cleanup.</x:v>
+      </x:c>
+      <x:c r="H22" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I22" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="J22" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K22" s="174" t="str">
+        <x:v>Production returned 200/200; branch focused tenant tests pass 6/6 and the full 775-test gate passes.</x:v>
+      </x:c>
+      <x:c r="L22" s="174" t="str">
+        <x:v>Both discovery runs completed 5/5 synthetic-account cleanup. The repair remains red until the deployed candidate proves both prohibited writes are rejected.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14310,7 +14598,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R680f6b7dc1ee47e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bccadb115b6483d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record database tenant guardrails
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re95865165f6842f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R061ac27910204b67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Re308fae81fbf4c22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R026ec276fc8441c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R07f421a5550f457e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R45979e7234d94ce3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R1a226ac2cb334581"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R57630a2693284c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Rcd150dcf4579474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rf5c8c7788a3e40d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -310,7 +310,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="175">
+  <x:cellXfs count="177">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -698,6 +698,12 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1312,7 +1318,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskTrackerTable" displayName="TaskTrackerTable" ref="A5:Q21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskTrackerTable" displayName="TaskTrackerTable" ref="A5:Q22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Task ID"/>
     <x:tableColumn id="2" name="Phase"/>
@@ -1337,7 +1343,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N109" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1359,7 +1365,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K94" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K99" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1378,7 +1384,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Gap ID"/>
     <x:tableColumn id="2" name="Found During Task"/>
@@ -1693,7 +1699,7 @@
     <x:row r="5">
       <x:c r="A5" s="134" t="n">
         <x:f>COUNTA('Task Tracker'!$A$6:$A$200)</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B5" s="135"/>
       <x:c r="C5" s="136" t="n">
@@ -1761,22 +1767,22 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>89</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>61</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Failed")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F9" s="141"/>
       <x:c r="G9" s="138" t="n">
         <x:f>COUNTIFS('Product Gaps'!$A$6:$A$200,"&lt;&gt;",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Closed",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Resolved",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Mitigated")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H9" s="139"/>
     </x:row>
@@ -1930,30 +1936,30 @@
         <x:v>Product failures and infrastructure failures stay separate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="148" customHeight="1">
+    <x:row r="17" ht="154" customHeight="1">
       <x:c r="A17" s="120" t="str">
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Live owner APIs pass 31/32 and safe lifecycles pass, but current production accepts both tested cross-company operational writes (200/200).</x:v>
+        <x:v>Live APIs remain 31/32; operational isolation is 200/200; read-only audit found 3 historical non-QA chemical product/company mismatches in one pair.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ cad0544; Browser-Base-QA @ 343a154 shared with yawbtng; complete 522-line PRD synchronized.</x:v>
+        <x:v>PestFlow PR #89 @ e4ea0a4; Browser-Base-QA @ 4b7351b shared with yawbtng; complete 546-line PRD synchronized.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Activation</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>Restore Actions; deploy cad0544; prove exact-SHA 32/32 APIs, 81/81 routes, and operational tenant isolation 404/404.</x:v>
+        <x:v>Restore Actions; deploy e4ea0a4; prove six schema constraints, exact-SHA 32/32 APIs, 81/81 routes, and operational 404/404.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>Draft PR mergeable/unstable; run 29212212813 was zero-step billing blocked, while full local branch gates passed.</x:v>
+        <x:v>No production record changed. T-017 requires authorized review before historical repair; run 29214102599 was zero-step billing blocked.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2614,11 +2620,11 @@
         <x:v>/private/tmp/pestflow-desktop-qa-guardian/qa/guardian/desktop-journeys.json</x:v>
       </x:c>
       <x:c r="N8" s="113" t="str">
-        <x:v>cad0544 + Browser-Base-QA 343a154; PR #89</x:v>
+        <x:v>e4ea0a4 + Browser-Base-QA 4b7351b; PR #89</x:v>
       </x:c>
       <x:c r="O8" s="113"/>
       <x:c r="P8" s="113" t="str">
-        <x:v>The standalone executor, 32 API contracts, tenant-boundary evidence, and complete 522-line PRD are synchronized.</x:v>
+        <x:v>Database guardrails, audit policy, schema oracle, and complete 546-line PRD are synchronized.</x:v>
       </x:c>
       <x:c r="Q8" s="163" t="n">
         <x:v>46215.27099571759</x:v>
@@ -2815,19 +2821,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M12" s="166" t="str">
-        <x:v>31/32 live APIs; resource + communications pass; operational tenant isolation fails 200/200</x:v>
+        <x:v>31/32 live APIs; operational writes fail isolation 200/200; historical audit finds 3 product mismatches</x:v>
       </x:c>
       <x:c r="N12" s="166" t="str">
-        <x:v>cad0544; PR #89</x:v>
+        <x:v>e4ea0a4; PR #89</x:v>
       </x:c>
       <x:c r="O12" s="166" t="str">
-        <x:v>Requires reviewed deploy, 404/404 production rerun, and restored GitHub Actions capacity.</x:v>
+        <x:v>Requires reviewed deploy, six-constraint schema proof, production 404/404, and restored Actions capacity.</x:v>
       </x:c>
       <x:c r="P12" s="166" t="str">
-        <x:v>Current production is not certified: cross-company operational references are accepted. Branch repair and full local gates pass.</x:v>
+        <x:v>Branch prevention is route plus database; current production remains uncertified and the three historical records remain unchanged.</x:v>
       </x:c>
       <x:c r="Q12" s="167" t="n">
-        <x:v>46215.95486111111</x:v>
+        <x:v>46215.99652777778</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2922,11 +2928,11 @@
         <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/pull/89</x:v>
       </x:c>
       <x:c r="N14" s="166" t="str">
-        <x:v>cad0544; PR #89</x:v>
+        <x:v>e4ea0a4; PR #89</x:v>
       </x:c>
       <x:c r="O14" s="166"/>
       <x:c r="P14" s="166" t="str">
-        <x:v>Latest production tenant test failed 200/200 with complete cleanup; exact-head cloud run 29212212813 was zero-step billing blocked.</x:v>
+        <x:v>Full branch gate passed; exact-head cloud run 29214102599 was zero-step billing blocked; production mismatch evidence remains red.</x:v>
       </x:c>
       <x:c r="Q14" s="167" t="n">
         <x:v>46215.913194444445</x:v>
@@ -3021,7 +3027,7 @@
         <x:v>Risk-selected + full production</x:v>
       </x:c>
       <x:c r="M16" s="166" t="str">
-        <x:v>Browser-Base-QA @ 343a154; PR #89 @ cad0544</x:v>
+        <x:v>Browser-Base-QA @ 4b7351b; PR #89 @ e4ea0a4</x:v>
       </x:c>
       <x:c r="N16" s="166" t="str">
         <x:v>Standalone API executor and complete PRD are current; promotion wiring remains pending.</x:v>
@@ -3030,7 +3036,7 @@
         <x:v>Needs Browserbase secrets/context, deploy ownership, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P16" s="166" t="str">
-        <x:v>Deploy reviewed head, then require 32/32 APIs, 81/81 routes, and operational isolation 404/404 on the exact SHA.</x:v>
+        <x:v>Deploy reviewed head, require six schema constraints, then 32/32 APIs, 81/81 routes, and operational 404/404 on the exact SHA.</x:v>
       </x:c>
       <x:c r="Q16" s="167" t="n">
         <x:v>46215.27099571759</x:v>
@@ -3282,39 +3288,73 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M21" s="170" t="str">
-        <x:v>31/32 production APIs; safe lifecycles pass; G-013–G-016; PR #89 @ cad0544</x:v>
+        <x:v>31/32 production APIs; G-013–G-016; DB guardrails ready; PR #89 @ e4ea0a4</x:v>
       </x:c>
       <x:c r="N21" s="170" t="str">
-        <x:v>cad0544; PR #89</x:v>
+        <x:v>e4ea0a4; PR #89</x:v>
       </x:c>
       <x:c r="O21" s="170" t="str">
-        <x:v>Needs merge/deploy authority, deployed commit identity, production 404/404, and restored Actions capacity.</x:v>
+        <x:v>Needs merge/deploy authority, exact schema identity, production 404/404, and restored Actions capacity.</x:v>
       </x:c>
       <x:c r="P21" s="170" t="str">
-        <x:v>Branch proof includes 775 unit tests and the operational tenant repair; current production remains uncertified.</x:v>
+        <x:v>Full branch proof is green; current production and historical mismatch inventory are deliberately not called fixed.</x:v>
       </x:c>
       <x:c r="Q21" s="171" t="n">
-        <x:v>46215.95486111111</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="133"/>
-      <x:c r="B22" s="133"/>
-      <x:c r="C22" s="133"/>
-      <x:c r="D22" s="133"/>
-      <x:c r="E22" s="133"/>
-      <x:c r="F22" s="133"/>
-      <x:c r="G22" s="133"/>
-      <x:c r="H22" s="133"/>
-      <x:c r="I22" s="133"/>
-      <x:c r="J22" s="133"/>
-      <x:c r="K22" s="133"/>
-      <x:c r="L22" s="133"/>
-      <x:c r="M22" s="133"/>
-      <x:c r="N22" s="133"/>
-      <x:c r="O22" s="133"/>
-      <x:c r="P22" s="133"/>
-      <x:c r="Q22" s="165"/>
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="138" customHeight="1">
+      <x:c r="A22" s="170" t="str">
+        <x:v>T-017</x:v>
+      </x:c>
+      <x:c r="B22" s="170" t="str">
+        <x:v>Data Integrity</x:v>
+      </x:c>
+      <x:c r="C22" s="170" t="str">
+        <x:v>Review and repair historical chemical-log product ownership mismatches</x:v>
+      </x:c>
+      <x:c r="D22" s="170" t="str">
+        <x:v>The three affected records are reviewed with authorized business context, only approved product mappings are repaired transactionally, the aggregate mismatch count reaches zero, and the composite constraint is validated.</x:v>
+      </x:c>
+      <x:c r="E22" s="170" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="F22" s="170" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G22" s="170" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="H22" s="170" t="str">
+        <x:v>Start with the aggregate audit; obtain record-review and repair authority; preview exact mappings and rollback plan; execute only approved changes; rerun audit; validate constraint.</x:v>
+      </x:c>
+      <x:c r="I22" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="J22" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="K22" s="170" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="L22" s="170" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="M22" s="170" t="str">
+        <x:v>94 chemical logs; 3 mismatches; 1 different-owner company pair; 2026-05-27 timestamp</x:v>
+      </x:c>
+      <x:c r="N22" s="170" t="str">
+        <x:v>e4ea0a4; G-017</x:v>
+      </x:c>
+      <x:c r="O22" s="170" t="str">
+        <x:v>Requires authorized business-record review and explicit production repair approval.</x:v>
+      </x:c>
+      <x:c r="P22" s="170" t="str">
+        <x:v>The prevention fix is ready, but the correct historical product mapping cannot be safely inferred from aggregate data.</x:v>
+      </x:c>
+      <x:c r="Q22" s="171" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="133"/>
@@ -5248,7 +5288,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1272a6b6a18e4ad2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dae778f71414c9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9753,33 +9793,225 @@
         <x:v>PR remains mergeable/unstable. The red check is infrastructure evidence and did not execute product tests.</x:v>
       </x:c>
     </x:row>
-    <x:row r="105">
-      <x:c r="A105" s="133"/>
-      <x:c r="B105" s="165"/>
-      <x:c r="C105" s="133"/>
-      <x:c r="D105" s="133"/>
-      <x:c r="E105" s="133"/>
-      <x:c r="F105" s="133"/>
-      <x:c r="G105" s="133"/>
-      <x:c r="H105" s="133"/>
-      <x:c r="I105" s="133"/>
-      <x:c r="J105" s="133"/>
-      <x:c r="K105" s="133"/>
-      <x:c r="L105" s="133"/>
-      <x:c r="M105" s="133"/>
-      <x:c r="N105" s="133"/>
-    </x:row>
-    <x:row r="106">
-      <x:c r="B106" s="164"/>
-    </x:row>
-    <x:row r="107">
-      <x:c r="B107" s="164"/>
-    </x:row>
-    <x:row r="108">
-      <x:c r="B108" s="164"/>
-    </x:row>
-    <x:row r="109">
-      <x:c r="B109" s="164"/>
+    <x:row r="105" ht="128" customHeight="1">
+      <x:c r="A105" s="170" t="str">
+        <x:v>AL-100</x:v>
+      </x:c>
+      <x:c r="B105" s="171" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+      <x:c r="C105" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D105" s="170" t="str">
+        <x:v>Inventory historical operational tenant relationships</x:v>
+      </x:c>
+      <x:c r="E105" s="170" t="str">
+        <x:v>Built and ran an acknowledged aggregate-only audit inside a database-enforced read-only production transaction.</x:v>
+      </x:c>
+      <x:c r="F105" s="170" t="str">
+        <x:v>Railway SSH + Postgres</x:v>
+      </x:c>
+      <x:c r="G105" s="170" t="str">
+        <x:v>Historical integrity signal quantified without row content</x:v>
+      </x:c>
+      <x:c r="H105" s="170" t="str">
+        <x:v>Chemical logs: 94 total, 3 product/company mismatches, 0 customer/technician/job mismatches, 2 legacy rows without product IDs. Job equipment: 1 total, 0 mismatches.</x:v>
+      </x:c>
+      <x:c r="I105" s="170" t="str">
+        <x:v>Production database</x:v>
+      </x:c>
+      <x:c r="J105" s="170" t="str">
+        <x:v>scripts/qa-operational-tenant-integrity.ts</x:v>
+      </x:c>
+      <x:c r="K105" s="170" t="str">
+        <x:v>G-016; G-017; e4ea0a4</x:v>
+      </x:c>
+      <x:c r="L105" s="170" t="str">
+        <x:v>Classify the three rows without exposing content and prevent recurrence below the API layer.</x:v>
+      </x:c>
+      <x:c r="M105" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N105" s="170" t="str">
+        <x:v>The report returned counts/timestamps only and changed no data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="128" customHeight="1">
+      <x:c r="A106" s="174" t="str">
+        <x:v>AL-101</x:v>
+      </x:c>
+      <x:c r="B106" s="176" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+      <x:c r="C106" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D106" s="174" t="str">
+        <x:v>Classify historical chemical-log mismatches</x:v>
+      </x:c>
+      <x:c r="E106" s="174" t="str">
+        <x:v>Narrowed the three mismatches using aggregate QA/non-QA, ownership, company-name, replacement-product, pair-count, and time-window buckets.</x:v>
+      </x:c>
+      <x:c r="F106" s="174" t="str">
+        <x:v>Read-only production SQL</x:v>
+      </x:c>
+      <x:c r="G106" s="174" t="str">
+        <x:v>One non-QA company pair isolated</x:v>
+      </x:c>
+      <x:c r="H106" s="174" t="str">
+        <x:v>All three involve different owners and different company names, share one pair and the same 2026-05-27 timestamp, and have no same-name product in the log-owning company.</x:v>
+      </x:c>
+      <x:c r="I106" s="174" t="str">
+        <x:v>Production database</x:v>
+      </x:c>
+      <x:c r="J106" s="174" t="str">
+        <x:v>Aggregate-only output</x:v>
+      </x:c>
+      <x:c r="K106" s="174" t="str">
+        <x:v>G-017</x:v>
+      </x:c>
+      <x:c r="L106" s="174" t="str">
+        <x:v>Require business-record review before any repair; do not infer the correct product automatically.</x:v>
+      </x:c>
+      <x:c r="M106" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N106" s="174" t="str">
+        <x:v>A single historical batch/import is plausible but not proven. No IDs, names, emails, product names, or notes were returned.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="128" customHeight="1">
+      <x:c r="A107" s="174" t="str">
+        <x:v>AL-102</x:v>
+      </x:c>
+      <x:c r="B107" s="176" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+      <x:c r="C107" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="D107" s="174" t="str">
+        <x:v>Add database tenant guardrails and release oracle</x:v>
+      </x:c>
+      <x:c r="E107" s="174" t="str">
+        <x:v>Added six composite company/reference foreign keys, route-independent read-only audit policy, schema-health evidence, and change-aware core/operations gate selection.</x:v>
+      </x:c>
+      <x:c r="F107" s="174" t="str">
+        <x:v>Postgres migration + Guardian</x:v>
+      </x:c>
+      <x:c r="G107" s="174" t="str">
+        <x:v>Defense-in-depth prevention implemented</x:v>
+      </x:c>
+      <x:c r="H107" s="174" t="str">
+        <x:v>New rows are enforced immediately with NOT VALID constraints while the three historical rows remain preserved. Schema promotion requires all six constraint names.</x:v>
+      </x:c>
+      <x:c r="I107" s="174" t="str">
+        <x:v>Database + release gate</x:v>
+      </x:c>
+      <x:c r="J107" s="174" t="str">
+        <x:v>migrations/a24_operational_tenant_integrity.sql; qa/guardian/outcome-oracles.json</x:v>
+      </x:c>
+      <x:c r="K107" s="174" t="str">
+        <x:v>e4ea0a4; PR #89</x:v>
+      </x:c>
+      <x:c r="L107" s="174" t="str">
+        <x:v>Deploy reviewed branch, prove schema oracle, then rerun API 404/404 and read-only mismatch audit.</x:v>
+      </x:c>
+      <x:c r="M107" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N107" s="174" t="str">
+        <x:v>The migration does not validate, rewrite, or delete historical records.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="128" customHeight="1">
+      <x:c r="A108" s="174" t="str">
+        <x:v>AL-103</x:v>
+      </x:c>
+      <x:c r="B108" s="176" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+      <x:c r="C108" s="174" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D108" s="174" t="str">
+        <x:v>Validate and publish tenant guardrails</x:v>
+      </x:c>
+      <x:c r="E108" s="174" t="str">
+        <x:v>Ran the complete branch gate, pushed PestFlow commit e4ea0a4, and synchronized the expanded 546-line PRD into Browser-Base-QA.</x:v>
+      </x:c>
+      <x:c r="F108" s="174" t="str">
+        <x:v>Local gates + GitHub</x:v>
+      </x:c>
+      <x:c r="G108" s="174" t="str">
+        <x:v>Implementation and canonical documentation published</x:v>
+      </x:c>
+      <x:c r="H108" s="174" t="str">
+        <x:v>775/775 unit, 48/48 Guardian policy, 16/16 incident, TypeScript, focused lint, and 5,699-module build passed. Browser-Base-QA PRD commit 4b7351b is byte-identical.</x:v>
+      </x:c>
+      <x:c r="I108" s="174" t="str">
+        <x:v>Code + documentation</x:v>
+      </x:c>
+      <x:c r="J108" s="174" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA/blob/main/docs/PRD.md</x:v>
+      </x:c>
+      <x:c r="K108" s="174" t="str">
+        <x:v>e4ea0a4; 4b7351b; PR #89</x:v>
+      </x:c>
+      <x:c r="L108" s="174" t="str">
+        <x:v>Record tracker evidence and require exact deployed-schema proof.</x:v>
+      </x:c>
+      <x:c r="M108" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N108" s="174" t="str">
+        <x:v>Nothing was deployed and no production record was changed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="128" customHeight="1">
+      <x:c r="A109" s="174" t="str">
+        <x:v>AL-104</x:v>
+      </x:c>
+      <x:c r="B109" s="176" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+      <x:c r="C109" s="174" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="D109" s="174" t="str">
+        <x:v>Classify exact database-guardrail PR gate</x:v>
+      </x:c>
+      <x:c r="E109" s="174" t="str">
+        <x:v>Inspected the automatic release gate for exact PestFlow head e4ea0a4 and verified whether a validation command executed.</x:v>
+      </x:c>
+      <x:c r="F109" s="174" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="G109" s="174" t="str">
+        <x:v>Cloud gate blocked before execution</x:v>
+      </x:c>
+      <x:c r="H109" s="174" t="str">
+        <x:v>Run 29214102599, job 86706726235 had zero steps and the verified failed-payment or spending-limit annotation.</x:v>
+      </x:c>
+      <x:c r="I109" s="174" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="J109" s="174" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/actions/runs/29214102599</x:v>
+      </x:c>
+      <x:c r="K109" s="174" t="str">
+        <x:v>e4ea0a4; PR #89</x:v>
+      </x:c>
+      <x:c r="L109" s="174" t="str">
+        <x:v>Restore Actions capacity and rerun the exact-head database-integrity selection and schema oracle.</x:v>
+      </x:c>
+      <x:c r="M109" s="174" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="N109" s="174" t="str">
+        <x:v>The PR remains mergeable/unstable; the red check contains no product-test result.</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="B110" s="164"/>
@@ -10079,7 +10311,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceb10aa6f5c24c1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45bd41a850414733"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13327,70 +13559,180 @@
         <x:v>Verified payment/spending refusal; no product or QA command started.</x:v>
       </x:c>
     </x:row>
-    <x:row r="95">
-      <x:c r="A95" s="133"/>
-      <x:c r="B95" s="133"/>
-      <x:c r="C95" s="133"/>
-      <x:c r="D95" s="133"/>
-      <x:c r="E95" s="133"/>
-      <x:c r="F95" s="133"/>
-      <x:c r="G95" s="133"/>
-      <x:c r="H95" s="133"/>
-      <x:c r="I95" s="165"/>
-      <x:c r="J95" s="133"/>
-      <x:c r="K95" s="133"/>
-    </x:row>
-    <x:row r="96">
-      <x:c r="A96" s="133"/>
-      <x:c r="B96" s="133"/>
-      <x:c r="C96" s="133"/>
-      <x:c r="D96" s="133"/>
-      <x:c r="E96" s="133"/>
-      <x:c r="F96" s="133"/>
-      <x:c r="G96" s="133"/>
-      <x:c r="H96" s="133"/>
-      <x:c r="I96" s="165"/>
-      <x:c r="J96" s="133"/>
-      <x:c r="K96" s="133"/>
-    </x:row>
-    <x:row r="97">
-      <x:c r="A97" s="133"/>
-      <x:c r="B97" s="133"/>
-      <x:c r="C97" s="133"/>
-      <x:c r="D97" s="133"/>
-      <x:c r="E97" s="133"/>
-      <x:c r="F97" s="133"/>
-      <x:c r="G97" s="133"/>
-      <x:c r="H97" s="133"/>
-      <x:c r="I97" s="165"/>
-      <x:c r="J97" s="133"/>
-      <x:c r="K97" s="133"/>
-    </x:row>
-    <x:row r="98">
-      <x:c r="A98" s="133"/>
-      <x:c r="B98" s="133"/>
-      <x:c r="C98" s="133"/>
-      <x:c r="D98" s="133"/>
-      <x:c r="E98" s="133"/>
-      <x:c r="F98" s="133"/>
-      <x:c r="G98" s="133"/>
-      <x:c r="H98" s="133"/>
-      <x:c r="I98" s="165"/>
-      <x:c r="J98" s="133"/>
-      <x:c r="K98" s="133"/>
-    </x:row>
-    <x:row r="99">
-      <x:c r="A99" s="133"/>
-      <x:c r="B99" s="133"/>
-      <x:c r="C99" s="133"/>
-      <x:c r="D99" s="133"/>
-      <x:c r="E99" s="133"/>
-      <x:c r="F99" s="133"/>
-      <x:c r="G99" s="133"/>
-      <x:c r="H99" s="133"/>
-      <x:c r="I99" s="165"/>
-      <x:c r="J99" s="133"/>
-      <x:c r="K99" s="133"/>
+    <x:row r="95" ht="88" customHeight="1">
+      <x:c r="A95" s="170" t="str">
+        <x:v>QA-090</x:v>
+      </x:c>
+      <x:c r="B95" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C95" s="170" t="str">
+        <x:v>Historical operational tenant integrity</x:v>
+      </x:c>
+      <x:c r="D95" s="170" t="str">
+        <x:v>94 chemical logs + 1 equipment-use row</x:v>
+      </x:c>
+      <x:c r="E95" s="170" t="str">
+        <x:v>Read-only Postgres</x:v>
+      </x:c>
+      <x:c r="F95" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G95" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H95" s="170" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="I95" s="171" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+      <x:c r="J95" s="170" t="str">
+        <x:v>3 product/company mismatches</x:v>
+      </x:c>
+      <x:c r="K95" s="170" t="str">
+        <x:v>Zero customer, technician, job, and equipment mismatches; the three non-QA rows share one different-owner company pair and timestamp.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="88" customHeight="1">
+      <x:c r="A96" s="170" t="str">
+        <x:v>QA-091</x:v>
+      </x:c>
+      <x:c r="B96" s="170" t="str">
+        <x:v>Safety</x:v>
+      </x:c>
+      <x:c r="C96" s="170" t="str">
+        <x:v>Aggregate-only operational audit policy</x:v>
+      </x:c>
+      <x:c r="D96" s="170" t="str">
+        <x:v>Source + live execution</x:v>
+      </x:c>
+      <x:c r="E96" s="170" t="str">
+        <x:v>Node policy + Postgres</x:v>
+      </x:c>
+      <x:c r="F96" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G96" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H96" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I96" s="171" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+      <x:c r="J96" s="170" t="str">
+        <x:v>readOnly=true; no row content</x:v>
+      </x:c>
+      <x:c r="K96" s="170" t="str">
+        <x:v>Confirmation, READ ONLY transaction, aggregate COUNT policy, and no identifier SELECTs are locked.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="88" customHeight="1">
+      <x:c r="A97" s="170" t="str">
+        <x:v>QA-092</x:v>
+      </x:c>
+      <x:c r="B97" s="170" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C97" s="170" t="str">
+        <x:v>Database tenant guardrails and release oracle</x:v>
+      </x:c>
+      <x:c r="D97" s="170" t="str">
+        <x:v>6 composite foreign keys</x:v>
+      </x:c>
+      <x:c r="E97" s="170" t="str">
+        <x:v>Node policy</x:v>
+      </x:c>
+      <x:c r="F97" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G97" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H97" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I97" s="171" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+      <x:c r="J97" s="170" t="str">
+        <x:v>6/6 constraint contracts + schema oracle</x:v>
+      </x:c>
+      <x:c r="K97" s="170" t="str">
+        <x:v>New writes are enforced while historical rows remain unvalidated and preserved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="88" customHeight="1">
+      <x:c r="A98" s="170" t="str">
+        <x:v>QA-093</x:v>
+      </x:c>
+      <x:c r="B98" s="170" t="str">
+        <x:v>Quality</x:v>
+      </x:c>
+      <x:c r="C98" s="170" t="str">
+        <x:v>Full database-guardrail branch validation</x:v>
+      </x:c>
+      <x:c r="D98" s="170" t="str">
+        <x:v>75 unit files + Guardian + incident + build</x:v>
+      </x:c>
+      <x:c r="E98" s="170" t="str">
+        <x:v>Vitest + Node + TypeScript + ESLint + Vite</x:v>
+      </x:c>
+      <x:c r="F98" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G98" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="H98" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I98" s="171" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+      <x:c r="J98" s="170" t="str">
+        <x:v>775/775; 48/48; 16/16; build passed</x:v>
+      </x:c>
+      <x:c r="K98" s="170" t="str">
+        <x:v>Focused lint and TypeScript passed; build transformed 5,699 modules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="88" customHeight="1">
+      <x:c r="A99" s="170" t="str">
+        <x:v>QA-094</x:v>
+      </x:c>
+      <x:c r="B99" s="170" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C99" s="170" t="str">
+        <x:v>Exact database-guardrail PR gate</x:v>
+      </x:c>
+      <x:c r="D99" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="E99" s="170" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F99" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G99" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H99" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I99" s="171" t="n">
+        <x:v>46215.99652777778</x:v>
+      </x:c>
+      <x:c r="J99" s="170" t="str">
+        <x:v>Run 29214102599: zero steps</x:v>
+      </x:c>
+      <x:c r="K99" s="170" t="str">
+        <x:v>Verified payment/spending refusal; no selector, schema oracle, product test, or QA command started.</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="133"/>
@@ -13783,7 +14125,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc512b8c00e0440cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4696bc467ac54a7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14558,10 +14900,48 @@
         <x:v>Trevor + Codex</x:v>
       </x:c>
       <x:c r="K22" s="174" t="str">
-        <x:v>Production returned 200/200; branch focused tenant tests pass 6/6 and the full 775-test gate passes.</x:v>
+        <x:v>Production 200/200; branch API tests 6/6; database constraints and schema oracle pass policy at e4ea0a4.</x:v>
       </x:c>
       <x:c r="L22" s="174" t="str">
-        <x:v>Both discovery runs completed 5/5 synthetic-account cleanup. The repair remains red until the deployed candidate proves both prohibited writes are rejected.</x:v>
+        <x:v>Prevention is now route plus database. Deployment and exact 404/404/schema proof remain open; historical records are tracked separately under G-017.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="138" customHeight="1">
+      <x:c r="A23" s="174" t="str">
+        <x:v>G-017</x:v>
+      </x:c>
+      <x:c r="B23" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="C23" s="174" t="str">
+        <x:v>Historical Data Integrity</x:v>
+      </x:c>
+      <x:c r="D23" s="174" t="str">
+        <x:v>Three non-QA chemical application logs reference a chemical product owned by one different company pair.</x:v>
+      </x:c>
+      <x:c r="E23" s="174" t="str">
+        <x:v>The affected business’s compliance history may display the wrong product identity, and automatic relinking would risk changing regulated records incorrectly.</x:v>
+      </x:c>
+      <x:c r="F23" s="174" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G23" s="174" t="str">
+        <x:v>Review the three records with the business owner, prepare a transaction-scoped preview, repair only approved mappings, prove mismatch count zero, then validate the database constraint.</x:v>
+      </x:c>
+      <x:c r="H23" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I23" s="174" t="str">
+        <x:v>T-017</x:v>
+      </x:c>
+      <x:c r="J23" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K23" s="174" t="str">
+        <x:v>Read-only production audit: 94 logs, 3 mismatches, one pair, one timestamp, different owners/names, no same-name local replacement.</x:v>
+      </x:c>
+      <x:c r="L23" s="174" t="str">
+        <x:v>No record IDs or content were returned and no repair was attempted. A batch/import origin is plausible but unproven.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14598,7 +14978,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bccadb115b6483d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcf5eb98b1ff46cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record core tenant hardening
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R45979e7234d94ce3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R1a226ac2cb334581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R57630a2693284c40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Rcd150dcf4579474c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rf5c8c7788a3e40d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R02174930613c4161"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R794af85a785e40b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Rb41c2003d41a4d85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Rceff6df857874d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rd54b3069005b460b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1343,7 +1343,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N109" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N114" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1365,7 +1365,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K99" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1384,7 +1384,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Gap ID"/>
     <x:tableColumn id="2" name="Found During Task"/>
@@ -1767,12 +1767,12 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>94</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>64</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
@@ -1782,7 +1782,7 @@
       <x:c r="F9" s="141"/>
       <x:c r="G9" s="138" t="n">
         <x:f>COUNTIFS('Product Gaps'!$A$6:$A$200,"&lt;&gt;",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Closed",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Resolved",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Mitigated")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="H9" s="139"/>
     </x:row>
@@ -1936,30 +1936,30 @@
         <x:v>Product failures and infrastructure failures stay separate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="154" customHeight="1">
+    <x:row r="17" ht="158" customHeight="1">
       <x:c r="A17" s="120" t="str">
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Live APIs remain 31/32; operational isolation is 200/200; read-only audit found 3 historical non-QA chemical product/company mismatches in one pair.</x:v>
+        <x:v>Core production data is 453/453 company-scoped and 29/29 relationship-consistent; operational isolation remains 200/200 and 3 historical chemical mismatches remain.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ e4ea0a4; Browser-Base-QA @ 4b7351b shared with yawbtng; complete 546-line PRD synchronized.</x:v>
+        <x:v>PestFlow PR #89 @ 4c27f8d; Browser-Base-QA @ f33c736 shared with yawbtng; complete 556-line PRD synchronized.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Activation</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>Restore Actions; deploy e4ea0a4; prove six schema constraints, exact-SHA 32/32 APIs, 81/81 routes, and operational 404/404.</x:v>
+        <x:v>Restore Actions; deploy 4c27f8d; prove 17 schema constraints, exact-SHA 32/32 APIs, 81/81 routes, and all core/operational rejection checks.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>No production record changed. T-017 requires authorized review before historical repair; run 29214102599 was zero-step billing blocked.</x:v>
+        <x:v>No production record changed. PR mergeable/unstable; run 29214865469 was zero-step billing blocked.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2620,11 +2620,11 @@
         <x:v>/private/tmp/pestflow-desktop-qa-guardian/qa/guardian/desktop-journeys.json</x:v>
       </x:c>
       <x:c r="N8" s="113" t="str">
-        <x:v>e4ea0a4 + Browser-Base-QA 4b7351b; PR #89</x:v>
+        <x:v>4c27f8d + Browser-Base-QA f33c736; PR #89</x:v>
       </x:c>
       <x:c r="O8" s="113"/>
       <x:c r="P8" s="113" t="str">
-        <x:v>Database guardrails, audit policy, schema oracle, and complete 546-line PRD are synchronized.</x:v>
+        <x:v>Shared validator, 17 constraints, expanded audit, schema oracle, and complete 556-line PRD are synchronized.</x:v>
       </x:c>
       <x:c r="Q8" s="163" t="n">
         <x:v>46215.27099571759</x:v>
@@ -2821,19 +2821,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M12" s="166" t="str">
-        <x:v>31/32 live APIs; operational writes fail isolation 200/200; historical audit finds 3 product mismatches</x:v>
+        <x:v>31/32 live APIs; operational isolation 200/200; core audit 453/453 scoped and 29/29 consistent</x:v>
       </x:c>
       <x:c r="N12" s="166" t="str">
-        <x:v>e4ea0a4; PR #89</x:v>
+        <x:v>4c27f8d; PR #89</x:v>
       </x:c>
       <x:c r="O12" s="166" t="str">
-        <x:v>Requires reviewed deploy, six-constraint schema proof, production 404/404, and restored Actions capacity.</x:v>
+        <x:v>Requires reviewed deploy, 17-constraint schema proof, production rejection matrix, and restored Actions capacity.</x:v>
       </x:c>
       <x:c r="P12" s="166" t="str">
-        <x:v>Branch prevention is route plus database; current production remains uncertified and the three historical records remain unchanged.</x:v>
+        <x:v>Branch now protects six core route families plus operational inventory at route and database layers; current production remains uncertified.</x:v>
       </x:c>
       <x:c r="Q12" s="167" t="n">
-        <x:v>46215.99652777778</x:v>
+        <x:v>46216.010416666664</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2928,11 +2928,11 @@
         <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/pull/89</x:v>
       </x:c>
       <x:c r="N14" s="166" t="str">
-        <x:v>e4ea0a4; PR #89</x:v>
+        <x:v>4c27f8d; PR #89</x:v>
       </x:c>
       <x:c r="O14" s="166"/>
       <x:c r="P14" s="166" t="str">
-        <x:v>Full branch gate passed; exact-head cloud run 29214102599 was zero-step billing blocked; production mismatch evidence remains red.</x:v>
+        <x:v>Full branch gate passed; exact-head cloud run 29214865469 was zero-step billing blocked; no product command ran.</x:v>
       </x:c>
       <x:c r="Q14" s="167" t="n">
         <x:v>46215.913194444445</x:v>
@@ -3027,7 +3027,7 @@
         <x:v>Risk-selected + full production</x:v>
       </x:c>
       <x:c r="M16" s="166" t="str">
-        <x:v>Browser-Base-QA @ 4b7351b; PR #89 @ e4ea0a4</x:v>
+        <x:v>Browser-Base-QA @ f33c736; PR #89 @ 4c27f8d</x:v>
       </x:c>
       <x:c r="N16" s="166" t="str">
         <x:v>Standalone API executor and complete PRD are current; promotion wiring remains pending.</x:v>
@@ -3036,7 +3036,7 @@
         <x:v>Needs Browserbase secrets/context, deploy ownership, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P16" s="166" t="str">
-        <x:v>Deploy reviewed head, require six schema constraints, then 32/32 APIs, 81/81 routes, and operational 404/404 on the exact SHA.</x:v>
+        <x:v>Deploy reviewed head, require 17 schema constraints, then 32/32 APIs, 81/81 routes, and the core/operational rejection matrix on the exact SHA.</x:v>
       </x:c>
       <x:c r="Q16" s="167" t="n">
         <x:v>46215.27099571759</x:v>
@@ -3288,19 +3288,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M21" s="170" t="str">
-        <x:v>31/32 production APIs; G-013–G-016; DB guardrails ready; PR #89 @ e4ea0a4</x:v>
+        <x:v>31/32 production APIs; G-013–G-016 and G-018; 17 DB guardrails ready; PR #89 @ 4c27f8d</x:v>
       </x:c>
       <x:c r="N21" s="170" t="str">
-        <x:v>e4ea0a4; PR #89</x:v>
+        <x:v>4c27f8d; PR #89</x:v>
       </x:c>
       <x:c r="O21" s="170" t="str">
-        <x:v>Needs merge/deploy authority, exact schema identity, production 404/404, and restored Actions capacity.</x:v>
+        <x:v>Needs merge/deploy authority, exact schema identity, production rejection proof, and restored Actions capacity.</x:v>
       </x:c>
       <x:c r="P21" s="170" t="str">
-        <x:v>Full branch proof is green; current production and historical mismatch inventory are deliberately not called fixed.</x:v>
+        <x:v>Full branch proof is green; current production and the three historical chemical mismatches remain deliberately uncertified.</x:v>
       </x:c>
       <x:c r="Q21" s="171" t="n">
-        <x:v>46215.99652777778</x:v>
+        <x:v>46216.010416666664</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="138" customHeight="1">
@@ -3344,13 +3344,13 @@
         <x:v>94 chemical logs; 3 mismatches; 1 different-owner company pair; 2026-05-27 timestamp</x:v>
       </x:c>
       <x:c r="N22" s="170" t="str">
-        <x:v>e4ea0a4; G-017</x:v>
+        <x:v>4c27f8d; G-017</x:v>
       </x:c>
       <x:c r="O22" s="170" t="str">
         <x:v>Requires authorized business-record review and explicit production repair approval.</x:v>
       </x:c>
       <x:c r="P22" s="170" t="str">
-        <x:v>The prevention fix is ready, but the correct historical product mapping cannot be safely inferred from aggregate data.</x:v>
+        <x:v>Core audit is clean; only the three previously identified chemical product/company mappings require historical review.</x:v>
       </x:c>
       <x:c r="Q22" s="171" t="n">
         <x:v>46215.99652777778</x:v>
@@ -5288,7 +5288,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dae778f71414c9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6eb7dfdc55d40e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10013,20 +10013,225 @@
         <x:v>The PR remains mergeable/unstable; the red check contains no product-test result.</x:v>
       </x:c>
     </x:row>
-    <x:row r="110">
-      <x:c r="B110" s="164"/>
-    </x:row>
-    <x:row r="111">
-      <x:c r="B111" s="164"/>
-    </x:row>
-    <x:row r="112">
-      <x:c r="B112" s="164"/>
-    </x:row>
-    <x:row r="113">
-      <x:c r="B113" s="164"/>
-    </x:row>
-    <x:row r="114">
-      <x:c r="B114" s="164"/>
+    <x:row r="110" ht="132" customHeight="1">
+      <x:c r="A110" s="174" t="str">
+        <x:v>AL-105</x:v>
+      </x:c>
+      <x:c r="B110" s="176" t="n">
+        <x:v>46216.010416666664</x:v>
+      </x:c>
+      <x:c r="C110" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D110" s="174" t="str">
+        <x:v>Audit core desktop foreign-record relationships</x:v>
+      </x:c>
+      <x:c r="E110" s="174" t="str">
+        <x:v>Expanded the database-enforced read-only inventory across jobs, invoices, customer notes, service agreements, service documents, and customer contracts.</x:v>
+      </x:c>
+      <x:c r="F110" s="174" t="str">
+        <x:v>Railway SSH + Postgres</x:v>
+      </x:c>
+      <x:c r="G110" s="174" t="str">
+        <x:v>Existing core relationships are company-consistent</x:v>
+      </x:c>
+      <x:c r="H110" s="174" t="str">
+        <x:v>All 453 populated company/reference relationships had zero mismatches. All 29 paired job/customer or invoice/customer relationships were internally consistent.</x:v>
+      </x:c>
+      <x:c r="I110" s="174" t="str">
+        <x:v>Production database</x:v>
+      </x:c>
+      <x:c r="J110" s="174" t="str">
+        <x:v>scripts/qa-operational-tenant-integrity.ts</x:v>
+      </x:c>
+      <x:c r="K110" s="174" t="str">
+        <x:v>4c27f8d; PR #89</x:v>
+      </x:c>
+      <x:c r="L110" s="174" t="str">
+        <x:v>Use the clean baseline to add preventative route and database enforcement without rewriting rows.</x:v>
+      </x:c>
+      <x:c r="M110" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N110" s="174" t="str">
+        <x:v>Read-only aggregate output contained no IDs, names, emails, addresses, product names, or notes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="132" customHeight="1">
+      <x:c r="A111" s="174" t="str">
+        <x:v>AL-106</x:v>
+      </x:c>
+      <x:c r="B111" s="176" t="n">
+        <x:v>46216.010416666664</x:v>
+      </x:c>
+      <x:c r="C111" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D111" s="174" t="str">
+        <x:v>Inventory core write-route ownership gaps</x:v>
+      </x:c>
+      <x:c r="E111" s="174" t="str">
+        <x:v>Traced every persisted customer, location, technician, job, and invoice reference in the core desktop write paths.</x:v>
+      </x:c>
+      <x:c r="F111" s="174" t="str">
+        <x:v>Source and schema audit</x:v>
+      </x:c>
+      <x:c r="G111" s="174" t="str">
+        <x:v>Six additional route families lacked consistent ownership validation</x:v>
+      </x:c>
+      <x:c r="H111" s="174" t="str">
+        <x:v>Jobs, invoices, customer notes, service agreements, service documents, and customer contracts could accept foreign IDs before database insertion; job locations could also mismatch the selected customer.</x:v>
+      </x:c>
+      <x:c r="I111" s="174" t="str">
+        <x:v>Desktop API</x:v>
+      </x:c>
+      <x:c r="J111" s="174" t="str">
+        <x:v>server/routes/*.ts</x:v>
+      </x:c>
+      <x:c r="K111" s="174" t="str">
+        <x:v>G-018</x:v>
+      </x:c>
+      <x:c r="L111" s="174" t="str">
+        <x:v>Centralize validation and enforce the same invariants below the API layer.</x:v>
+      </x:c>
+      <x:c r="M111" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N111" s="174" t="str">
+        <x:v>This finding is source-proven; no uncontrolled production write was used to demonstrate it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="132" customHeight="1">
+      <x:c r="A112" s="174" t="str">
+        <x:v>AL-107</x:v>
+      </x:c>
+      <x:c r="B112" s="176" t="n">
+        <x:v>46216.010416666664</x:v>
+      </x:c>
+      <x:c r="C112" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="D112" s="174" t="str">
+        <x:v>Harden core references at route and database layers</x:v>
+      </x:c>
+      <x:c r="E112" s="174" t="str">
+        <x:v>Added one typed company-reference inspector, wired six route families, expanded the migration from 6 to 17 composite constraints, and made the schema oracle require all 17 names.</x:v>
+      </x:c>
+      <x:c r="F112" s="174" t="str">
+        <x:v>PestFlow API + Postgres + Guardian</x:v>
+      </x:c>
+      <x:c r="G112" s="174" t="str">
+        <x:v>Core tenant prevention implemented</x:v>
+      </x:c>
+      <x:c r="H112" s="174" t="str">
+        <x:v>Malformed/inconsistent references return 400; foreign/missing references return 404 before persistence. NOT VALID constraints enforce every new/changed row while preserving historical evidence.</x:v>
+      </x:c>
+      <x:c r="I112" s="174" t="str">
+        <x:v>Desktop API + database</x:v>
+      </x:c>
+      <x:c r="J112" s="174" t="str">
+        <x:v>server/lib/companyReferences.ts; migrations/a24_operational_tenant_integrity.sql</x:v>
+      </x:c>
+      <x:c r="K112" s="174" t="str">
+        <x:v>4c27f8d; G-018; PR #89</x:v>
+      </x:c>
+      <x:c r="L112" s="174" t="str">
+        <x:v>Deploy reviewed branch and prove exact-SHA schema plus production route rejection.</x:v>
+      </x:c>
+      <x:c r="M112" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N112" s="174" t="str">
+        <x:v>Also removed 15 existing touched-file explicit-any lint violations instead of excluding the files.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="132" customHeight="1">
+      <x:c r="A113" s="174" t="str">
+        <x:v>AL-108</x:v>
+      </x:c>
+      <x:c r="B113" s="176" t="n">
+        <x:v>46216.010416666664</x:v>
+      </x:c>
+      <x:c r="C113" s="174" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D113" s="174" t="str">
+        <x:v>Validate and publish core tenant hardening</x:v>
+      </x:c>
+      <x:c r="E113" s="174" t="str">
+        <x:v>Ran the full branch gate, pushed PestFlow commit 4c27f8d, and synchronized the 556-line PRD into Browser-Base-QA.</x:v>
+      </x:c>
+      <x:c r="F113" s="174" t="str">
+        <x:v>Local gates + GitHub</x:v>
+      </x:c>
+      <x:c r="G113" s="174" t="str">
+        <x:v>Implementation and shared documentation published</x:v>
+      </x:c>
+      <x:c r="H113" s="174" t="str">
+        <x:v>786/786 unit across 77 files, 48/48 Guardian policy, 16/16 incident, TypeScript, touched-file lint, and the 5,699-module build passed. Browser-Base-QA commit f33c736 is byte-identical.</x:v>
+      </x:c>
+      <x:c r="I113" s="174" t="str">
+        <x:v>Code + documentation</x:v>
+      </x:c>
+      <x:c r="J113" s="174" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA/blob/main/docs/PRD.md</x:v>
+      </x:c>
+      <x:c r="K113" s="174" t="str">
+        <x:v>4c27f8d; f33c736; PR #89</x:v>
+      </x:c>
+      <x:c r="L113" s="174" t="str">
+        <x:v>Update tracker evidence and require deployment certification.</x:v>
+      </x:c>
+      <x:c r="M113" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N113" s="174" t="str">
+        <x:v>Current production was only read; no existing relationship changed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="132" customHeight="1">
+      <x:c r="A114" s="174" t="str">
+        <x:v>AL-109</x:v>
+      </x:c>
+      <x:c r="B114" s="176" t="n">
+        <x:v>46216.010416666664</x:v>
+      </x:c>
+      <x:c r="C114" s="174" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="D114" s="174" t="str">
+        <x:v>Classify exact core-hardening PR gate</x:v>
+      </x:c>
+      <x:c r="E114" s="174" t="str">
+        <x:v>Inspected the automatic release gate for exact PestFlow head 4c27f8d and verified whether a command executed.</x:v>
+      </x:c>
+      <x:c r="F114" s="174" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="G114" s="174" t="str">
+        <x:v>Cloud gate blocked before execution</x:v>
+      </x:c>
+      <x:c r="H114" s="174" t="str">
+        <x:v>Run 29214865469, job 86708695743 had zero steps and the verified failed-payment or spending-limit annotation.</x:v>
+      </x:c>
+      <x:c r="I114" s="174" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="J114" s="174" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/actions/runs/29214865469</x:v>
+      </x:c>
+      <x:c r="K114" s="174" t="str">
+        <x:v>4c27f8d; PR #89</x:v>
+      </x:c>
+      <x:c r="L114" s="174" t="str">
+        <x:v>Restore Actions capacity and rerun exact-head selection, schema oracle, deterministic, and browser gates.</x:v>
+      </x:c>
+      <x:c r="M114" s="174" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="N114" s="174" t="str">
+        <x:v>PR remains mergeable/unstable. The red check contains no product-test verdict.</x:v>
+      </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="B115" s="164"/>
@@ -10311,7 +10516,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45bd41a850414733"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ecb165b1d894e37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13734,70 +13939,180 @@
         <x:v>Verified payment/spending refusal; no selector, schema oracle, product test, or QA command started.</x:v>
       </x:c>
     </x:row>
-    <x:row r="100">
-      <x:c r="A100" s="133"/>
-      <x:c r="B100" s="133"/>
-      <x:c r="C100" s="133"/>
-      <x:c r="D100" s="133"/>
-      <x:c r="E100" s="133"/>
-      <x:c r="F100" s="133"/>
-      <x:c r="G100" s="133"/>
-      <x:c r="H100" s="133"/>
-      <x:c r="I100" s="165"/>
-      <x:c r="J100" s="133"/>
-      <x:c r="K100" s="133"/>
-    </x:row>
-    <x:row r="101">
-      <x:c r="A101" s="133"/>
-      <x:c r="B101" s="133"/>
-      <x:c r="C101" s="133"/>
-      <x:c r="D101" s="133"/>
-      <x:c r="E101" s="133"/>
-      <x:c r="F101" s="133"/>
-      <x:c r="G101" s="133"/>
-      <x:c r="H101" s="133"/>
-      <x:c r="I101" s="165"/>
-      <x:c r="J101" s="133"/>
-      <x:c r="K101" s="133"/>
-    </x:row>
-    <x:row r="102">
-      <x:c r="A102" s="133"/>
-      <x:c r="B102" s="133"/>
-      <x:c r="C102" s="133"/>
-      <x:c r="D102" s="133"/>
-      <x:c r="E102" s="133"/>
-      <x:c r="F102" s="133"/>
-      <x:c r="G102" s="133"/>
-      <x:c r="H102" s="133"/>
-      <x:c r="I102" s="165"/>
-      <x:c r="J102" s="133"/>
-      <x:c r="K102" s="133"/>
-    </x:row>
-    <x:row r="103">
-      <x:c r="A103" s="133"/>
-      <x:c r="B103" s="133"/>
-      <x:c r="C103" s="133"/>
-      <x:c r="D103" s="133"/>
-      <x:c r="E103" s="133"/>
-      <x:c r="F103" s="133"/>
-      <x:c r="G103" s="133"/>
-      <x:c r="H103" s="133"/>
-      <x:c r="I103" s="165"/>
-      <x:c r="J103" s="133"/>
-      <x:c r="K103" s="133"/>
-    </x:row>
-    <x:row r="104">
-      <x:c r="A104" s="133"/>
-      <x:c r="B104" s="133"/>
-      <x:c r="C104" s="133"/>
-      <x:c r="D104" s="133"/>
-      <x:c r="E104" s="133"/>
-      <x:c r="F104" s="133"/>
-      <x:c r="G104" s="133"/>
-      <x:c r="H104" s="133"/>
-      <x:c r="I104" s="165"/>
-      <x:c r="J104" s="133"/>
-      <x:c r="K104" s="133"/>
+    <x:row r="100" ht="90" customHeight="1">
+      <x:c r="A100" s="170" t="str">
+        <x:v>QA-095</x:v>
+      </x:c>
+      <x:c r="B100" s="170" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C100" s="170" t="str">
+        <x:v>Core desktop company-reference integrity</x:v>
+      </x:c>
+      <x:c r="D100" s="170" t="str">
+        <x:v>453 populated references + 29 paired relationships</x:v>
+      </x:c>
+      <x:c r="E100" s="170" t="str">
+        <x:v>Read-only Postgres</x:v>
+      </x:c>
+      <x:c r="F100" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G100" s="170" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H100" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I100" s="171" t="n">
+        <x:v>46216.010416666664</x:v>
+      </x:c>
+      <x:c r="J100" s="170" t="str">
+        <x:v>453/453 scoped; 29/29 consistent</x:v>
+      </x:c>
+      <x:c r="K100" s="170" t="str">
+        <x:v>Jobs, invoices, notes, agreements, documents, and contracts contained zero company or parent/customer mismatches.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="90" customHeight="1">
+      <x:c r="A101" s="170" t="str">
+        <x:v>QA-096</x:v>
+      </x:c>
+      <x:c r="B101" s="170" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C101" s="170" t="str">
+        <x:v>Shared and route-level company-reference rejection</x:v>
+      </x:c>
+      <x:c r="D101" s="170" t="str">
+        <x:v>3 focused test files</x:v>
+      </x:c>
+      <x:c r="E101" s="170" t="str">
+        <x:v>Vitest</x:v>
+      </x:c>
+      <x:c r="F101" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G101" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H101" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I101" s="171" t="n">
+        <x:v>46216.010416666664</x:v>
+      </x:c>
+      <x:c r="J101" s="170" t="str">
+        <x:v>17/17 passed</x:v>
+      </x:c>
+      <x:c r="K101" s="170" t="str">
+        <x:v>Validator, six core routes, and original operational inventory routes reject malformed, foreign, and inconsistent references.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="90" customHeight="1">
+      <x:c r="A102" s="170" t="str">
+        <x:v>QA-097</x:v>
+      </x:c>
+      <x:c r="B102" s="170" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C102" s="170" t="str">
+        <x:v>Database tenant constraint release contract</x:v>
+      </x:c>
+      <x:c r="D102" s="170" t="str">
+        <x:v>17 composite foreign keys</x:v>
+      </x:c>
+      <x:c r="E102" s="170" t="str">
+        <x:v>Node policy</x:v>
+      </x:c>
+      <x:c r="F102" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G102" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H102" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I102" s="171" t="n">
+        <x:v>46216.010416666664</x:v>
+      </x:c>
+      <x:c r="J102" s="170" t="str">
+        <x:v>17/17 names required</x:v>
+      </x:c>
+      <x:c r="K102" s="170" t="str">
+        <x:v>Schema health and the release oracle fail closed if any core/operational constraint is absent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="90" customHeight="1">
+      <x:c r="A103" s="170" t="str">
+        <x:v>QA-098</x:v>
+      </x:c>
+      <x:c r="B103" s="170" t="str">
+        <x:v>Quality</x:v>
+      </x:c>
+      <x:c r="C103" s="170" t="str">
+        <x:v>Full core-hardening branch validation</x:v>
+      </x:c>
+      <x:c r="D103" s="170" t="str">
+        <x:v>77 unit files + Guardian + incident + build</x:v>
+      </x:c>
+      <x:c r="E103" s="170" t="str">
+        <x:v>Vitest + Node + TypeScript + ESLint + Vite</x:v>
+      </x:c>
+      <x:c r="F103" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G103" s="170" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="H103" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I103" s="171" t="n">
+        <x:v>46216.010416666664</x:v>
+      </x:c>
+      <x:c r="J103" s="170" t="str">
+        <x:v>786/786; 48/48; 16/16; build passed</x:v>
+      </x:c>
+      <x:c r="K103" s="170" t="str">
+        <x:v>Touched-file lint is clean and production build transformed 5,699 modules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="90" customHeight="1">
+      <x:c r="A104" s="170" t="str">
+        <x:v>QA-099</x:v>
+      </x:c>
+      <x:c r="B104" s="170" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C104" s="170" t="str">
+        <x:v>Exact core-hardening PR gate</x:v>
+      </x:c>
+      <x:c r="D104" s="170" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="E104" s="170" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F104" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G104" s="170" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H104" s="170" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I104" s="171" t="n">
+        <x:v>46216.010416666664</x:v>
+      </x:c>
+      <x:c r="J104" s="170" t="str">
+        <x:v>Run 29214865469: zero steps</x:v>
+      </x:c>
+      <x:c r="K104" s="170" t="str">
+        <x:v>Verified payment/spending refusal; no selector, schema oracle, product test, or browser command started.</x:v>
+      </x:c>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="133"/>
@@ -14125,7 +14440,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4696bc467ac54a7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03939a43477d40be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14942,6 +15257,44 @@
       </x:c>
       <x:c r="L23" s="174" t="str">
         <x:v>No record IDs or content were returned and no repair was attempted. A batch/import origin is plausible but unproven.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="142" customHeight="1">
+      <x:c r="A24" s="174" t="str">
+        <x:v>G-018</x:v>
+      </x:c>
+      <x:c r="B24" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="C24" s="174" t="str">
+        <x:v>Core Tenant Integrity</x:v>
+      </x:c>
+      <x:c r="D24" s="174" t="str">
+        <x:v>Core job, invoice, note, agreement, document, and customer-contract write paths did not consistently prove that supplied foreign-record IDs belonged to the authenticated company.</x:v>
+      </x:c>
+      <x:c r="E24" s="174" t="str">
+        <x:v>A crafted or stale request could corrupt customer operations, scheduling, billing, notes, agreements, or documents with another company’s record linkage.</x:v>
+      </x:c>
+      <x:c r="F24" s="174" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G24" s="174" t="str">
+        <x:v>Deploy 4c27f8d, prove all 17 schema constraints on the exact SHA, and run controlled synthetic rejection checks for each route family before certification.</x:v>
+      </x:c>
+      <x:c r="H24" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I24" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="J24" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K24" s="174" t="str">
+        <x:v>Source audit plus 17/17 focused tests; production read-only inventory found 453/453 existing core references correctly scoped.</x:v>
+      </x:c>
+      <x:c r="L24" s="174" t="str">
+        <x:v>Branch prevention is ready at route and database layers. Current production was not mutated to demonstrate each source-proven gap.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14978,7 +15331,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcf5eb98b1ff46cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R782e7b3b64744ee6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record provider field hardening
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R02174930613c4161"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R794af85a785e40b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Rb41c2003d41a4d85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Rceff6df857874d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rd54b3069005b460b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2a2f4333fbdf429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R24aeedbf59d640e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Rc95e2add13464b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R5f700a3ed6d54f82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R36372977c6af4187"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1343,7 +1343,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N114" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1365,7 +1365,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K109" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1384,7 +1384,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Gap ID"/>
     <x:tableColumn id="2" name="Found During Task"/>
@@ -1767,12 +1767,12 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>99</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>68</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
@@ -1782,7 +1782,7 @@
       <x:c r="F9" s="141"/>
       <x:c r="G9" s="138" t="n">
         <x:f>COUNTIFS('Product Gaps'!$A$6:$A$200,"&lt;&gt;",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Closed",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Resolved",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Mitigated")</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H9" s="139"/>
     </x:row>
@@ -1936,30 +1936,30 @@
         <x:v>Product failures and infrastructure failures stay separate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="158" customHeight="1">
+    <x:row r="17" ht="162" customHeight="1">
       <x:c r="A17" s="120" t="str">
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Core production data is 453/453 company-scoped and 29/29 relationship-consistent; operational isolation remains 200/200 and 3 historical chemical mismatches remain.</x:v>
+        <x:v>Core production data is 453/453 scoped; provider/field data is 536/536 scoped and 259/259 paired-consistent. Operational isolation remains 200/200 until deployment.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ 4c27f8d; Browser-Base-QA @ f33c736 shared with yawbtng; complete 556-line PRD synchronized.</x:v>
+        <x:v>PestFlow PR #89 @ a9c9e66; Browser-Base-QA @ 8eff452 shared with yawbtng; PRD and full implementation guide synchronized.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Activation</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>Restore Actions; deploy 4c27f8d; prove 17 schema constraints, exact-SHA 32/32 APIs, 81/81 routes, and all core/operational rejection checks.</x:v>
+        <x:v>Restore Actions; deploy a9c9e66; prove 26 schema constraints, exact-SHA 32/32 APIs, 81/81 routes, and the complete tenant rejection matrix.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>No production record changed. PR mergeable/unstable; run 29214865469 was zero-step billing blocked.</x:v>
+        <x:v>No production row or provider was changed. PR mergeable/unstable; run 29215702743 was zero-step billing blocked.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2620,11 +2620,11 @@
         <x:v>/private/tmp/pestflow-desktop-qa-guardian/qa/guardian/desktop-journeys.json</x:v>
       </x:c>
       <x:c r="N8" s="113" t="str">
-        <x:v>4c27f8d + Browser-Base-QA f33c736; PR #89</x:v>
+        <x:v>a9c9e66 + Browser-Base-QA 8eff452; PR #89</x:v>
       </x:c>
       <x:c r="O8" s="113"/>
       <x:c r="P8" s="113" t="str">
-        <x:v>Shared validator, 17 constraints, expanded audit, schema oracle, and complete 556-line PRD are synchronized.</x:v>
+        <x:v>Shared validator, 26 constraints, expanded audit, schema oracle, 571-line PRD, and 581-line implementation guide are synchronized.</x:v>
       </x:c>
       <x:c r="Q8" s="163" t="n">
         <x:v>46215.27099571759</x:v>
@@ -2821,19 +2821,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M12" s="166" t="str">
-        <x:v>31/32 live APIs; operational isolation 200/200; core audit 453/453 scoped and 29/29 consistent</x:v>
+        <x:v>Core 453/453 + provider/field 536/536 references scoped; 29/29 + 259/259 paired relationships consistent</x:v>
       </x:c>
       <x:c r="N12" s="166" t="str">
-        <x:v>4c27f8d; PR #89</x:v>
+        <x:v>a9c9e66; PR #89</x:v>
       </x:c>
       <x:c r="O12" s="166" t="str">
-        <x:v>Requires reviewed deploy, 17-constraint schema proof, production rejection matrix, and restored Actions capacity.</x:v>
+        <x:v>Requires reviewed deploy, 26-constraint schema proof, production rejection matrix, and restored Actions capacity.</x:v>
       </x:c>
       <x:c r="P12" s="166" t="str">
-        <x:v>Branch now protects six core route families plus operational inventory at route and database layers; current production remains uncertified.</x:v>
+        <x:v>Branch now protects core, operational, provider, and field references at route and database layers; current production remains uncertified.</x:v>
       </x:c>
       <x:c r="Q12" s="167" t="n">
-        <x:v>46216.010416666664</x:v>
+        <x:v>46216.02777777778</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2928,11 +2928,11 @@
         <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/pull/89</x:v>
       </x:c>
       <x:c r="N14" s="166" t="str">
-        <x:v>4c27f8d; PR #89</x:v>
+        <x:v>a9c9e66; PR #89</x:v>
       </x:c>
       <x:c r="O14" s="166"/>
       <x:c r="P14" s="166" t="str">
-        <x:v>Full branch gate passed; exact-head cloud run 29214865469 was zero-step billing blocked; no product command ran.</x:v>
+        <x:v>Full branch gate passed; exact-head cloud run 29215702743 was zero-step billing blocked; no product command ran.</x:v>
       </x:c>
       <x:c r="Q14" s="167" t="n">
         <x:v>46215.913194444445</x:v>
@@ -3027,16 +3027,16 @@
         <x:v>Risk-selected + full production</x:v>
       </x:c>
       <x:c r="M16" s="166" t="str">
-        <x:v>Browser-Base-QA @ f33c736; PR #89 @ 4c27f8d</x:v>
+        <x:v>Browser-Base-QA @ 8eff452; PR #89 @ a9c9e66</x:v>
       </x:c>
       <x:c r="N16" s="166" t="str">
-        <x:v>Standalone API executor and complete PRD are current; promotion wiring remains pending.</x:v>
+        <x:v>Standalone gate, PRD, integration contract, and full PestFlow QA implementation guide are current.</x:v>
       </x:c>
       <x:c r="O16" s="166" t="str">
         <x:v>Needs Browserbase secrets/context, deploy ownership, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P16" s="166" t="str">
-        <x:v>Deploy reviewed head, require 17 schema constraints, then 32/32 APIs, 81/81 routes, and the core/operational rejection matrix on the exact SHA.</x:v>
+        <x:v>Deploy reviewed head, require 26 schema constraints, then 32/32 APIs, 81/81 routes, and all tenant-rejection checks on the exact SHA.</x:v>
       </x:c>
       <x:c r="Q16" s="167" t="n">
         <x:v>46215.27099571759</x:v>
@@ -3288,19 +3288,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M21" s="170" t="str">
-        <x:v>31/32 production APIs; G-013–G-016 and G-018; 17 DB guardrails ready; PR #89 @ 4c27f8d</x:v>
+        <x:v>31/32 production APIs; G-013–G-016, G-018, G-019; 26 DB guardrails ready; PR #89 @ a9c9e66</x:v>
       </x:c>
       <x:c r="N21" s="170" t="str">
-        <x:v>4c27f8d; PR #89</x:v>
+        <x:v>a9c9e66; PR #89</x:v>
       </x:c>
       <x:c r="O21" s="170" t="str">
         <x:v>Needs merge/deploy authority, exact schema identity, production rejection proof, and restored Actions capacity.</x:v>
       </x:c>
       <x:c r="P21" s="170" t="str">
-        <x:v>Full branch proof is green; current production and the three historical chemical mismatches remain deliberately uncertified.</x:v>
+        <x:v>Full branch proof is green; current production and three historical chemical mismatches remain deliberately uncertified.</x:v>
       </x:c>
       <x:c r="Q21" s="171" t="n">
-        <x:v>46216.010416666664</x:v>
+        <x:v>46216.02777777778</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="138" customHeight="1">
@@ -5288,7 +5288,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6eb7dfdc55d40e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb413b2910b3469a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10233,20 +10233,225 @@
         <x:v>PR remains mergeable/unstable. The red check contains no product-test verdict.</x:v>
       </x:c>
     </x:row>
-    <x:row r="115">
-      <x:c r="B115" s="164"/>
-    </x:row>
-    <x:row r="116">
-      <x:c r="B116" s="164"/>
-    </x:row>
-    <x:row r="117">
-      <x:c r="B117" s="164"/>
-    </x:row>
-    <x:row r="118">
-      <x:c r="B118" s="164"/>
-    </x:row>
-    <x:row r="119">
-      <x:c r="B119" s="164"/>
+    <x:row r="115" ht="132" customHeight="1">
+      <x:c r="A115" s="174" t="str">
+        <x:v>AL-110</x:v>
+      </x:c>
+      <x:c r="B115" s="176" t="n">
+        <x:v>46216.02777777778</x:v>
+      </x:c>
+      <x:c r="C115" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D115" s="174" t="str">
+        <x:v>Audit provider and field-operation reference writes</x:v>
+      </x:c>
+      <x:c r="E115" s="174" t="str">
+        <x:v>Traced scheduled SMS, ProGlove trap scans, team invites, commercial portal ledgers, and contract-signing email from UI callers through route persistence and provider boundaries.</x:v>
+      </x:c>
+      <x:c r="F115" s="174" t="str">
+        <x:v>Source + schema audit</x:v>
+      </x:c>
+      <x:c r="G115" s="174" t="str">
+        <x:v>Four unguarded tenant-reference surfaces confirmed</x:v>
+      </x:c>
+      <x:c r="H115" s="174" t="str">
+        <x:v>Foreign IDs could reach scheduled-message, scan, invite, or email-ledger writes; signing email did not prove document/customer ownership or recipient identity before Resend.</x:v>
+      </x:c>
+      <x:c r="I115" s="174" t="str">
+        <x:v>API + provider boundary</x:v>
+      </x:c>
+      <x:c r="J115" s="174" t="str">
+        <x:v>server/routes/messaging.ts; invites.ts; sms-scheduled.ts; proglove.ts</x:v>
+      </x:c>
+      <x:c r="K115" s="174" t="str">
+        <x:v>G-019</x:v>
+      </x:c>
+      <x:c r="L115" s="174" t="str">
+        <x:v>Reuse the typed company-reference boundary and reject before any provider call.</x:v>
+      </x:c>
+      <x:c r="M115" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N115" s="174" t="str">
+        <x:v>No live email, SMS, invitation, or field write was used to prove the source-level gaps.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="132" customHeight="1">
+      <x:c r="A116" s="174" t="str">
+        <x:v>AL-111</x:v>
+      </x:c>
+      <x:c r="B116" s="176" t="n">
+        <x:v>46216.02777777778</x:v>
+      </x:c>
+      <x:c r="C116" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D116" s="174" t="str">
+        <x:v>Audit existing provider and field data read-only</x:v>
+      </x:c>
+      <x:c r="E116" s="174" t="str">
+        <x:v>Extended the database-enforced read-only inventory across notification email, scheduled SMS, invites, and ProGlove records.</x:v>
+      </x:c>
+      <x:c r="F116" s="174" t="str">
+        <x:v>Railway + Postgres READ ONLY</x:v>
+      </x:c>
+      <x:c r="G116" s="174" t="str">
+        <x:v>Production relationships are clean</x:v>
+      </x:c>
+      <x:c r="H116" s="174" t="str">
+        <x:v>All four expected tables exist. 536/536 populated company references and 259/259 paired document/job-to-customer relationships had zero mismatches.</x:v>
+      </x:c>
+      <x:c r="I116" s="174" t="str">
+        <x:v>Production database</x:v>
+      </x:c>
+      <x:c r="J116" s="174" t="str">
+        <x:v>scripts/qa-operational-tenant-integrity.ts</x:v>
+      </x:c>
+      <x:c r="K116" s="174" t="str">
+        <x:v>a9c9e66; G-019</x:v>
+      </x:c>
+      <x:c r="L116" s="174" t="str">
+        <x:v>Use the clean baseline for preventative enforcement; do not rewrite rows.</x:v>
+      </x:c>
+      <x:c r="M116" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N116" s="174" t="str">
+        <x:v>Aggregate output contained no record IDs, names, emails, phone numbers, message bodies, or document content.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="132" customHeight="1">
+      <x:c r="A117" s="174" t="str">
+        <x:v>AL-112</x:v>
+      </x:c>
+      <x:c r="B117" s="176" t="n">
+        <x:v>46216.02777777778</x:v>
+      </x:c>
+      <x:c r="C117" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="D117" s="174" t="str">
+        <x:v>Harden provider and field tenant references</x:v>
+      </x:c>
+      <x:c r="E117" s="174" t="str">
+        <x:v>Extended the shared validator to service documents, guarded four route families, bound signing recipients to owned records, added the missing ProGlove schema migration, and expanded the release oracle from 17 to 26 constraints.</x:v>
+      </x:c>
+      <x:c r="F117" s="174" t="str">
+        <x:v>PestFlow API + Postgres + Guardian</x:v>
+      </x:c>
+      <x:c r="G117" s="174" t="str">
+        <x:v>Provider and field prevention implemented</x:v>
+      </x:c>
+      <x:c r="H117" s="174" t="str">
+        <x:v>Malformed/inconsistent IDs return 400 and foreign/missing IDs return 404 before persistence or delivery. Nine new composite constraints enforce future writes.</x:v>
+      </x:c>
+      <x:c r="I117" s="174" t="str">
+        <x:v>API + database</x:v>
+      </x:c>
+      <x:c r="J117" s="174" t="str">
+        <x:v>migrations/a25_provider_field_tenant_integrity.sql</x:v>
+      </x:c>
+      <x:c r="K117" s="174" t="str">
+        <x:v>a9c9e66; PR #89</x:v>
+      </x:c>
+      <x:c r="L117" s="174" t="str">
+        <x:v>Deploy the reviewed head and prove all 26 constraints on its exact SHA.</x:v>
+      </x:c>
+      <x:c r="M117" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N117" s="174" t="str">
+        <x:v>Commercial portal access can still invite new contacts; only a supplied customer ledger ID is company-validated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="132" customHeight="1">
+      <x:c r="A118" s="174" t="str">
+        <x:v>AL-113</x:v>
+      </x:c>
+      <x:c r="B118" s="176" t="n">
+        <x:v>46216.02777777778</x:v>
+      </x:c>
+      <x:c r="C118" s="174" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D118" s="174" t="str">
+        <x:v>Validate, document, and publish provider hardening</x:v>
+      </x:c>
+      <x:c r="E118" s="174" t="str">
+        <x:v>Ran every local gate, pushed PestFlow a9c9e66, synchronized the 571-line PRD, and added a 581-line implementation guide to Browser-Base-QA at 8eff452.</x:v>
+      </x:c>
+      <x:c r="F118" s="174" t="str">
+        <x:v>Vitest + Node + TypeScript + ESLint + Vite + GitHub</x:v>
+      </x:c>
+      <x:c r="G118" s="174" t="str">
+        <x:v>Implementation and shared documentation published</x:v>
+      </x:c>
+      <x:c r="H118" s="174" t="str">
+        <x:v>794/794 unit across 78 files, 48/48 Guardian policy, 16/16 incident, typecheck, lint, and the 5,699-module build passed. Browser-Base-QA tests passed 6/6.</x:v>
+      </x:c>
+      <x:c r="I118" s="174" t="str">
+        <x:v>Code + documentation</x:v>
+      </x:c>
+      <x:c r="J118" s="174" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA/blob/main/docs/PRD.md</x:v>
+      </x:c>
+      <x:c r="K118" s="174" t="str">
+        <x:v>a9c9e66; 8eff452; PR #89</x:v>
+      </x:c>
+      <x:c r="L118" s="174" t="str">
+        <x:v>Record exact-head cloud-gate evidence and await deploy authority.</x:v>
+      </x:c>
+      <x:c r="M118" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N118" s="174" t="str">
+        <x:v>PRD is byte-identical to PestFlow; the separate implementation guide documents PestFlow QA folders and files.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="132" customHeight="1">
+      <x:c r="A119" s="174" t="str">
+        <x:v>AL-114</x:v>
+      </x:c>
+      <x:c r="B119" s="176" t="n">
+        <x:v>46216.02777777778</x:v>
+      </x:c>
+      <x:c r="C119" s="174" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="D119" s="174" t="str">
+        <x:v>Classify exact provider-hardening PR gate</x:v>
+      </x:c>
+      <x:c r="E119" s="174" t="str">
+        <x:v>Inspected the automatic release gate for exact PestFlow head a9c9e66 and verified whether any command executed.</x:v>
+      </x:c>
+      <x:c r="F119" s="174" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="G119" s="174" t="str">
+        <x:v>Cloud gate blocked before execution</x:v>
+      </x:c>
+      <x:c r="H119" s="174" t="str">
+        <x:v>Run 29215702743, job 86711046743 had zero steps and the verified failed-payment or spending-limit annotation.</x:v>
+      </x:c>
+      <x:c r="I119" s="174" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="J119" s="174" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/actions/runs/29215702743</x:v>
+      </x:c>
+      <x:c r="K119" s="174" t="str">
+        <x:v>a9c9e66; PR #89</x:v>
+      </x:c>
+      <x:c r="L119" s="174" t="str">
+        <x:v>Restore Actions capacity and rerun exact-head selector, schema oracle, deterministic, and browser gates.</x:v>
+      </x:c>
+      <x:c r="M119" s="174" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="N119" s="174" t="str">
+        <x:v>PR is mergeable/unstable. This red check contains no product-test verdict.</x:v>
+      </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="B120" s="164"/>
@@ -10516,7 +10721,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ecb165b1d894e37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8c0f8000b4b4254"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14114,30 +14319,180 @@
         <x:v>Verified payment/spending refusal; no selector, schema oracle, product test, or browser command started.</x:v>
       </x:c>
     </x:row>
-    <x:row r="105">
-      <x:c r="A105" s="133"/>
-      <x:c r="B105" s="133"/>
-      <x:c r="C105" s="133"/>
-      <x:c r="D105" s="133"/>
-      <x:c r="E105" s="133"/>
-      <x:c r="F105" s="133"/>
-      <x:c r="G105" s="133"/>
-      <x:c r="H105" s="133"/>
-      <x:c r="I105" s="165"/>
-      <x:c r="J105" s="133"/>
-      <x:c r="K105" s="133"/>
-    </x:row>
-    <x:row r="106">
-      <x:c r="I106" s="164"/>
-    </x:row>
-    <x:row r="107">
-      <x:c r="I107" s="164"/>
-    </x:row>
-    <x:row r="108">
-      <x:c r="I108" s="164"/>
-    </x:row>
-    <x:row r="109">
-      <x:c r="I109" s="164"/>
+    <x:row r="105" ht="94" customHeight="1">
+      <x:c r="A105" s="170" t="str">
+        <x:v>QA-100</x:v>
+      </x:c>
+      <x:c r="B105" s="170" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C105" s="170" t="str">
+        <x:v>Provider and field tenant route boundary</x:v>
+      </x:c>
+      <x:c r="D105" s="170" t="str">
+        <x:v>8 focused tests</x:v>
+      </x:c>
+      <x:c r="E105" s="170" t="str">
+        <x:v>Vitest</x:v>
+      </x:c>
+      <x:c r="F105" s="170" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G105" s="170" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H105" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I105" s="171" t="n">
+        <x:v>46216.02777777778</x:v>
+      </x:c>
+      <x:c r="J105" s="170" t="str">
+        <x:v>8/8 passed</x:v>
+      </x:c>
+      <x:c r="K105" s="170" t="str">
+        <x:v>Rejected foreign SMS, scan, invite, portal-ledger, document, and recipient references before writes/provider delivery; valid SMS/email paths still pass.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="94" customHeight="1">
+      <x:c r="A106" s="174" t="str">
+        <x:v>QA-101</x:v>
+      </x:c>
+      <x:c r="B106" s="174" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="C106" s="174" t="str">
+        <x:v>Provider and field relationship integrity</x:v>
+      </x:c>
+      <x:c r="D106" s="174" t="str">
+        <x:v>536 references + 259 paired rows</x:v>
+      </x:c>
+      <x:c r="E106" s="174" t="str">
+        <x:v>Read-only Postgres</x:v>
+      </x:c>
+      <x:c r="F106" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G106" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="H106" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I106" s="176" t="n">
+        <x:v>46216.02777777778</x:v>
+      </x:c>
+      <x:c r="J106" s="174" t="str">
+        <x:v>536/536 scoped; 259/259 consistent</x:v>
+      </x:c>
+      <x:c r="K106" s="174" t="str">
+        <x:v>All four expected tables were present; no company or document/job-to-customer mismatch was found.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="94" customHeight="1">
+      <x:c r="A107" s="174" t="str">
+        <x:v>QA-102</x:v>
+      </x:c>
+      <x:c r="B107" s="174" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="C107" s="174" t="str">
+        <x:v>Provider and field constraint migration</x:v>
+      </x:c>
+      <x:c r="D107" s="174" t="str">
+        <x:v>Disposable PostgreSQL 17</x:v>
+      </x:c>
+      <x:c r="E107" s="174" t="str">
+        <x:v>psql</x:v>
+      </x:c>
+      <x:c r="F107" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G107" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H107" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I107" s="176" t="n">
+        <x:v>46216.02777777778</x:v>
+      </x:c>
+      <x:c r="J107" s="174" t="str">
+        <x:v>9/9 constraints installed</x:v>
+      </x:c>
+      <x:c r="K107" s="174" t="str">
+        <x:v>Synthetic cross-company insert failed; valid customer deletion cleared only customer_id and retained non-null company_id.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="94" customHeight="1">
+      <x:c r="A108" s="174" t="str">
+        <x:v>QA-103</x:v>
+      </x:c>
+      <x:c r="B108" s="174" t="str">
+        <x:v>Quality</x:v>
+      </x:c>
+      <x:c r="C108" s="174" t="str">
+        <x:v>Full provider-hardening branch validation</x:v>
+      </x:c>
+      <x:c r="D108" s="174" t="str">
+        <x:v>78 unit files + Guardian + incident + build</x:v>
+      </x:c>
+      <x:c r="E108" s="174" t="str">
+        <x:v>Vitest + Node + TypeScript + ESLint + Vite</x:v>
+      </x:c>
+      <x:c r="F108" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G108" s="174" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="H108" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I108" s="176" t="n">
+        <x:v>46216.02777777778</x:v>
+      </x:c>
+      <x:c r="J108" s="174" t="str">
+        <x:v>794/794; 48/48; 16/16; build passed</x:v>
+      </x:c>
+      <x:c r="K108" s="174" t="str">
+        <x:v>Typecheck and touched-file lint are clean; production build transformed 5,699 modules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="94" customHeight="1">
+      <x:c r="A109" s="174" t="str">
+        <x:v>QA-104</x:v>
+      </x:c>
+      <x:c r="B109" s="174" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C109" s="174" t="str">
+        <x:v>Exact provider-hardening PR gate</x:v>
+      </x:c>
+      <x:c r="D109" s="174" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="E109" s="174" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F109" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G109" s="174" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H109" s="174" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I109" s="176" t="n">
+        <x:v>46216.02777777778</x:v>
+      </x:c>
+      <x:c r="J109" s="174" t="str">
+        <x:v>Run 29215702743: zero steps</x:v>
+      </x:c>
+      <x:c r="K109" s="174" t="str">
+        <x:v>Verified payment/spending refusal; no selector, schema oracle, product test, or browser command started.</x:v>
+      </x:c>
     </x:row>
     <x:row r="110">
       <x:c r="I110" s="164"/>
@@ -14440,7 +14795,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03939a43477d40be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b071bd56231419c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15295,6 +15650,44 @@
       </x:c>
       <x:c r="L24" s="174" t="str">
         <x:v>Branch prevention is ready at route and database layers. Current production was not mutated to demonstrate each source-proven gap.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="150" customHeight="1">
+      <x:c r="A25" s="174" t="str">
+        <x:v>G-019</x:v>
+      </x:c>
+      <x:c r="B25" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="C25" s="174" t="str">
+        <x:v>Provider and Field Tenant Integrity</x:v>
+      </x:c>
+      <x:c r="D25" s="174" t="str">
+        <x:v>Scheduled SMS, ProGlove scans, team/portal invite ledgers, and contract-signing email did not consistently prove supplied record IDs and recipients belonged to the authenticated company before persistence or delivery.</x:v>
+      </x:c>
+      <x:c r="E25" s="174" t="str">
+        <x:v>A crafted or stale request could create cross-company operational links or send a branded signing email without an owned document/customer-recipient match.</x:v>
+      </x:c>
+      <x:c r="F25" s="174" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G25" s="174" t="str">
+        <x:v>Deploy a9c9e66, prove all 26 schema constraints on the exact SHA, then run controlled synthetic rejection checks without real provider sends.</x:v>
+      </x:c>
+      <x:c r="H25" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I25" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="J25" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K25" s="174" t="str">
+        <x:v>8/8 focused regressions; disposable Postgres enforcement passed; production read-only audit found 536/536 references and 259/259 paired rows clean.</x:v>
+      </x:c>
+      <x:c r="L25" s="174" t="str">
+        <x:v>Branch prevention is ready. Current production remains uncertified until exact-SHA deployment and schema/rejection proof.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15331,7 +15724,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R782e7b3b64744ee6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R363c669ccf364bd8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record provider diagnostic safeguards
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2a2f4333fbdf429d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R24aeedbf59d640e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="Rc95e2add13464b62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R5f700a3ed6d54f82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R36372977c6af4187"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9568972441b14528"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R955f921b743a46df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R4e689623fa0548d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R7f8dcc80b2bd48a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R161c54fbc58f4d5e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1343,7 +1343,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N123" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1365,7 +1365,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K109" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K113" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1384,7 +1384,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Gap ID"/>
     <x:tableColumn id="2" name="Found During Task"/>
@@ -1767,12 +1767,12 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>104</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>72</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
@@ -1782,7 +1782,7 @@
       <x:c r="F9" s="141"/>
       <x:c r="G9" s="138" t="n">
         <x:f>COUNTIFS('Product Gaps'!$A$6:$A$200,"&lt;&gt;",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Closed",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Resolved",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Mitigated")</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H9" s="139"/>
     </x:row>
@@ -1941,25 +1941,25 @@
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Core production data is 453/453 scoped; provider/field data is 536/536 scoped and 259/259 paired-consistent. Operational isolation remains 200/200 until deployment.</x:v>
+        <x:v>Tenant audits are clean outside 3 historical chemical mappings; provider diagnostics now fail closed or deduplicate. Current production still awaits the reviewed deploy.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ a9c9e66; Browser-Base-QA @ 8eff452 shared with yawbtng; PRD and full implementation guide synchronized.</x:v>
+        <x:v>PestFlow PR #89 @ 36e7ab7; Browser-Base-QA @ e1089df shared with yawbtng; PRD and implementation guide synchronized.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Activation</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>Restore Actions; deploy a9c9e66; prove 26 schema constraints, exact-SHA 32/32 APIs, 81/81 routes, and the complete tenant rejection matrix.</x:v>
+        <x:v>Restore Actions; deploy 36e7ab7; prove 26 constraints, provider safeguards, exact-SHA 32/32 APIs, 81/81 routes, and tenant rejection matrix.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>No production row or provider was changed. PR mergeable/unstable; run 29215702743 was zero-step billing blocked.</x:v>
+        <x:v>No production row or provider was changed. Run 29216078831 was zero-step billing blocked.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2620,11 +2620,11 @@
         <x:v>/private/tmp/pestflow-desktop-qa-guardian/qa/guardian/desktop-journeys.json</x:v>
       </x:c>
       <x:c r="N8" s="113" t="str">
-        <x:v>a9c9e66 + Browser-Base-QA 8eff452; PR #89</x:v>
+        <x:v>36e7ab7 + Browser-Base-QA e1089df; PR #89</x:v>
       </x:c>
       <x:c r="O8" s="113"/>
       <x:c r="P8" s="113" t="str">
-        <x:v>Shared validator, 26 constraints, expanded audit, schema oracle, 571-line PRD, and 581-line implementation guide are synchronized.</x:v>
+        <x:v>PRD, full implementation guide, provider/field constraints, and provider diagnostic safeguards are synchronized.</x:v>
       </x:c>
       <x:c r="Q8" s="163" t="n">
         <x:v>46215.27099571759</x:v>
@@ -2821,19 +2821,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M12" s="166" t="str">
-        <x:v>Core 453/453 + provider/field 536/536 references scoped; 29/29 + 259/259 paired relationships consistent</x:v>
+        <x:v>Tenant data clean; provider diagnostics now confirmation/idempotency guarded; live operational isolation remains 200/200 until deploy</x:v>
       </x:c>
       <x:c r="N12" s="166" t="str">
-        <x:v>a9c9e66; PR #89</x:v>
+        <x:v>36e7ab7; PR #89</x:v>
       </x:c>
       <x:c r="O12" s="166" t="str">
-        <x:v>Requires reviewed deploy, 26-constraint schema proof, production rejection matrix, and restored Actions capacity.</x:v>
+        <x:v>Requires reviewed deploy, 26-constraint proof, provider diagnostic proof, tenant rejection matrix, and restored Actions.</x:v>
       </x:c>
       <x:c r="P12" s="166" t="str">
-        <x:v>Branch now protects core, operational, provider, and field references at route and database layers; current production remains uncertified.</x:v>
+        <x:v>Branch guards tenant references plus external diagnostic destinations/retries; current production remains uncertified.</x:v>
       </x:c>
       <x:c r="Q12" s="167" t="n">
-        <x:v>46216.02777777778</x:v>
+        <x:v>46216.03611111111</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2928,11 +2928,11 @@
         <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/pull/89</x:v>
       </x:c>
       <x:c r="N14" s="166" t="str">
-        <x:v>a9c9e66; PR #89</x:v>
+        <x:v>36e7ab7; PR #89</x:v>
       </x:c>
       <x:c r="O14" s="166"/>
       <x:c r="P14" s="166" t="str">
-        <x:v>Full branch gate passed; exact-head cloud run 29215702743 was zero-step billing blocked; no product command ran.</x:v>
+        <x:v>798-test branch gate passed; exact-head cloud run 29216078831 was zero-step billing blocked.</x:v>
       </x:c>
       <x:c r="Q14" s="167" t="n">
         <x:v>46215.913194444445</x:v>
@@ -3027,7 +3027,7 @@
         <x:v>Risk-selected + full production</x:v>
       </x:c>
       <x:c r="M16" s="166" t="str">
-        <x:v>Browser-Base-QA @ 8eff452; PR #89 @ a9c9e66</x:v>
+        <x:v>Browser-Base-QA @ e1089df; PR #89 @ 36e7ab7</x:v>
       </x:c>
       <x:c r="N16" s="166" t="str">
         <x:v>Standalone gate, PRD, integration contract, and full PestFlow QA implementation guide are current.</x:v>
@@ -3036,7 +3036,7 @@
         <x:v>Needs Browserbase secrets/context, deploy ownership, and restored GitHub Actions capacity.</x:v>
       </x:c>
       <x:c r="P16" s="166" t="str">
-        <x:v>Deploy reviewed head, require 26 schema constraints, then 32/32 APIs, 81/81 routes, and all tenant-rejection checks on the exact SHA.</x:v>
+        <x:v>Deploy reviewed head, require 26 constraints, prove provider safeguards, then 32/32 APIs, 81/81 routes, and tenant rejection checks.</x:v>
       </x:c>
       <x:c r="Q16" s="167" t="n">
         <x:v>46215.27099571759</x:v>
@@ -3288,19 +3288,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M21" s="170" t="str">
-        <x:v>31/32 production APIs; G-013–G-016, G-018, G-019; 26 DB guardrails ready; PR #89 @ a9c9e66</x:v>
+        <x:v>31/32 production APIs; G-013–G-016 and G-018–G-020; 26 DB guards + provider safeguards ready; PR #89 @ 36e7ab7</x:v>
       </x:c>
       <x:c r="N21" s="170" t="str">
-        <x:v>a9c9e66; PR #89</x:v>
+        <x:v>36e7ab7; PR #89</x:v>
       </x:c>
       <x:c r="O21" s="170" t="str">
-        <x:v>Needs merge/deploy authority, exact schema identity, production rejection proof, and restored Actions capacity.</x:v>
+        <x:v>Needs merge/deploy authority, exact schema/provider proof, tenant rejection proof, and restored Actions.</x:v>
       </x:c>
       <x:c r="P21" s="170" t="str">
         <x:v>Full branch proof is green; current production and three historical chemical mismatches remain deliberately uncertified.</x:v>
       </x:c>
       <x:c r="Q21" s="171" t="n">
-        <x:v>46216.02777777778</x:v>
+        <x:v>46216.03611111111</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="138" customHeight="1">
@@ -5288,7 +5288,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb413b2910b3469a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59aea61eabb34c20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10453,17 +10453,181 @@
         <x:v>PR is mergeable/unstable. This red check contains no product-test verdict.</x:v>
       </x:c>
     </x:row>
-    <x:row r="120">
-      <x:c r="B120" s="164"/>
-    </x:row>
-    <x:row r="121">
-      <x:c r="B121" s="164"/>
-    </x:row>
-    <x:row r="122">
-      <x:c r="B122" s="164"/>
-    </x:row>
-    <x:row r="123">
-      <x:c r="B123" s="164"/>
+    <x:row r="120" ht="132" customHeight="1">
+      <x:c r="A120" s="174" t="str">
+        <x:v>AL-115</x:v>
+      </x:c>
+      <x:c r="B120" s="176" t="n">
+        <x:v>46216.03611111111</x:v>
+      </x:c>
+      <x:c r="C120" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="D120" s="174" t="str">
+        <x:v>Sweep remaining external-provider diagnostics</x:v>
+      </x:c>
+      <x:c r="E120" s="174" t="str">
+        <x:v>Inventoried authenticated routes that can email, text, invite, charge, or call Stripe/Resend and traced their UI callers and existing confirmation/idempotency boundaries.</x:v>
+      </x:c>
+      <x:c r="F120" s="174" t="str">
+        <x:v>Source + caller audit</x:v>
+      </x:c>
+      <x:c r="G120" s="174" t="str">
+        <x:v>Two diagnostic safety gaps confirmed</x:v>
+      </x:c>
+      <x:c r="H120" s="174" t="str">
+        <x:v>The staging 28-email proof was callable in production, and the real $1 Stripe test-send had no server confirmation or retry idempotency.</x:v>
+      </x:c>
+      <x:c r="I120" s="174" t="str">
+        <x:v>Provider boundary</x:v>
+      </x:c>
+      <x:c r="J120" s="174" t="str">
+        <x:v>server/routes/feature-actions.ts; server/routes/invoices.ts</x:v>
+      </x:c>
+      <x:c r="K120" s="174" t="str">
+        <x:v>G-020</x:v>
+      </x:c>
+      <x:c r="L120" s="174" t="str">
+        <x:v>Fail closed for staging-only bulk proof and deduplicate intentional Stripe diagnostics.</x:v>
+      </x:c>
+      <x:c r="M120" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N120" s="174" t="str">
+        <x:v>No live provider action was executed during discovery or validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="132" customHeight="1">
+      <x:c r="A121" s="174" t="str">
+        <x:v>AL-116</x:v>
+      </x:c>
+      <x:c r="B121" s="176" t="n">
+        <x:v>46216.03611111111</x:v>
+      </x:c>
+      <x:c r="C121" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="D121" s="174" t="str">
+        <x:v>Make provider diagnostics fail safe</x:v>
+      </x:c>
+      <x:c r="E121" s="174" t="str">
+        <x:v>Returned 404 for the 28-email batch in production; required a server-verified confirmation for Stripe test-send; added operation-specific Stripe idempotency across customer, invoice, item, finalize, and send; updated all four callers.</x:v>
+      </x:c>
+      <x:c r="F121" s="174" t="str">
+        <x:v>PestFlow API + desktop/mobile UI</x:v>
+      </x:c>
+      <x:c r="G121" s="174" t="str">
+        <x:v>Accidental provider duplication prevented</x:v>
+      </x:c>
+      <x:c r="H121" s="174" t="str">
+        <x:v>Retries to the same company/email within ten minutes reuse the same Stripe operations, while intentional one-off owner diagnostics still work.</x:v>
+      </x:c>
+      <x:c r="I121" s="174" t="str">
+        <x:v>API + provider</x:v>
+      </x:c>
+      <x:c r="J121" s="174" t="str">
+        <x:v>server/routes/invoices.ts; server/routes/feature-actions.ts</x:v>
+      </x:c>
+      <x:c r="K121" s="174" t="str">
+        <x:v>36e7ab7; PR #89</x:v>
+      </x:c>
+      <x:c r="L121" s="174" t="str">
+        <x:v>Deploy and prove production bulk-preview denial before enabling live diagnostic certification.</x:v>
+      </x:c>
+      <x:c r="M121" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N121" s="174" t="str">
+        <x:v>Also removed 15 touched-file explicit-any violations from MobileInvoicesPage instead of hiding lint debt.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="132" customHeight="1">
+      <x:c r="A122" s="174" t="str">
+        <x:v>AL-117</x:v>
+      </x:c>
+      <x:c r="B122" s="176" t="n">
+        <x:v>46216.03611111111</x:v>
+      </x:c>
+      <x:c r="C122" s="174" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="D122" s="174" t="str">
+        <x:v>Validate and publish provider diagnostic safeguards</x:v>
+      </x:c>
+      <x:c r="E122" s="174" t="str">
+        <x:v>Ran the complete gate, pushed PestFlow 36e7ab7, and synchronized the updated PRD and implementation guide to Browser-Base-QA e1089df.</x:v>
+      </x:c>
+      <x:c r="F122" s="174" t="str">
+        <x:v>Vitest + Node + TypeScript + ESLint + Vite + GitHub</x:v>
+      </x:c>
+      <x:c r="G122" s="174" t="str">
+        <x:v>Provider safeguards published</x:v>
+      </x:c>
+      <x:c r="H122" s="174" t="str">
+        <x:v>798/798 unit across 79 files, 48/48 Guardian policy, 16/16 incident, typecheck, lint, and the 5,699-module build passed. Browser-Base-QA passed 6/6.</x:v>
+      </x:c>
+      <x:c r="I122" s="174" t="str">
+        <x:v>Code + documentation</x:v>
+      </x:c>
+      <x:c r="J122" s="174" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/pull/89</x:v>
+      </x:c>
+      <x:c r="K122" s="174" t="str">
+        <x:v>36e7ab7; e1089df</x:v>
+      </x:c>
+      <x:c r="L122" s="174" t="str">
+        <x:v>Record the exact-head cloud gate and update the shared tracker.</x:v>
+      </x:c>
+      <x:c r="M122" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N122" s="174" t="str">
+        <x:v>Focused provider-safety suite passed 8/8; no Stripe or Resend network request was made by validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="132" customHeight="1">
+      <x:c r="A123" s="174" t="str">
+        <x:v>AL-118</x:v>
+      </x:c>
+      <x:c r="B123" s="176" t="n">
+        <x:v>46216.03611111111</x:v>
+      </x:c>
+      <x:c r="C123" s="174" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="D123" s="174" t="str">
+        <x:v>Classify exact diagnostic-safety PR gate</x:v>
+      </x:c>
+      <x:c r="E123" s="174" t="str">
+        <x:v>Inspected the automatic release gate for exact PestFlow head 36e7ab7 and verified whether any command executed.</x:v>
+      </x:c>
+      <x:c r="F123" s="174" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="G123" s="174" t="str">
+        <x:v>Cloud gate blocked before execution</x:v>
+      </x:c>
+      <x:c r="H123" s="174" t="str">
+        <x:v>Run 29216078831, job 86712135690 had zero steps under the same verified account billing/spending refusal.</x:v>
+      </x:c>
+      <x:c r="I123" s="174" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="J123" s="174" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/actions/runs/29216078831</x:v>
+      </x:c>
+      <x:c r="K123" s="174" t="str">
+        <x:v>36e7ab7; PR #89</x:v>
+      </x:c>
+      <x:c r="L123" s="174" t="str">
+        <x:v>Restore Actions capacity and rerun the exact-head release gate.</x:v>
+      </x:c>
+      <x:c r="M123" s="174" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="N123" s="174" t="str">
+        <x:v>The red check contains no product-test verdict.</x:v>
+      </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="B124" s="164"/>
@@ -10721,7 +10885,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8c0f8000b4b4254"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea9d7abcf6c6437a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14494,17 +14658,145 @@
         <x:v>Verified payment/spending refusal; no selector, schema oracle, product test, or browser command started.</x:v>
       </x:c>
     </x:row>
-    <x:row r="110">
-      <x:c r="I110" s="164"/>
-    </x:row>
-    <x:row r="111">
-      <x:c r="I111" s="164"/>
-    </x:row>
-    <x:row r="112">
-      <x:c r="I112" s="164"/>
-    </x:row>
-    <x:row r="113">
-      <x:c r="I113" s="164"/>
+    <x:row r="110" ht="94" customHeight="1">
+      <x:c r="A110" s="174" t="str">
+        <x:v>QA-105</x:v>
+      </x:c>
+      <x:c r="B110" s="174" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="C110" s="174" t="str">
+        <x:v>Production bulk-email preview denial</x:v>
+      </x:c>
+      <x:c r="D110" s="174" t="str">
+        <x:v>28-template preview endpoint</x:v>
+      </x:c>
+      <x:c r="E110" s="174" t="str">
+        <x:v>Vitest</x:v>
+      </x:c>
+      <x:c r="F110" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G110" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H110" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I110" s="176" t="n">
+        <x:v>46216.03611111111</x:v>
+      </x:c>
+      <x:c r="J110" s="174" t="str">
+        <x:v>404 before SQL/provider</x:v>
+      </x:c>
+      <x:c r="K110" s="174" t="str">
+        <x:v>Production request returned Not found; fetch and SQL mocks remained untouched.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="94" customHeight="1">
+      <x:c r="A111" s="174" t="str">
+        <x:v>QA-106</x:v>
+      </x:c>
+      <x:c r="B111" s="174" t="str">
+        <x:v>Reliability</x:v>
+      </x:c>
+      <x:c r="C111" s="174" t="str">
+        <x:v>Stripe diagnostic confirmation and idempotency</x:v>
+      </x:c>
+      <x:c r="D111" s="174" t="str">
+        <x:v>Server route + four callers</x:v>
+      </x:c>
+      <x:c r="E111" s="174" t="str">
+        <x:v>Source contract + TypeScript</x:v>
+      </x:c>
+      <x:c r="F111" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G111" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="H111" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I111" s="176" t="n">
+        <x:v>46216.03611111111</x:v>
+      </x:c>
+      <x:c r="J111" s="174" t="str">
+        <x:v>5/5 operations idempotent</x:v>
+      </x:c>
+      <x:c r="K111" s="174" t="str">
+        <x:v>Confirmation precedes company/Stripe lookup; customer, invoice, item, finalize, and send use operation-specific keys in a ten-minute window.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="94" customHeight="1">
+      <x:c r="A112" s="174" t="str">
+        <x:v>QA-107</x:v>
+      </x:c>
+      <x:c r="B112" s="174" t="str">
+        <x:v>Quality</x:v>
+      </x:c>
+      <x:c r="C112" s="174" t="str">
+        <x:v>Full diagnostic-safety branch validation</x:v>
+      </x:c>
+      <x:c r="D112" s="174" t="str">
+        <x:v>79 unit files + Guardian + incident + build</x:v>
+      </x:c>
+      <x:c r="E112" s="174" t="str">
+        <x:v>Vitest + Node + TypeScript + ESLint + Vite</x:v>
+      </x:c>
+      <x:c r="F112" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G112" s="174" t="str">
+        <x:v>T-009</x:v>
+      </x:c>
+      <x:c r="H112" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I112" s="176" t="n">
+        <x:v>46216.03611111111</x:v>
+      </x:c>
+      <x:c r="J112" s="174" t="str">
+        <x:v>798/798; 48/48; 16/16; build passed</x:v>
+      </x:c>
+      <x:c r="K112" s="174" t="str">
+        <x:v>Touched-file lint is clean and production build transformed 5,699 modules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="94" customHeight="1">
+      <x:c r="A113" s="174" t="str">
+        <x:v>QA-108</x:v>
+      </x:c>
+      <x:c r="B113" s="174" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C113" s="174" t="str">
+        <x:v>Exact diagnostic-safety PR gate</x:v>
+      </x:c>
+      <x:c r="D113" s="174" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="E113" s="174" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F113" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G113" s="174" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H113" s="174" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I113" s="176" t="n">
+        <x:v>46216.03611111111</x:v>
+      </x:c>
+      <x:c r="J113" s="174" t="str">
+        <x:v>Run 29216078831: zero steps</x:v>
+      </x:c>
+      <x:c r="K113" s="174" t="str">
+        <x:v>Verified payment/spending refusal; no product command started.</x:v>
+      </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="I114" s="164"/>
@@ -14795,7 +15087,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b071bd56231419c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2687a90aa8bf4405"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15688,6 +15980,44 @@
       </x:c>
       <x:c r="L25" s="174" t="str">
         <x:v>Branch prevention is ready. Current production remains uncertified until exact-SHA deployment and schema/rejection proof.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="150" customHeight="1">
+      <x:c r="A26" s="174" t="str">
+        <x:v>G-020</x:v>
+      </x:c>
+      <x:c r="B26" s="174" t="str">
+        <x:v>T-007</x:v>
+      </x:c>
+      <x:c r="C26" s="174" t="str">
+        <x:v>Provider Diagnostic Safety</x:v>
+      </x:c>
+      <x:c r="D26" s="174" t="str">
+        <x:v>A staging-only 28-email preview was reachable in production, and the real $1 Stripe test-send lacked server confirmation and provider idempotency.</x:v>
+      </x:c>
+      <x:c r="E26" s="174" t="str">
+        <x:v>An authenticated mistake, retry, or double-click could schedule bulk proof email or create duplicate Stripe test customers, invoices, items, finalizations, and sends.</x:v>
+      </x:c>
+      <x:c r="F26" s="174" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G26" s="174" t="str">
+        <x:v>Deploy 36e7ab7, prove the preview returns 404 in production, and verify repeated confirmed test-send requests return one Stripe operation set.</x:v>
+      </x:c>
+      <x:c r="H26" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I26" s="174" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="J26" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K26" s="174" t="str">
+        <x:v>8/8 focused safeguards; 798/798 full unit; type/lint/build green; no live provider request used for verification.</x:v>
+      </x:c>
+      <x:c r="L26" s="174" t="str">
+        <x:v>Branch prevention is ready. Exact production provider proof remains intentionally pending deployment and an approved test recipient.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15724,7 +16054,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R363c669ccf364bd8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20dbcffc68f84f02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record full stack reliability validation
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9568972441b14528"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R955f921b743a46df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R4e689623fa0548d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R7f8dcc80b2bd48a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R161c54fbc58f4d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R95a1032832fe4c94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="Rc49384986b034da8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R138ac5aed1b2402f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Rdcb465de143b48b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R4c26bd66d16a4f6d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1318,7 +1318,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskTrackerTable" displayName="TaskTrackerTable" ref="A5:Q22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskTrackerTable" displayName="TaskTrackerTable" ref="A5:Q26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Task ID"/>
     <x:tableColumn id="2" name="Phase"/>
@@ -1343,7 +1343,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N123" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N128" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1365,7 +1365,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K113" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K121" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1384,7 +1384,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Gap ID"/>
     <x:tableColumn id="2" name="Found During Task"/>
@@ -1699,17 +1699,17 @@
     <x:row r="5">
       <x:c r="A5" s="134" t="n">
         <x:f>COUNTA('Task Tracker'!$A$6:$A$200)</x:f>
-        <x:v>17</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B5" s="135"/>
       <x:c r="C5" s="136" t="n">
         <x:f>COUNTIF('Task Tracker'!$E$6:$E$200,"Done")</x:f>
-        <x:v>9</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D5" s="137"/>
       <x:c r="E5" s="138" t="n">
         <x:f>COUNTIF('Task Tracker'!$E$6:$E$200,"In Progress")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F5" s="139"/>
       <x:c r="G5" s="140" t="n">
@@ -1767,22 +1767,22 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>108</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>75</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Failed")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F9" s="141"/>
       <x:c r="G9" s="138" t="n">
         <x:f>COUNTIFS('Product Gaps'!$A$6:$A$200,"&lt;&gt;",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Closed",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Resolved",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Mitigated")</x:f>
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H9" s="139"/>
     </x:row>
@@ -1941,25 +1941,25 @@
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Tenant audits are clean outside 3 historical chemical mappings; provider diagnostics now fail closed or deduplicate. Current production still awaits the reviewed deploy.</x:v>
+        <x:v>All 24 direct Resend deliveries are retry-safe and both TypeScript graphs are release-gated. Local unit, policy, incident, build, and browser checks pass.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ 36e7ab7; Browser-Base-QA @ e1089df shared with yawbtng; PRD and implementation guide synchronized.</x:v>
+        <x:v>PestFlow PR #89 @ 9083c93; Browser-Base-QA @ 9fafd28, shared with yawbtng; PRD and implementation guide synchronized.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
-        <x:v>Activation</x:v>
+        <x:v>Architecture</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>Restore Actions; deploy 36e7ab7; prove 26 constraints, provider safeguards, exact-SHA 32/32 APIs, 81/81 routes, and tenant rejection matrix.</x:v>
+        <x:v>One hybrid journey: Stagehand adapts navigation, Playwright owns deterministic verdicts, and Browserbase provides remote browser infrastructure and evidence.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>No production row or provider was changed. Run 29216078831 was zero-step billing blocked.</x:v>
+        <x:v>Production still awaits reviewed deploy and exact-SHA Browserbase proof. Full lint and build-warning debt remain explicit future work.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -3356,81 +3356,217 @@
         <x:v>46215.99652777778</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="133"/>
-      <x:c r="B23" s="133"/>
-      <x:c r="C23" s="133"/>
-      <x:c r="D23" s="133"/>
-      <x:c r="E23" s="133"/>
-      <x:c r="F23" s="133"/>
-      <x:c r="G23" s="133"/>
-      <x:c r="H23" s="133"/>
-      <x:c r="I23" s="133"/>
-      <x:c r="J23" s="133"/>
-      <x:c r="K23" s="133"/>
-      <x:c r="L23" s="133"/>
-      <x:c r="M23" s="133"/>
-      <x:c r="N23" s="133"/>
-      <x:c r="O23" s="133"/>
-      <x:c r="P23" s="133"/>
-      <x:c r="Q23" s="165"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="133"/>
-      <x:c r="B24" s="133"/>
-      <x:c r="C24" s="133"/>
-      <x:c r="D24" s="133"/>
-      <x:c r="E24" s="133"/>
-      <x:c r="F24" s="133"/>
-      <x:c r="G24" s="133"/>
-      <x:c r="H24" s="133"/>
-      <x:c r="I24" s="133"/>
-      <x:c r="J24" s="133"/>
-      <x:c r="K24" s="133"/>
-      <x:c r="L24" s="133"/>
-      <x:c r="M24" s="133"/>
-      <x:c r="N24" s="133"/>
-      <x:c r="O24" s="133"/>
-      <x:c r="P24" s="133"/>
-      <x:c r="Q24" s="165"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="133"/>
-      <x:c r="B25" s="133"/>
-      <x:c r="C25" s="133"/>
-      <x:c r="D25" s="133"/>
-      <x:c r="E25" s="133"/>
-      <x:c r="F25" s="133"/>
-      <x:c r="G25" s="133"/>
-      <x:c r="H25" s="133"/>
-      <x:c r="I25" s="133"/>
-      <x:c r="J25" s="133"/>
-      <x:c r="K25" s="133"/>
-      <x:c r="L25" s="133"/>
-      <x:c r="M25" s="133"/>
-      <x:c r="N25" s="133"/>
-      <x:c r="O25" s="133"/>
-      <x:c r="P25" s="133"/>
-      <x:c r="Q25" s="165"/>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="133"/>
-      <x:c r="B26" s="133"/>
-      <x:c r="C26" s="133"/>
-      <x:c r="D26" s="133"/>
-      <x:c r="E26" s="133"/>
-      <x:c r="F26" s="133"/>
-      <x:c r="G26" s="133"/>
-      <x:c r="H26" s="133"/>
-      <x:c r="I26" s="133"/>
-      <x:c r="J26" s="133"/>
-      <x:c r="K26" s="133"/>
-      <x:c r="L26" s="133"/>
-      <x:c r="M26" s="133"/>
-      <x:c r="N26" s="133"/>
-      <x:c r="O26" s="133"/>
-      <x:c r="P26" s="133"/>
-      <x:c r="Q26" s="165"/>
+    <x:row r="23" ht="150" customHeight="1">
+      <x:c r="A23" s="170" t="str">
+        <x:v>T-018</x:v>
+      </x:c>
+      <x:c r="B23" s="170" t="str">
+        <x:v>Reliability</x:v>
+      </x:c>
+      <x:c r="C23" s="170" t="str">
+        <x:v>Make every direct Resend delivery retry-safe</x:v>
+      </x:c>
+      <x:c r="D23" s="170" t="str">
+        <x:v>All direct Resend email calls carry a privacy-safe deterministic idempotency key and the contract fails if a future call omits it.</x:v>
+      </x:c>
+      <x:c r="E23" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F23" s="170" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G23" s="170" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H23" s="170" t="str">
+        <x:v>Run AST coverage, focused key tests, full unit suite, server typecheck, and production build.</x:v>
+      </x:c>
+      <x:c r="I23" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="J23" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="K23" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L23" s="170" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="M23" s="170" t="str">
+        <x:v>24/24 direct calls; 4/4 key tests; 808/808 full unit</x:v>
+      </x:c>
+      <x:c r="N23" s="170" t="str">
+        <x:v>9083c93</x:v>
+      </x:c>
+      <x:c r="O23" s="170" t="str">
+        <x:v>Production proof awaits reviewed deploy.</x:v>
+      </x:c>
+      <x:c r="P23" s="170" t="str">
+        <x:v>Same logical delivery reuses a key; intentional manual resend receives a new minute-bucket key.</x:v>
+      </x:c>
+      <x:c r="Q23" s="171" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="150" customHeight="1">
+      <x:c r="A24" s="170" t="str">
+        <x:v>T-019</x:v>
+      </x:c>
+      <x:c r="B24" s="170" t="str">
+        <x:v>Quality Gate</x:v>
+      </x:c>
+      <x:c r="C24" s="170" t="str">
+        <x:v>Compile the complete frontend and server graph</x:v>
+      </x:c>
+      <x:c r="D24" s="170" t="str">
+        <x:v>The release workflow typechecks the Vite frontend and every Hono server module, with regression contracts for bugs exposed during adoption.</x:v>
+      </x:c>
+      <x:c r="E24" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F24" s="170" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G24" s="170" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H24" s="170" t="str">
+        <x:v>Run npm run typecheck, server reliability contracts, full unit suite, Guardian policy, incident tests, and Vite build.</x:v>
+      </x:c>
+      <x:c r="I24" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="J24" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="K24" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L24" s="170" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="M24" s="170" t="str">
+        <x:v>Frontend + server typecheck; 10 reliability contracts; 808/808 unit</x:v>
+      </x:c>
+      <x:c r="N24" s="170" t="str">
+        <x:v>9083c93</x:v>
+      </x:c>
+      <x:c r="O24" s="170" t="str">
+        <x:v>GitHub Actions account capacity remains separately blocked.</x:v>
+      </x:c>
+      <x:c r="P24" s="170" t="str">
+        <x:v>Caught real runtime, Stripe SDK, auth, JSON parameter, mobile role, API response, PDF, and conditional-hook defects.</x:v>
+      </x:c>
+      <x:c r="Q24" s="171" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="150" customHeight="1">
+      <x:c r="A25" s="170" t="str">
+        <x:v>T-020</x:v>
+      </x:c>
+      <x:c r="B25" s="170" t="str">
+        <x:v>Browser QA</x:v>
+      </x:c>
+      <x:c r="C25" s="170" t="str">
+        <x:v>Define and verify the hybrid Stagehand + Playwright contract</x:v>
+      </x:c>
+      <x:c r="D25" s="170" t="str">
+        <x:v>One journey uses Stagehand only for adaptable semantic navigation, Playwright for deterministic assertions, and Browserbase for remote execution and evidence; no duplicate suites.</x:v>
+      </x:c>
+      <x:c r="E25" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F25" s="170" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G25" s="170" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H25" s="170" t="str">
+        <x:v>Verify dashboard, service notification, billing, documents, SMS contacts, console health, overflow, and mobile handoff across representative sizes.</x:v>
+      </x:c>
+      <x:c r="I25" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="J25" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="K25" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L25" s="170" t="str">
+        <x:v>1440x900, 1280x800, 1024x767, 767x1024</x:v>
+      </x:c>
+      <x:c r="M25" s="170" t="str">
+        <x:v>Dashboard 4/4; service preview 3/3; billing 2/2; SMS 2/2; documents 1/1; zero console errors</x:v>
+      </x:c>
+      <x:c r="N25" s="170" t="str">
+        <x:v>9083c93; 9fafd28</x:v>
+      </x:c>
+      <x:c r="O25" s="170" t="str">
+        <x:v>Live Browserbase sessions still require project secrets/context.</x:v>
+      </x:c>
+      <x:c r="P25" s="170" t="str">
+        <x:v>Browserbase is infrastructure, Stagehand is the adaptable operator, and Playwright is the strict referee.</x:v>
+      </x:c>
+      <x:c r="Q25" s="171" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="150" customHeight="1">
+      <x:c r="A26" s="170" t="str">
+        <x:v>T-021</x:v>
+      </x:c>
+      <x:c r="B26" s="170" t="str">
+        <x:v>Debt Burn-down</x:v>
+      </x:c>
+      <x:c r="C26" s="170" t="str">
+        <x:v>Eliminate repository lint and build-warning debt</x:v>
+      </x:c>
+      <x:c r="D26" s="170" t="str">
+        <x:v>Repository-wide ESLint is green and browser build warnings are either fixed or measured with explicit budgets.</x:v>
+      </x:c>
+      <x:c r="E26" s="170" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="F26" s="170" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="G26" s="170" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="H26" s="170" t="str">
+        <x:v>Fix by bounded file family, rerun full lint, update bundle budgets, refresh browserslist data, and retain regression tests.</x:v>
+      </x:c>
+      <x:c r="I26" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="J26" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="K26" s="170" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="L26" s="170" t="str">
+        <x:v>All desktop sizes after each behavior-affecting batch</x:v>
+      </x:c>
+      <x:c r="M26" s="170" t="str">
+        <x:v>G-021; G-022</x:v>
+      </x:c>
+      <x:c r="N26" s="170" t="str">
+        <x:v>Pending future checkpoints</x:v>
+      </x:c>
+      <x:c r="O26" s="170" t="str">
+        <x:v>Large pre-existing baseline must be reduced without hiding rules or mass-changing behavior.</x:v>
+      </x:c>
+      <x:c r="P26" s="170" t="str">
+        <x:v>High-signal conditional-hook and side-effect findings in touched paths are already fixed and clean.</x:v>
+      </x:c>
+      <x:c r="Q26" s="171" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="133"/>
@@ -5288,7 +5424,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59aea61eabb34c20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d841d7e3d75456d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10629,20 +10765,225 @@
         <x:v>The red check contains no product-test verdict.</x:v>
       </x:c>
     </x:row>
-    <x:row r="124">
-      <x:c r="B124" s="164"/>
-    </x:row>
-    <x:row r="125">
-      <x:c r="B125" s="164"/>
-    </x:row>
-    <x:row r="126">
-      <x:c r="B126" s="164"/>
-    </x:row>
-    <x:row r="127">
-      <x:c r="B127" s="164"/>
-    </x:row>
-    <x:row r="128">
-      <x:c r="B128" s="164"/>
+    <x:row r="124" ht="142" customHeight="1">
+      <x:c r="A124" s="174" t="str">
+        <x:v>AL-119</x:v>
+      </x:c>
+      <x:c r="B124" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="C124" s="174" t="str">
+        <x:v>T-018</x:v>
+      </x:c>
+      <x:c r="D124" s="174" t="str">
+        <x:v>Inventory and harden all direct Resend deliveries</x:v>
+      </x:c>
+      <x:c r="E124" s="174" t="str">
+        <x:v>Traced every direct Resend API call and added deterministic, privacy-safe idempotency keys using durable record IDs or explicit manual-resend time buckets.</x:v>
+      </x:c>
+      <x:c r="F124" s="174" t="str">
+        <x:v>PestFlow server</x:v>
+      </x:c>
+      <x:c r="G124" s="174" t="str">
+        <x:v>24/24 direct calls protected</x:v>
+      </x:c>
+      <x:c r="H124" s="174" t="str">
+        <x:v>A TypeScript AST contract now fails if a future Resend call omits the inline Idempotency-Key header.</x:v>
+      </x:c>
+      <x:c r="I124" s="174" t="str">
+        <x:v>Server email paths</x:v>
+      </x:c>
+      <x:c r="J124" s="174" t="str">
+        <x:v>server/lib/resendIdempotency.ts; src/test/resendIdempotencyCoverage.test.ts</x:v>
+      </x:c>
+      <x:c r="K124" s="174" t="str">
+        <x:v>9083c93</x:v>
+      </x:c>
+      <x:c r="L124" s="174" t="str">
+        <x:v>Deploy and retain provider response IDs for live operational reconciliation.</x:v>
+      </x:c>
+      <x:c r="M124" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N124" s="174" t="str">
+        <x:v>No email or provider request was sent during implementation or validation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="142" customHeight="1">
+      <x:c r="A125" s="174" t="str">
+        <x:v>AL-120</x:v>
+      </x:c>
+      <x:c r="B125" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="C125" s="174" t="str">
+        <x:v>T-019</x:v>
+      </x:c>
+      <x:c r="D125" s="174" t="str">
+        <x:v>Adopt a full frontend and server compiler gate</x:v>
+      </x:c>
+      <x:c r="E125" s="174" t="str">
+        <x:v>Added a dedicated server tsconfig, wired both TypeScript graphs into the release workflow, and repaired the runtime and SDK defects the compiler exposed.</x:v>
+      </x:c>
+      <x:c r="F125" s="174" t="str">
+        <x:v>TypeScript + source contracts</x:v>
+      </x:c>
+      <x:c r="G125" s="174" t="str">
+        <x:v>Complete graph typechecks</x:v>
+      </x:c>
+      <x:c r="H125" s="174" t="str">
+        <x:v>Repairs include Website Chat import, Stripe embedded/session APIs, SetupIntent account options, current invoice subscription shape, SQL JSON parameters, auth narrowing, mobile role, API shapes, and PDF canvas.</x:v>
+      </x:c>
+      <x:c r="I125" s="174" t="str">
+        <x:v>Frontend + API</x:v>
+      </x:c>
+      <x:c r="J125" s="174" t="str">
+        <x:v>tsconfig.server.json; src/test/serverReliabilityContracts.test.ts; src/test/frontendReliabilityContracts.test.ts</x:v>
+      </x:c>
+      <x:c r="K125" s="174" t="str">
+        <x:v>9083c93</x:v>
+      </x:c>
+      <x:c r="L125" s="174" t="str">
+        <x:v>Keep every newly discovered runtime contract locked by focused tests.</x:v>
+      </x:c>
+      <x:c r="M125" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N125" s="174" t="str">
+        <x:v>The release workflow now rejects compile drift before browser execution.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="142" customHeight="1">
+      <x:c r="A126" s="174" t="str">
+        <x:v>AL-121</x:v>
+      </x:c>
+      <x:c r="B126" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="C126" s="174" t="str">
+        <x:v>T-019</x:v>
+      </x:c>
+      <x:c r="D126" s="174" t="str">
+        <x:v>Run the complete local reliability gate</x:v>
+      </x:c>
+      <x:c r="E126" s="174" t="str">
+        <x:v>Ran both compiler graphs, the complete unit suite, Guardian policy suite, incident suite, focused reliability contracts, production build, and high-signal touched-file lint.</x:v>
+      </x:c>
+      <x:c r="F126" s="174" t="str">
+        <x:v>Vitest + Node + TypeScript + ESLint + Vite</x:v>
+      </x:c>
+      <x:c r="G126" s="174" t="str">
+        <x:v>Branch validation passed</x:v>
+      </x:c>
+      <x:c r="H126" s="174" t="str">
+        <x:v>808/808 unit across 82 files, 48/48 Guardian policy, 16/16 incident, focused 51/51, typecheck, and 5,699-module build passed.</x:v>
+      </x:c>
+      <x:c r="I126" s="174" t="str">
+        <x:v>Code + automation</x:v>
+      </x:c>
+      <x:c r="J126" s="174" t="str">
+        <x:v>package.json; .github/workflows/desktop-qa-release-gate.yml</x:v>
+      </x:c>
+      <x:c r="K126" s="174" t="str">
+        <x:v>9083c93</x:v>
+      </x:c>
+      <x:c r="L126" s="174" t="str">
+        <x:v>Restore GitHub Actions billing/spending capacity and rerun the exact head in the cloud.</x:v>
+      </x:c>
+      <x:c r="M126" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N126" s="174" t="str">
+        <x:v>Full ESLint remains red on a quantified pre-existing baseline and is tracked separately, not mislabeled green.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="142" customHeight="1">
+      <x:c r="A127" s="174" t="str">
+        <x:v>AL-122</x:v>
+      </x:c>
+      <x:c r="B127" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="C127" s="174" t="str">
+        <x:v>T-020</x:v>
+      </x:c>
+      <x:c r="D127" s="174" t="str">
+        <x:v>Verify critical desktop surfaces in a real browser</x:v>
+      </x:c>
+      <x:c r="E127" s="174" t="str">
+        <x:v>Checked authenticated dev-mode dashboard, service notification preview, billing, documents, SMS contacts, and the mobile document handoff across representative viewport sizes.</x:v>
+      </x:c>
+      <x:c r="F127" s="174" t="str">
+        <x:v>In-app browser + Playwright assertions</x:v>
+      </x:c>
+      <x:c r="G127" s="174" t="str">
+        <x:v>12 responsive route-size checks passed</x:v>
+      </x:c>
+      <x:c r="H127" s="174" t="str">
+        <x:v>No horizontal overflow, visible runtime alert, missing primary heading, or console error was found; the document job handoff reached the field app.</x:v>
+      </x:c>
+      <x:c r="I127" s="174" t="str">
+        <x:v>1440x900, 1280x800, 1024x767, 767x1024</x:v>
+      </x:c>
+      <x:c r="J127" s="174" t="str">
+        <x:v>Local preview http://127.0.0.1:4173</x:v>
+      </x:c>
+      <x:c r="K127" s="174" t="str">
+        <x:v>9083c93</x:v>
+      </x:c>
+      <x:c r="L127" s="174" t="str">
+        <x:v>Repeat the same deterministic checks on the exact deployed SHA through Browserbase.</x:v>
+      </x:c>
+      <x:c r="M127" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N127" s="174" t="str">
+        <x:v>Viewport was reset after verification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="142" customHeight="1">
+      <x:c r="A128" s="174" t="str">
+        <x:v>AL-123</x:v>
+      </x:c>
+      <x:c r="B128" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="C128" s="174" t="str">
+        <x:v>T-020</x:v>
+      </x:c>
+      <x:c r="D128" s="174" t="str">
+        <x:v>Document the non-duplicative browser architecture</x:v>
+      </x:c>
+      <x:c r="E128" s="174" t="str">
+        <x:v>Defined one hybrid journey contract: Stagehand handles semantic/adaptive navigation, Playwright owns exact assertions and network evidence, and Browserbase hosts remote sessions and recordings.</x:v>
+      </x:c>
+      <x:c r="F128" s="174" t="str">
+        <x:v>PRD + implementation guide</x:v>
+      </x:c>
+      <x:c r="G128" s="174" t="str">
+        <x:v>Architecture clarified</x:v>
+      </x:c>
+      <x:c r="H128" s="174" t="str">
+        <x:v>The separation avoids parallel duplicate suites while retaining self-healing navigation and deterministic release verdicts.</x:v>
+      </x:c>
+      <x:c r="I128" s="174" t="str">
+        <x:v>Browser-Base-QA + PestFlow</x:v>
+      </x:c>
+      <x:c r="J128" s="174" t="str">
+        <x:v>docs/PRD.md; docs/PESTFLOW_QA_IMPLEMENTATION_GUIDE.md</x:v>
+      </x:c>
+      <x:c r="K128" s="174" t="str">
+        <x:v>9083c93; 9fafd28</x:v>
+      </x:c>
+      <x:c r="L128" s="174" t="str">
+        <x:v>Activate Browserbase secrets and run the same candidate workflow against an approved QA tenant.</x:v>
+      </x:c>
+      <x:c r="M128" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N128" s="174" t="str">
+        <x:v>Browserbase does not replace Stagehand; Stagehand runs on Browserbase and can interoperate with Playwright.</x:v>
+      </x:c>
     </x:row>
     <x:row r="129">
       <x:c r="B129" s="164"/>
@@ -10885,7 +11226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea9d7abcf6c6437a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a32453bd1d043d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14798,29 +15139,285 @@
         <x:v>Verified payment/spending refusal; no product command started.</x:v>
       </x:c>
     </x:row>
-    <x:row r="114">
-      <x:c r="I114" s="164"/>
-    </x:row>
-    <x:row r="115">
-      <x:c r="I115" s="164"/>
-    </x:row>
-    <x:row r="116">
-      <x:c r="I116" s="164"/>
-    </x:row>
-    <x:row r="117">
-      <x:c r="I117" s="164"/>
-    </x:row>
-    <x:row r="118">
-      <x:c r="I118" s="164"/>
-    </x:row>
-    <x:row r="119">
-      <x:c r="I119" s="164"/>
-    </x:row>
-    <x:row r="120">
-      <x:c r="I120" s="164"/>
-    </x:row>
-    <x:row r="121">
-      <x:c r="I121" s="164"/>
+    <x:row r="114" ht="94" customHeight="1">
+      <x:c r="A114" s="174" t="str">
+        <x:v>QA-109</x:v>
+      </x:c>
+      <x:c r="B114" s="174" t="str">
+        <x:v>Reliability</x:v>
+      </x:c>
+      <x:c r="C114" s="174" t="str">
+        <x:v>Direct Resend idempotency coverage</x:v>
+      </x:c>
+      <x:c r="D114" s="174" t="str">
+        <x:v>24 direct calls</x:v>
+      </x:c>
+      <x:c r="E114" s="174" t="str">
+        <x:v>TypeScript AST + Vitest</x:v>
+      </x:c>
+      <x:c r="F114" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G114" s="174" t="str">
+        <x:v>T-018</x:v>
+      </x:c>
+      <x:c r="H114" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I114" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="J114" s="174" t="str">
+        <x:v>24/24 calls; 4/4 key tests</x:v>
+      </x:c>
+      <x:c r="K114" s="174" t="str">
+        <x:v>Keys are stable, bounded, privacy-safe, event-isolated, and manual resend can intentionally advance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="94" customHeight="1">
+      <x:c r="A115" s="174" t="str">
+        <x:v>QA-110</x:v>
+      </x:c>
+      <x:c r="B115" s="174" t="str">
+        <x:v>Quality</x:v>
+      </x:c>
+      <x:c r="C115" s="174" t="str">
+        <x:v>Frontend and full server TypeScript graph</x:v>
+      </x:c>
+      <x:c r="D115" s="174" t="str">
+        <x:v>Vite + Hono server</x:v>
+      </x:c>
+      <x:c r="E115" s="174" t="str">
+        <x:v>tsc project references</x:v>
+      </x:c>
+      <x:c r="F115" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G115" s="174" t="str">
+        <x:v>T-019</x:v>
+      </x:c>
+      <x:c r="H115" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I115" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="J115" s="174" t="str">
+        <x:v>Both compiler graphs exited 0</x:v>
+      </x:c>
+      <x:c r="K115" s="174" t="str">
+        <x:v>Release workflow runs npm run typecheck before its later build/browser gates.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="94" customHeight="1">
+      <x:c r="A116" s="174" t="str">
+        <x:v>QA-111</x:v>
+      </x:c>
+      <x:c r="B116" s="174" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C116" s="174" t="str">
+        <x:v>Complete branch unit and policy validation</x:v>
+      </x:c>
+      <x:c r="D116" s="174" t="str">
+        <x:v>82 unit files + Guardian + incident</x:v>
+      </x:c>
+      <x:c r="E116" s="174" t="str">
+        <x:v>Vitest + Node</x:v>
+      </x:c>
+      <x:c r="F116" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G116" s="174" t="str">
+        <x:v>T-019</x:v>
+      </x:c>
+      <x:c r="H116" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I116" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="J116" s="174" t="str">
+        <x:v>808/808; 48/48; 16/16</x:v>
+      </x:c>
+      <x:c r="K116" s="174" t="str">
+        <x:v>Focused final reliability and hook suite also passed 51/51.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="94" customHeight="1">
+      <x:c r="A117" s="174" t="str">
+        <x:v>QA-112</x:v>
+      </x:c>
+      <x:c r="B117" s="174" t="str">
+        <x:v>Build</x:v>
+      </x:c>
+      <x:c r="C117" s="174" t="str">
+        <x:v>Production frontend build</x:v>
+      </x:c>
+      <x:c r="D117" s="174" t="str">
+        <x:v>5,699 modules</x:v>
+      </x:c>
+      <x:c r="E117" s="174" t="str">
+        <x:v>Vite</x:v>
+      </x:c>
+      <x:c r="F117" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G117" s="174" t="str">
+        <x:v>T-019</x:v>
+      </x:c>
+      <x:c r="H117" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I117" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="J117" s="174" t="str">
+        <x:v>Build exited 0</x:v>
+      </x:c>
+      <x:c r="K117" s="174" t="str">
+        <x:v>Bundle/dependency warnings are recorded under G-022 rather than hidden.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="94" customHeight="1">
+      <x:c r="A118" s="174" t="str">
+        <x:v>QA-113</x:v>
+      </x:c>
+      <x:c r="B118" s="174" t="str">
+        <x:v>Browser</x:v>
+      </x:c>
+      <x:c r="C118" s="174" t="str">
+        <x:v>Dashboard responsive matrix</x:v>
+      </x:c>
+      <x:c r="D118" s="174" t="str">
+        <x:v>4 sizes</x:v>
+      </x:c>
+      <x:c r="E118" s="174" t="str">
+        <x:v>In-app browser + Playwright</x:v>
+      </x:c>
+      <x:c r="F118" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G118" s="174" t="str">
+        <x:v>T-020</x:v>
+      </x:c>
+      <x:c r="H118" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I118" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="J118" s="174" t="str">
+        <x:v>4/4 sizes</x:v>
+      </x:c>
+      <x:c r="K118" s="174" t="str">
+        <x:v>1440x900, 1280x800, 1024x767, and 767x1024 had no overflow, alerts, missing heading, or hidden main.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="94" customHeight="1">
+      <x:c r="A119" s="174" t="str">
+        <x:v>QA-114</x:v>
+      </x:c>
+      <x:c r="B119" s="174" t="str">
+        <x:v>Browser</x:v>
+      </x:c>
+      <x:c r="C119" s="174" t="str">
+        <x:v>Service notification responsive preview</x:v>
+      </x:c>
+      <x:c r="D119" s="174" t="str">
+        <x:v>3 sizes</x:v>
+      </x:c>
+      <x:c r="E119" s="174" t="str">
+        <x:v>In-app browser + Playwright</x:v>
+      </x:c>
+      <x:c r="F119" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G119" s="174" t="str">
+        <x:v>T-020</x:v>
+      </x:c>
+      <x:c r="H119" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I119" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="J119" s="174" t="str">
+        <x:v>3/3 sizes + mobile handoff</x:v>
+      </x:c>
+      <x:c r="K119" s="174" t="str">
+        <x:v>Preview remained visible without overflow and job mode reached the field app.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="94" customHeight="1">
+      <x:c r="A120" s="174" t="str">
+        <x:v>QA-115</x:v>
+      </x:c>
+      <x:c r="B120" s="174" t="str">
+        <x:v>Browser</x:v>
+      </x:c>
+      <x:c r="C120" s="174" t="str">
+        <x:v>Billing, SMS Contacts, and Documents</x:v>
+      </x:c>
+      <x:c r="D120" s="174" t="str">
+        <x:v>5 route-size checks</x:v>
+      </x:c>
+      <x:c r="E120" s="174" t="str">
+        <x:v>In-app browser + Playwright</x:v>
+      </x:c>
+      <x:c r="F120" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G120" s="174" t="str">
+        <x:v>T-020</x:v>
+      </x:c>
+      <x:c r="H120" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I120" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="J120" s="174" t="str">
+        <x:v>5/5 checks; 0 console errors</x:v>
+      </x:c>
+      <x:c r="K120" s="174" t="str">
+        <x:v>Primary headings and main regions remained visible with no horizontal overflow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="94" customHeight="1">
+      <x:c r="A121" s="174" t="str">
+        <x:v>QA-116</x:v>
+      </x:c>
+      <x:c r="B121" s="174" t="str">
+        <x:v>Quality</x:v>
+      </x:c>
+      <x:c r="C121" s="174" t="str">
+        <x:v>Repository-wide ESLint baseline</x:v>
+      </x:c>
+      <x:c r="D121" s="174" t="str">
+        <x:v>Whole repository</x:v>
+      </x:c>
+      <x:c r="E121" s="174" t="str">
+        <x:v>ESLint</x:v>
+      </x:c>
+      <x:c r="F121" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G121" s="174" t="str">
+        <x:v>T-021</x:v>
+      </x:c>
+      <x:c r="H121" s="174" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="I121" s="176" t="n">
+        <x:v>46216.09027777778</x:v>
+      </x:c>
+      <x:c r="J121" s="174" t="str">
+        <x:v>617 findings: 571 errors, 46 warnings</x:v>
+      </x:c>
+      <x:c r="K121" s="174" t="str">
+        <x:v>Mostly legacy explicit-any debt; touched high-signal hook and side-effect findings were repaired and rechecked clean.</x:v>
+      </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="I122" s="164"/>
@@ -15087,7 +15684,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2687a90aa8bf4405"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re320d7a2f4f14559"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16018,6 +16615,82 @@
       </x:c>
       <x:c r="L26" s="174" t="str">
         <x:v>Branch prevention is ready. Exact production provider proof remains intentionally pending deployment and an approved test recipient.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="158" customHeight="1">
+      <x:c r="A27" s="174" t="str">
+        <x:v>G-021</x:v>
+      </x:c>
+      <x:c r="B27" s="174" t="str">
+        <x:v>T-019</x:v>
+      </x:c>
+      <x:c r="C27" s="174" t="str">
+        <x:v>Code Quality</x:v>
+      </x:c>
+      <x:c r="D27" s="174" t="str">
+        <x:v>Repository-wide ESLint currently reports 617 findings: 571 errors and 46 warnings, dominated by legacy explicit-any use across application, test, Supabase, and scratch paths.</x:v>
+      </x:c>
+      <x:c r="E27" s="174" t="str">
+        <x:v>The signal-to-noise ratio can hide newly introduced lifecycle or correctness defects and prevents lint from serving as a complete release gate.</x:v>
+      </x:c>
+      <x:c r="F27" s="174" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="G27" s="174" t="str">
+        <x:v>Burn debt down by bounded file family, preserve rules, add regression contracts for behavior changes, and require no new violations in every touched path.</x:v>
+      </x:c>
+      <x:c r="H27" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I27" s="174" t="str">
+        <x:v>T-021</x:v>
+      </x:c>
+      <x:c r="J27" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K27" s="174" t="str">
+        <x:v>Full npm run lint baseline; touched hook and side-effect findings are clean.</x:v>
+      </x:c>
+      <x:c r="L27" s="174" t="str">
+        <x:v>Do not mass-disable rules or claim the full lint gate is green until the baseline reaches zero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="158" customHeight="1">
+      <x:c r="A28" s="174" t="str">
+        <x:v>G-022</x:v>
+      </x:c>
+      <x:c r="B28" s="174" t="str">
+        <x:v>T-019</x:v>
+      </x:c>
+      <x:c r="C28" s="174" t="str">
+        <x:v>Performance / Maintenance</x:v>
+      </x:c>
+      <x:c r="D28" s="174" t="str">
+        <x:v>The production build succeeds but reports stale caniuse-lite data, a Bluebird eval warning, a dual static/dynamic service-area import, and chunks above 500 kB including a largest chunk around 722 kB.</x:v>
+      </x:c>
+      <x:c r="E28" s="174" t="str">
+        <x:v>Large bundles can slow first use on weaker connections, while stale dependency metadata and warnings make genuine build regressions harder to spot.</x:v>
+      </x:c>
+      <x:c r="F28" s="174" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="G28" s="174" t="str">
+        <x:v>Refresh browser data in a controlled dependency update, measure route-level loading, split justified large chunks, and define an explicit bundle-warning budget.</x:v>
+      </x:c>
+      <x:c r="H28" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I28" s="174" t="str">
+        <x:v>T-021</x:v>
+      </x:c>
+      <x:c r="J28" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K28" s="174" t="str">
+        <x:v>Successful Vite production build; 5,699 modules transformed.</x:v>
+      </x:c>
+      <x:c r="L28" s="174" t="str">
+        <x:v>Prioritize measured user impact and avoid speculative chunk splitting.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -16054,7 +16727,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20dbcffc68f84f02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R138c833b7ebc44ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: classify exact-head cloud gate
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R95a1032832fe4c94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="Rc49384986b034da8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R138ac5aed1b2402f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Rdcb465de143b48b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R4c26bd66d16a4f6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re5aec7267ca649c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R6de40ab798884148"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R730e3a108f564670"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Rc86c18857f064c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rf123bb31779d4a52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1343,7 +1343,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N128" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N129" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1365,7 +1365,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K121" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K122" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1767,7 +1767,7 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>116</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
@@ -1959,7 +1959,7 @@
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>Production still awaits reviewed deploy and exact-SHA Browserbase proof. Full lint and build-warning debt remain explicit future work.</x:v>
+        <x:v>Production still awaits reviewed deploy and exact-SHA Browserbase proof. Run 29219180313 was zero-step billing blocked; full lint and build-warning debt remain explicit future work.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -3288,19 +3288,19 @@
         <x:v>Authenticated API; 1440×900; 1280×800; 1024×768</x:v>
       </x:c>
       <x:c r="M21" s="170" t="str">
-        <x:v>31/32 production APIs; G-013–G-016 and G-018–G-020; 26 DB guards + provider safeguards ready; PR #89 @ 36e7ab7</x:v>
+        <x:v>31/32 production APIs; G-013–G-016 and G-018–G-022; 26 DB guards, provider safeguards, retry-safe email, and full type gate ready; PR #89 @ 9083c93</x:v>
       </x:c>
       <x:c r="N21" s="170" t="str">
-        <x:v>36e7ab7; PR #89</x:v>
+        <x:v>9083c93; PR #89</x:v>
       </x:c>
       <x:c r="O21" s="170" t="str">
-        <x:v>Needs merge/deploy authority, exact schema/provider proof, tenant rejection proof, and restored Actions.</x:v>
+        <x:v>Needs merge/deploy authority, exact production proof, tenant rejection proof, Browserbase activation, and restored Actions.</x:v>
       </x:c>
       <x:c r="P21" s="170" t="str">
-        <x:v>Full branch proof is green; current production and three historical chemical mismatches remain deliberately uncertified.</x:v>
+        <x:v>Full local proof is green; exact-head cloud run 29219180313 had zero steps; current production and three historical chemical mismatches remain deliberately uncertified.</x:v>
       </x:c>
       <x:c r="Q21" s="171" t="n">
-        <x:v>46216.03611111111</x:v>
+        <x:v>46216.095138888886</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="138" customHeight="1">
@@ -5424,7 +5424,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d841d7e3d75456d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6330540397c24514"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10985,8 +10985,49 @@
         <x:v>Browserbase does not replace Stagehand; Stagehand runs on Browserbase and can interoperate with Playwright.</x:v>
       </x:c>
     </x:row>
-    <x:row r="129">
-      <x:c r="B129" s="164"/>
+    <x:row r="129" ht="142" customHeight="1">
+      <x:c r="A129" s="174" t="str">
+        <x:v>AL-124</x:v>
+      </x:c>
+      <x:c r="B129" s="176" t="n">
+        <x:v>46216.095138888886</x:v>
+      </x:c>
+      <x:c r="C129" s="174" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="D129" s="174" t="str">
+        <x:v>Classify exact full-stack PR gate</x:v>
+      </x:c>
+      <x:c r="E129" s="174" t="str">
+        <x:v>Inspected the automatic release gate for exact PestFlow head 9083c93, verified that no command ran, and read the GitHub check annotation.</x:v>
+      </x:c>
+      <x:c r="F129" s="174" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="G129" s="174" t="str">
+        <x:v>Cloud gate blocked before execution</x:v>
+      </x:c>
+      <x:c r="H129" s="174" t="str">
+        <x:v>Run 29219180313, job 86720836158 had zero steps because recent account payments failed or the spending limit must be increased.</x:v>
+      </x:c>
+      <x:c r="I129" s="174" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="J129" s="174" t="str">
+        <x:v>https://github.com/gicheru214/pestflow-checkout-rebuild/actions/runs/29219180313</x:v>
+      </x:c>
+      <x:c r="K129" s="174" t="str">
+        <x:v>9083c93; PR #89</x:v>
+      </x:c>
+      <x:c r="L129" s="174" t="str">
+        <x:v>Restore Actions capacity and rerun the exact-head type, unit, policy, incident, build, and browser gate.</x:v>
+      </x:c>
+      <x:c r="M129" s="174" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="N129" s="174" t="str">
+        <x:v>The red check is infrastructure evidence and contains no PestFlow product-test verdict.</x:v>
+      </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="B130" s="164"/>
@@ -11226,7 +11267,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a32453bd1d043d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f63d1ce8bae4ae2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15419,8 +15460,40 @@
         <x:v>Mostly legacy explicit-any debt; touched high-signal hook and side-effect findings were repaired and rechecked clean.</x:v>
       </x:c>
     </x:row>
-    <x:row r="122">
-      <x:c r="I122" s="164"/>
+    <x:row r="122" ht="94" customHeight="1">
+      <x:c r="A122" s="174" t="str">
+        <x:v>QA-117</x:v>
+      </x:c>
+      <x:c r="B122" s="174" t="str">
+        <x:v>Infrastructure</x:v>
+      </x:c>
+      <x:c r="C122" s="174" t="str">
+        <x:v>Exact full-stack PR release gate</x:v>
+      </x:c>
+      <x:c r="D122" s="174" t="str">
+        <x:v>GitHub runner</x:v>
+      </x:c>
+      <x:c r="E122" s="174" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F122" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G122" s="174" t="str">
+        <x:v>T-011</x:v>
+      </x:c>
+      <x:c r="H122" s="174" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="I122" s="176" t="n">
+        <x:v>46216.095138888886</x:v>
+      </x:c>
+      <x:c r="J122" s="174" t="str">
+        <x:v>Run 29219180313: zero steps</x:v>
+      </x:c>
+      <x:c r="K122" s="174" t="str">
+        <x:v>Verified account payment/spending refusal; no repository command started.</x:v>
+      </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="I123" s="164"/>
@@ -15684,7 +15757,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re320d7a2f4f14559"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80dd2df3485e4d0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16727,7 +16800,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R138c833b7ebc44ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d01a971c8c34f9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record CLI and dashboard checkpoint
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re5aec7267ca649c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R6de40ab798884148"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R730e3a108f564670"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Rc86c18857f064c2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rf123bb31779d4a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R59798fea43674833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R8e37ded0f4354a37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R3f194bc07f504b29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R296366b4c6c146d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rb861ee4157af471a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1318,7 +1318,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskTrackerTable" displayName="TaskTrackerTable" ref="A5:Q26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskTrackerTable" displayName="TaskTrackerTable" ref="A5:Q28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Task ID"/>
     <x:tableColumn id="2" name="Phase"/>
@@ -1343,7 +1343,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N129" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N132" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1365,7 +1365,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K122" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K126" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1384,7 +1384,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Gap ID"/>
     <x:tableColumn id="2" name="Found During Task"/>
@@ -1699,12 +1699,12 @@
     <x:row r="5">
       <x:c r="A5" s="134" t="n">
         <x:f>COUNTA('Task Tracker'!$A$6:$A$200)</x:f>
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B5" s="135"/>
       <x:c r="C5" s="136" t="n">
         <x:f>COUNTIF('Task Tracker'!$E$6:$E$200,"Done")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D5" s="137"/>
       <x:c r="E5" s="138" t="n">
@@ -1767,12 +1767,12 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>117</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>82</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
@@ -1782,7 +1782,7 @@
       <x:c r="F9" s="141"/>
       <x:c r="G9" s="138" t="n">
         <x:f>COUNTIFS('Product Gaps'!$A$6:$A$200,"&lt;&gt;",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Closed",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Resolved",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Mitigated")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="H9" s="139"/>
     </x:row>
@@ -1941,25 +1941,25 @@
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>All 24 direct Resend deliveries are retry-safe and both TypeScript graphs are release-gated. Local unit, policy, incident, build, and browser checks pass.</x:v>
+        <x:v>Browser-Base-QA now ships one CLI and a responsive read-only dashboard over the same registry and artifact evidence; local validation is green.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ 9083c93; Browser-Base-QA @ 9fafd28, shared with yawbtng; PRD and implementation guide synchronized.</x:v>
+        <x:v>PestFlow PR #89 @ 9083c93; Browser-Base-QA @ f477538, shared with yawbtng; PRD, code guide, CLI, and dashboard are current.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
-        <x:v>Architecture</x:v>
+        <x:v>Interface</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>One hybrid journey: Stagehand adapts navigation, Playwright owns deterministic verdicts, and Browserbase provides remote browser infrastructure and evidence.</x:v>
+        <x:v>browser-base-qa runs the engine; browser-base-qa dashboard displays its evidence without launching tests or mutating PestFlow.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>Production still awaits reviewed deploy and exact-SHA Browserbase proof. Run 29219180313 was zero-step billing blocked; full lint and build-warning debt remain explicit future work.</x:v>
+        <x:v>The current dashboard is local and latest-artifact based. Durable hosted history and owner authentication are tracked under T-023 / G-023.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -3568,43 +3568,111 @@
         <x:v>46216.09027777778</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="133"/>
-      <x:c r="B27" s="133"/>
-      <x:c r="C27" s="133"/>
-      <x:c r="D27" s="133"/>
-      <x:c r="E27" s="133"/>
-      <x:c r="F27" s="133"/>
-      <x:c r="G27" s="133"/>
-      <x:c r="H27" s="133"/>
-      <x:c r="I27" s="133"/>
-      <x:c r="J27" s="133"/>
-      <x:c r="K27" s="133"/>
-      <x:c r="L27" s="133"/>
-      <x:c r="M27" s="133"/>
-      <x:c r="N27" s="133"/>
-      <x:c r="O27" s="133"/>
-      <x:c r="P27" s="133"/>
-      <x:c r="Q27" s="165"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="133"/>
-      <x:c r="B28" s="133"/>
-      <x:c r="C28" s="133"/>
-      <x:c r="D28" s="133"/>
-      <x:c r="E28" s="133"/>
-      <x:c r="F28" s="133"/>
-      <x:c r="G28" s="133"/>
-      <x:c r="H28" s="133"/>
-      <x:c r="I28" s="133"/>
-      <x:c r="J28" s="133"/>
-      <x:c r="K28" s="133"/>
-      <x:c r="L28" s="133"/>
-      <x:c r="M28" s="133"/>
-      <x:c r="N28" s="133"/>
-      <x:c r="O28" s="133"/>
-      <x:c r="P28" s="133"/>
-      <x:c r="Q28" s="165"/>
+    <x:row r="27" ht="150" customHeight="1">
+      <x:c r="A27" s="170" t="str">
+        <x:v>T-022</x:v>
+      </x:c>
+      <x:c r="B27" s="170" t="str">
+        <x:v>Product Surface</x:v>
+      </x:c>
+      <x:c r="C27" s="170" t="str">
+        <x:v>Ship one QA CLI with an artifact-backed dashboard</x:v>
+      </x:c>
+      <x:c r="D27" s="170" t="str">
+        <x:v>A single browser-base-qa command lists, plans, runs, checks oracles, calculates the verdict, and starts a responsive read-only dashboard from the same evidence.</x:v>
+      </x:c>
+      <x:c r="E27" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F27" s="170" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G27" s="170" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H27" s="170" t="str">
+        <x:v>Test command delegation and exit behavior; verify dashboard API/security; inspect desktop/mobile layout, refresh, console, and overflow.</x:v>
+      </x:c>
+      <x:c r="I27" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="J27" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="K27" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L27" s="170" t="str">
+        <x:v>1440x900 desktop; 390x844 mobile</x:v>
+      </x:c>
+      <x:c r="M27" s="170" t="str">
+        <x:v>10/10 tests; 12-entry dry run; dashboard 200/405/404; 0 browser errors</x:v>
+      </x:c>
+      <x:c r="N27" s="170" t="str">
+        <x:v>f477538</x:v>
+      </x:c>
+      <x:c r="O27" s="170" t="str">
+        <x:v>Live sessions still require Browserbase configuration.</x:v>
+      </x:c>
+      <x:c r="P27" s="170" t="str">
+        <x:v>The dashboard reads artifacts only; it does not trigger QA or mutate PestFlow.</x:v>
+      </x:c>
+      <x:c r="Q27" s="171" t="n">
+        <x:v>46216.149305555555</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="150" customHeight="1">
+      <x:c r="A28" s="170" t="str">
+        <x:v>T-023</x:v>
+      </x:c>
+      <x:c r="B28" s="170" t="str">
+        <x:v>Command Center</x:v>
+      </x:c>
+      <x:c r="C28" s="170" t="str">
+        <x:v>Add durable hosted dashboard history and owner access</x:v>
+      </x:c>
+      <x:c r="D28" s="170" t="str">
+        <x:v>Authorized owners can securely review historical runs, incidents, costs, replays, and trends without relying on one machine's artifact folder.</x:v>
+      </x:c>
+      <x:c r="E28" s="170" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="F28" s="170" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="G28" s="170" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="H28" s="170" t="str">
+        <x:v>Design the durable run schema and auth boundary, import current artifacts, add retention/redaction policy, then test tenant and role isolation.</x:v>
+      </x:c>
+      <x:c r="I28" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="J28" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="K28" s="170" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="L28" s="170" t="str">
+        <x:v>Desktop, tablet, and mobile before launch</x:v>
+      </x:c>
+      <x:c r="M28" s="170" t="str">
+        <x:v>G-023; local dashboard foundation @ f477538</x:v>
+      </x:c>
+      <x:c r="N28" s="170" t="str">
+        <x:v>Pending future checkpoint</x:v>
+      </x:c>
+      <x:c r="O28" s="170" t="str">
+        <x:v>Needs hosting, storage, authentication, retention, and operating-cost decisions.</x:v>
+      </x:c>
+      <x:c r="P28" s="170" t="str">
+        <x:v>Do not add remote mutation controls until read-only ownership and auditability are proven.</x:v>
+      </x:c>
+      <x:c r="Q28" s="171" t="n">
+        <x:v>46216.149305555555</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="133"/>
@@ -5424,7 +5492,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6330540397c24514"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re38af253df3a42a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11029,14 +11097,137 @@
         <x:v>The red check is infrastructure evidence and contains no PestFlow product-test verdict.</x:v>
       </x:c>
     </x:row>
-    <x:row r="130">
-      <x:c r="B130" s="164"/>
-    </x:row>
-    <x:row r="131">
-      <x:c r="B131" s="164"/>
-    </x:row>
-    <x:row r="132">
-      <x:c r="B132" s="164"/>
+    <x:row r="130" ht="142" customHeight="1">
+      <x:c r="A130" s="174" t="str">
+        <x:v>AL-125</x:v>
+      </x:c>
+      <x:c r="B130" s="176" t="n">
+        <x:v>46216.149305555555</x:v>
+      </x:c>
+      <x:c r="C130" s="174" t="str">
+        <x:v>T-022</x:v>
+      </x:c>
+      <x:c r="D130" s="174" t="str">
+        <x:v>Unify the QA command surface</x:v>
+      </x:c>
+      <x:c r="E130" s="174" t="str">
+        <x:v>Added the browser-base-qa executable with list, plan, run, oracles, verdict, and dashboard subcommands while preserving each guarded program's exit code.</x:v>
+      </x:c>
+      <x:c r="F130" s="174" t="str">
+        <x:v>Node CLI</x:v>
+      </x:c>
+      <x:c r="G130" s="174" t="str">
+        <x:v>One operational entry point</x:v>
+      </x:c>
+      <x:c r="H130" s="174" t="str">
+        <x:v>Command help, command-specific help, tier filtering, dry-run selection, packaging, and executable permissions were verified.</x:v>
+      </x:c>
+      <x:c r="I130" s="174" t="str">
+        <x:v>Local + package</x:v>
+      </x:c>
+      <x:c r="J130" s="174" t="str">
+        <x:v>bin/browser-base-qa.mjs; package.json</x:v>
+      </x:c>
+      <x:c r="K130" s="174" t="str">
+        <x:v>f477538</x:v>
+      </x:c>
+      <x:c r="L130" s="174" t="str">
+        <x:v>Use the same command from CI and operator runbooks instead of maintaining shell-specific aliases.</x:v>
+      </x:c>
+      <x:c r="M130" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N130" s="174" t="str">
+        <x:v>The CLI delegates to existing policy-enforced programs rather than cloning their logic.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="142" customHeight="1">
+      <x:c r="A131" s="174" t="str">
+        <x:v>AL-126</x:v>
+      </x:c>
+      <x:c r="B131" s="176" t="n">
+        <x:v>46216.149305555555</x:v>
+      </x:c>
+      <x:c r="C131" s="174" t="str">
+        <x:v>T-022</x:v>
+      </x:c>
+      <x:c r="D131" s="174" t="str">
+        <x:v>Build the local Reliability Command Center dashboard</x:v>
+      </x:c>
+      <x:c r="E131" s="174" t="str">
+        <x:v>Added a localhost-only responsive dashboard that normalizes registry and artifact evidence into release readiness, blockers, coverage, journeys, oracles, replays, and registry views.</x:v>
+      </x:c>
+      <x:c r="F131" s="174" t="str">
+        <x:v>Read-only dashboard</x:v>
+      </x:c>
+      <x:c r="G131" s="174" t="str">
+        <x:v>Artifact-backed UI operational</x:v>
+      </x:c>
+      <x:c r="H131" s="174" t="str">
+        <x:v>The server rejects non-GET requests, exposes only normalized fields, redacts secret-like text, allowlists Browserbase replay domains, and sets strict browser security headers.</x:v>
+      </x:c>
+      <x:c r="I131" s="174" t="str">
+        <x:v>Desktop + mobile</x:v>
+      </x:c>
+      <x:c r="J131" s="174" t="str">
+        <x:v>dashboard/; scripts/qa-dashboard-server.mjs; scripts/lib/qa-dashboard-model.mjs</x:v>
+      </x:c>
+      <x:c r="K131" s="174" t="str">
+        <x:v>f477538</x:v>
+      </x:c>
+      <x:c r="L131" s="174" t="str">
+        <x:v>Add durable hosted history only after owner auth, storage, and retention contracts are approved.</x:v>
+      </x:c>
+      <x:c r="M131" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N131" s="174" t="str">
+        <x:v>Refresh reads current evidence every 15 seconds but never reruns tests or writes to PestFlow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="142" customHeight="1">
+      <x:c r="A132" s="174" t="str">
+        <x:v>AL-127</x:v>
+      </x:c>
+      <x:c r="B132" s="176" t="n">
+        <x:v>46216.149305555555</x:v>
+      </x:c>
+      <x:c r="C132" s="174" t="str">
+        <x:v>T-022</x:v>
+      </x:c>
+      <x:c r="D132" s="174" t="str">
+        <x:v>Validate, document, and publish CLI plus dashboard</x:v>
+      </x:c>
+      <x:c r="E132" s="174" t="str">
+        <x:v>Ran the full repository tests, CLI list/dry-run, audit threshold, package manifest check, dashboard HTTP contracts, and real-browser desktop/mobile verification; updated README, PRD, and code guides.</x:v>
+      </x:c>
+      <x:c r="F132" s="174" t="str">
+        <x:v>Node + browser + GitHub</x:v>
+      </x:c>
+      <x:c r="G132" s="174" t="str">
+        <x:v>CLI/dashboard checkpoint published</x:v>
+      </x:c>
+      <x:c r="H132" s="174" t="str">
+        <x:v>10/10 tests passed; tier-1 dry run selected 12 entries; package contained 38 files; dashboard rendered 6 metrics and 5 registry rows with no overflow or console errors.</x:v>
+      </x:c>
+      <x:c r="I132" s="174" t="str">
+        <x:v>1440x900; 390x844</x:v>
+      </x:c>
+      <x:c r="J132" s="174" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA</x:v>
+      </x:c>
+      <x:c r="K132" s="174" t="str">
+        <x:v>f477538</x:v>
+      </x:c>
+      <x:c r="L132" s="174" t="str">
+        <x:v>Record this checkpoint in the shared tracker and continue with T-023 only after product decisions.</x:v>
+      </x:c>
+      <x:c r="M132" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N132" s="174" t="str">
+        <x:v>npm audit remained below the moderate blocking threshold; 19 low Stagehand transitive advisories remain documented.</x:v>
+      </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="B133" s="164"/>
@@ -11267,7 +11458,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f63d1ce8bae4ae2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2490f85433a94c93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15495,17 +15686,145 @@
         <x:v>Verified account payment/spending refusal; no repository command started.</x:v>
       </x:c>
     </x:row>
-    <x:row r="123">
-      <x:c r="I123" s="164"/>
-    </x:row>
-    <x:row r="124">
-      <x:c r="I124" s="164"/>
-    </x:row>
-    <x:row r="125">
-      <x:c r="I125" s="164"/>
-    </x:row>
-    <x:row r="126">
-      <x:c r="I126" s="164"/>
+    <x:row r="123" ht="100" customHeight="1">
+      <x:c r="A123" s="174" t="str">
+        <x:v>QA-118</x:v>
+      </x:c>
+      <x:c r="B123" s="174" t="str">
+        <x:v>CLI</x:v>
+      </x:c>
+      <x:c r="C123" s="174" t="str">
+        <x:v>Unified command delegation and safety</x:v>
+      </x:c>
+      <x:c r="D123" s="174" t="str">
+        <x:v>6 commands + help</x:v>
+      </x:c>
+      <x:c r="E123" s="174" t="str">
+        <x:v>Node test</x:v>
+      </x:c>
+      <x:c r="F123" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G123" s="174" t="str">
+        <x:v>T-022</x:v>
+      </x:c>
+      <x:c r="H123" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I123" s="176" t="n">
+        <x:v>46216.149305555555</x:v>
+      </x:c>
+      <x:c r="J123" s="174" t="str">
+        <x:v>4 focused CLI/dashboard tests; 10/10 full</x:v>
+      </x:c>
+      <x:c r="K123" s="174" t="str">
+        <x:v>Help, guarded list delegation, secret redaction, and replay-domain allowlisting passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="100" customHeight="1">
+      <x:c r="A124" s="174" t="str">
+        <x:v>QA-119</x:v>
+      </x:c>
+      <x:c r="B124" s="174" t="str">
+        <x:v>CLI</x:v>
+      </x:c>
+      <x:c r="C124" s="174" t="str">
+        <x:v>Guardian selection through unified command</x:v>
+      </x:c>
+      <x:c r="D124" s="174" t="str">
+        <x:v>Tier 0 + tier 1</x:v>
+      </x:c>
+      <x:c r="E124" s="174" t="str">
+        <x:v>Node CLI</x:v>
+      </x:c>
+      <x:c r="F124" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G124" s="174" t="str">
+        <x:v>T-022</x:v>
+      </x:c>
+      <x:c r="H124" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I124" s="176" t="n">
+        <x:v>46216.149305555555</x:v>
+      </x:c>
+      <x:c r="J124" s="174" t="str">
+        <x:v>4 tier-0 entries; 12 tier-1 entries</x:v>
+      </x:c>
+      <x:c r="K124" s="174" t="str">
+        <x:v>Both list and dry-run returned valid registry-backed JSON without opening Browserbase.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="100" customHeight="1">
+      <x:c r="A125" s="174" t="str">
+        <x:v>QA-120</x:v>
+      </x:c>
+      <x:c r="B125" s="174" t="str">
+        <x:v>Dashboard</x:v>
+      </x:c>
+      <x:c r="C125" s="174" t="str">
+        <x:v>Dashboard API, method, path, and package contracts</x:v>
+      </x:c>
+      <x:c r="D125" s="174" t="str">
+        <x:v>Local server + npm package</x:v>
+      </x:c>
+      <x:c r="E125" s="174" t="str">
+        <x:v>curl + npm pack</x:v>
+      </x:c>
+      <x:c r="F125" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G125" s="174" t="str">
+        <x:v>T-022</x:v>
+      </x:c>
+      <x:c r="H125" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I125" s="176" t="n">
+        <x:v>46216.149305555555</x:v>
+      </x:c>
+      <x:c r="J125" s="174" t="str">
+        <x:v>200 model; 405 POST; 404 unknown; 38 package files</x:v>
+      </x:c>
+      <x:c r="K125" s="174" t="str">
+        <x:v>The package includes the executable, dashboard assets, model, and server.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="100" customHeight="1">
+      <x:c r="A126" s="174" t="str">
+        <x:v>QA-121</x:v>
+      </x:c>
+      <x:c r="B126" s="174" t="str">
+        <x:v>Browser</x:v>
+      </x:c>
+      <x:c r="C126" s="174" t="str">
+        <x:v>Dashboard responsive and refresh behavior</x:v>
+      </x:c>
+      <x:c r="D126" s="174" t="str">
+        <x:v>Desktop + mobile</x:v>
+      </x:c>
+      <x:c r="E126" s="174" t="str">
+        <x:v>In-app browser + Playwright</x:v>
+      </x:c>
+      <x:c r="F126" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G126" s="174" t="str">
+        <x:v>T-022</x:v>
+      </x:c>
+      <x:c r="H126" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I126" s="176" t="n">
+        <x:v>46216.149305555555</x:v>
+      </x:c>
+      <x:c r="J126" s="174" t="str">
+        <x:v>2/2 sizes; refresh changed timestamp; 0 console errors</x:v>
+      </x:c>
+      <x:c r="K126" s="174" t="str">
+        <x:v>1440x900 and 390x844 showed readiness, blockers, six metrics, five registry journeys, no horizontal overflow, and a working refresh.</x:v>
+      </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="I127" s="164"/>
@@ -15757,7 +16076,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80dd2df3485e4d0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fea4dbefc734293"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16764,6 +17083,44 @@
       </x:c>
       <x:c r="L28" s="174" t="str">
         <x:v>Prioritize measured user impact and avoid speculative chunk splitting.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="164" customHeight="1">
+      <x:c r="A29" s="174" t="str">
+        <x:v>G-023</x:v>
+      </x:c>
+      <x:c r="B29" s="174" t="str">
+        <x:v>T-022</x:v>
+      </x:c>
+      <x:c r="C29" s="174" t="str">
+        <x:v>Command Center Platform</x:v>
+      </x:c>
+      <x:c r="D29" s="174" t="str">
+        <x:v>The new dashboard reads the latest local artifact files and has no durable run database, hosted owner authentication, historical incident timeline, cost history, or remote retention service.</x:v>
+      </x:c>
+      <x:c r="E29" s="174" t="str">
+        <x:v>A reviewer can inspect the current machine's evidence clearly, but cannot yet compare releases over time or safely share an authenticated hosted view with the team.</x:v>
+      </x:c>
+      <x:c r="F29" s="174" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="G29" s="174" t="str">
+        <x:v>Keep the current dashboard read-only, design the durable schema and owner-auth boundary, import normalized artifacts, define retention/redaction, then add historical and trend views.</x:v>
+      </x:c>
+      <x:c r="H29" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I29" s="174" t="str">
+        <x:v>T-023</x:v>
+      </x:c>
+      <x:c r="J29" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K29" s="174" t="str">
+        <x:v>Responsive local dashboard and normalized artifact API published at f477538.</x:v>
+      </x:c>
+      <x:c r="L29" s="174" t="str">
+        <x:v>This is a deliberate phase boundary, not a missing local feature; hosting decisions must precede remote access.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -16800,7 +17157,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d01a971c8c34f9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13fb3d71db7244e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record AADP checkpoint
</commit_message>
<xml_diff>
--- a/tracker/Browser-Base-QA-Activity-Tracker.xlsx
+++ b/tracker/Browser-Base-QA-Activity-Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R59798fea43674833"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="R8e37ded0f4354a37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R3f194bc07f504b29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="R296366b4c6c146d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="Rb861ee4157af471a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0d08986038814cbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="2" r:id="Rd40ddf5d083f46eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity Log" sheetId="3" r:id="R7b4934f2a4d14694"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Matrix" sheetId="4" r:id="Rae1d4cf4ccee464e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Gaps" sheetId="5" r:id="R11fed2b9399a428a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1318,7 +1318,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskTrackerTable" displayName="TaskTrackerTable" ref="A5:Q28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TaskTrackerTable" displayName="TaskTrackerTable" ref="A5:Q30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Task ID"/>
     <x:tableColumn id="2" name="Phase"/>
@@ -1343,7 +1343,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N132" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ActivityLogTable" displayName="ActivityLogTable" ref="A5:N135" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Log ID"/>
     <x:tableColumn id="2" name="Timestamp"/>
@@ -1365,7 +1365,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K126" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QAMatrixTable" displayName="QAMatrixTable" ref="A5:K129" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="QA ID"/>
     <x:tableColumn id="2" name="Device Class"/>
@@ -1384,7 +1384,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductGapsTable" displayName="ProductGapsTable" ref="A5:L30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Gap ID"/>
     <x:tableColumn id="2" name="Found During Task"/>
@@ -1699,12 +1699,12 @@
     <x:row r="5">
       <x:c r="A5" s="134" t="n">
         <x:f>COUNTA('Task Tracker'!$A$6:$A$200)</x:f>
-        <x:v>23</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B5" s="135"/>
       <x:c r="C5" s="136" t="n">
         <x:f>COUNTIF('Task Tracker'!$E$6:$E$200,"Done")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D5" s="137"/>
       <x:c r="E5" s="138" t="n">
@@ -1767,12 +1767,12 @@
     <x:row r="9">
       <x:c r="A9" s="134" t="n">
         <x:f>COUNTA('QA Matrix'!$A$6:$A$200)</x:f>
-        <x:v>121</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B9" s="135"/>
       <x:c r="C9" s="136" t="n">
         <x:f>COUNTIF('QA Matrix'!$H$6:$H$200,"Passed")</x:f>
-        <x:v>86</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="D9" s="137"/>
       <x:c r="E9" s="140" t="n">
@@ -1782,7 +1782,7 @@
       <x:c r="F9" s="141"/>
       <x:c r="G9" s="138" t="n">
         <x:f>COUNTIFS('Product Gaps'!$A$6:$A$200,"&lt;&gt;",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Closed",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Resolved",'Product Gaps'!$H$6:$H$200,"&lt;&gt;Mitigated")</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="H9" s="139"/>
     </x:row>
@@ -1936,30 +1936,30 @@
         <x:v>Product failures and infrastructure failures stay separate.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="162" customHeight="1">
+    <x:row r="17" ht="174" customHeight="1">
       <x:c r="A17" s="120" t="str">
         <x:v>Current</x:v>
       </x:c>
       <x:c r="B17" s="121" t="str">
-        <x:v>Browser-Base-QA now ships one CLI and a responsive read-only dashboard over the same registry and artifact evidence; local validation is green.</x:v>
+        <x:v>Browser-Base-QA now enforces Adaptive Action -&gt; Deterministic Proof (AADP): every Stagehand act must immediately pass independent Playwright proof or the journey fails.</x:v>
       </x:c>
       <x:c r="C17" s="121" t="str">
         <x:v>Repositories</x:v>
       </x:c>
       <x:c r="D17" s="121" t="str">
-        <x:v>PestFlow PR #89 @ 9083c93; Browser-Base-QA @ f477538, shared with yawbtng; PRD, code guide, CLI, and dashboard are current.</x:v>
+        <x:v>PestFlow PR #89 @ 9083c93; Browser-Base-QA @ 0e52316, shared with yawbtng; PRD, engine, tests, CLI, and dashboard are current.</x:v>
       </x:c>
       <x:c r="E17" s="121" t="str">
         <x:v>Interface</x:v>
       </x:c>
       <x:c r="F17" s="121" t="str">
-        <x:v>browser-base-qa runs the engine; browser-base-qa dashboard displays its evidence without launching tests or mutating PestFlow.</x:v>
+        <x:v>Stagehand finds and operates changing UI; Playwright proves URL, visible/value state, HTTP/API outcome, and console/network health.</x:v>
       </x:c>
       <x:c r="G17" s="121" t="str">
         <x:v>Review</x:v>
       </x:c>
       <x:c r="H17" s="122" t="str">
-        <x:v>The current dashboard is local and latest-artifact based. Durable hosted history and owner authentication are tracked under T-023 / G-023.</x:v>
+        <x:v>The engine contract is complete and green. The first approved live write-enabled journey remains T-025 / G-024; durable hosted history remains T-023 / G-023.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -3674,43 +3674,111 @@
         <x:v>46216.149305555555</x:v>
       </x:c>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="133"/>
-      <x:c r="B29" s="133"/>
-      <x:c r="C29" s="133"/>
-      <x:c r="D29" s="133"/>
-      <x:c r="E29" s="133"/>
-      <x:c r="F29" s="133"/>
-      <x:c r="G29" s="133"/>
-      <x:c r="H29" s="133"/>
-      <x:c r="I29" s="133"/>
-      <x:c r="J29" s="133"/>
-      <x:c r="K29" s="133"/>
-      <x:c r="L29" s="133"/>
-      <x:c r="M29" s="133"/>
-      <x:c r="N29" s="133"/>
-      <x:c r="O29" s="133"/>
-      <x:c r="P29" s="133"/>
-      <x:c r="Q29" s="165"/>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="133"/>
-      <x:c r="B30" s="133"/>
-      <x:c r="C30" s="133"/>
-      <x:c r="D30" s="133"/>
-      <x:c r="E30" s="133"/>
-      <x:c r="F30" s="133"/>
-      <x:c r="G30" s="133"/>
-      <x:c r="H30" s="133"/>
-      <x:c r="I30" s="133"/>
-      <x:c r="J30" s="133"/>
-      <x:c r="K30" s="133"/>
-      <x:c r="L30" s="133"/>
-      <x:c r="M30" s="133"/>
-      <x:c r="N30" s="133"/>
-      <x:c r="O30" s="133"/>
-      <x:c r="P30" s="133"/>
-      <x:c r="Q30" s="165"/>
+    <x:row r="29" ht="160" customHeight="1">
+      <x:c r="A29" s="170" t="str">
+        <x:v>T-024</x:v>
+      </x:c>
+      <x:c r="B29" s="170" t="str">
+        <x:v>Reliability</x:v>
+      </x:c>
+      <x:c r="C29" s="170" t="str">
+        <x:v>Enforce Adaptive Action -&gt; Deterministic Proof (AADP)</x:v>
+      </x:c>
+      <x:c r="D29" s="170" t="str">
+        <x:v>Every Stagehand act is rejected unless it declares and immediately passes objective Playwright proof: URL, visible/value state, first-party HTTP response, or follow-up API contract, plus console and network failure budgets.</x:v>
+      </x:c>
+      <x:c r="E29" s="170" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="F29" s="170" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G29" s="170" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="H29" s="170" t="str">
+        <x:v>Validate the registry fail-closed behavior, proof-signal execution, write-safety requirements, full test suite, tier-1 dry run, documentation, and package audit threshold.</x:v>
+      </x:c>
+      <x:c r="I29" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="J29" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="K29" s="170" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L29" s="170" t="str">
+        <x:v>N/A - engine and contract validation</x:v>
+      </x:c>
+      <x:c r="M29" s="170" t="str">
+        <x:v>4/4 focused AADP tests; 14/14 full tests; 12-entry tier-1 dry run</x:v>
+      </x:c>
+      <x:c r="N29" s="170" t="str">
+        <x:v>0e52316</x:v>
+      </x:c>
+      <x:c r="O29" s="170" t="str">
+        <x:v>No approved live write-enabled journey is registered yet; activation is tracked by T-025 / G-024.</x:v>
+      </x:c>
+      <x:c r="P29" s="170" t="str">
+        <x:v>Stagehand chooses and operates resiliently; Playwright independently decides whether the requested outcome actually happened.</x:v>
+      </x:c>
+      <x:c r="Q29" s="171" t="n">
+        <x:v>46216.17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="160" customHeight="1">
+      <x:c r="A30" s="170" t="str">
+        <x:v>T-025</x:v>
+      </x:c>
+      <x:c r="B30" s="170" t="str">
+        <x:v>Reliability</x:v>
+      </x:c>
+      <x:c r="C30" s="170" t="str">
+        <x:v>Activate the first safe AADP write journey</x:v>
+      </x:c>
+      <x:c r="D30" s="170" t="str">
+        <x:v>A high-value isolated QA-tenant workflow uses Stagehand to perform the UI action and AADP to prove the saved system-of-record outcome repeatedly, with idempotency, cleanup, and no customer impact.</x:v>
+      </x:c>
+      <x:c r="E30" s="170" t="str">
+        <x:v>Not Started</x:v>
+      </x:c>
+      <x:c r="F30" s="170" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G30" s="170" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="H30" s="170" t="str">
+        <x:v>Select one reversible workflow; approve the QA tenant and allowlists; define response/API proof and cleanup; run multiple Browserbase sessions; review evidence before scheduling.</x:v>
+      </x:c>
+      <x:c r="I30" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="J30" s="170" t="str">
+        <x:v>Not Needed</x:v>
+      </x:c>
+      <x:c r="K30" s="170" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="L30" s="170" t="str">
+        <x:v>1440, 1280, 1024, and 390 before scheduling</x:v>
+      </x:c>
+      <x:c r="M30" s="170" t="str">
+        <x:v>G-024; AADP engine @ 0e52316</x:v>
+      </x:c>
+      <x:c r="N30" s="170" t="str">
+        <x:v>Pending activation checkpoint</x:v>
+      </x:c>
+      <x:c r="O30" s="170" t="str">
+        <x:v>Requires Browserbase credentials/context plus an approved isolated QA tenant and reversible write policy.</x:v>
+      </x:c>
+      <x:c r="P30" s="170" t="str">
+        <x:v>Recommended first target: create a disposable QA customer/job, prove the saved record through the API, then clean it up.</x:v>
+      </x:c>
+      <x:c r="Q30" s="171" t="n">
+        <x:v>46216.17</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="133"/>
@@ -5492,7 +5560,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re38af253df3a42a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc72f2e81c85d4a6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11229,14 +11297,137 @@
         <x:v>npm audit remained below the moderate blocking threshold; 19 low Stagehand transitive advisories remain documented.</x:v>
       </x:c>
     </x:row>
-    <x:row r="133">
-      <x:c r="B133" s="164"/>
-    </x:row>
-    <x:row r="134">
-      <x:c r="B134" s="164"/>
-    </x:row>
-    <x:row r="135">
-      <x:c r="B135" s="164"/>
+    <x:row r="133" ht="150" customHeight="1">
+      <x:c r="A133" s="174" t="str">
+        <x:v>AL-128</x:v>
+      </x:c>
+      <x:c r="B133" s="176" t="n">
+        <x:v>46216.17</x:v>
+      </x:c>
+      <x:c r="C133" s="174" t="str">
+        <x:v>T-024</x:v>
+      </x:c>
+      <x:c r="D133" s="174" t="str">
+        <x:v>Audit the Stagehand and Playwright responsibility split</x:v>
+      </x:c>
+      <x:c r="E133" s="174" t="str">
+        <x:v>Confirmed the existing runner used Stagehand for semantic observation and Playwright for exact navigation, status, and API checks, but did not require proof immediately after every future Stagehand act.</x:v>
+      </x:c>
+      <x:c r="F133" s="174" t="str">
+        <x:v>Code + PRD audit</x:v>
+      </x:c>
+      <x:c r="G133" s="174" t="str">
+        <x:v>Partial capability identified</x:v>
+      </x:c>
+      <x:c r="H133" s="174" t="str">
+        <x:v>Mapped the act runner, registry policy, navigation assertions, owner API contracts, console capture, and network capture before changing the contract.</x:v>
+      </x:c>
+      <x:c r="I133" s="174" t="str">
+        <x:v>Browser-Base-QA</x:v>
+      </x:c>
+      <x:c r="J133" s="174" t="str">
+        <x:v>scripts/qa-guardian-stagehand.mjs; scripts/lib/qa-guardian-policy.mjs; docs/PRD.md</x:v>
+      </x:c>
+      <x:c r="K133" s="174" t="str">
+        <x:v>0e52316</x:v>
+      </x:c>
+      <x:c r="L133" s="174" t="str">
+        <x:v>Create one named fail-closed contract rather than relying on an implied convention.</x:v>
+      </x:c>
+      <x:c r="M133" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N133" s="174" t="str">
+        <x:v>The gap was enforcement and evidence coupling, not the absence of both tools.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" ht="150" customHeight="1">
+      <x:c r="A134" s="174" t="str">
+        <x:v>AL-129</x:v>
+      </x:c>
+      <x:c r="B134" s="176" t="n">
+        <x:v>46216.17</x:v>
+      </x:c>
+      <x:c r="C134" s="174" t="str">
+        <x:v>T-024</x:v>
+      </x:c>
+      <x:c r="D134" s="174" t="str">
+        <x:v>Implement Adaptive Action -&gt; Deterministic Proof</x:v>
+      </x:c>
+      <x:c r="E134" s="174" t="str">
+        <x:v>Added a reusable AADP validator/verifier, required the execution contract in the registry, and made every act step fail before browser launch when proof is missing or unsafe.</x:v>
+      </x:c>
+      <x:c r="F134" s="174" t="str">
+        <x:v>Node + Stagehand + Playwright</x:v>
+      </x:c>
+      <x:c r="G134" s="174" t="str">
+        <x:v>AADP enforced</x:v>
+      </x:c>
+      <x:c r="H134" s="174" t="str">
+        <x:v>Proof supports exact/prefix URL, visible text/value, first-party method/path/status, authenticated GET API shape, and critical console/network budgets; write-enabled actions require response or API proof.</x:v>
+      </x:c>
+      <x:c r="I134" s="174" t="str">
+        <x:v>Master QA engine</x:v>
+      </x:c>
+      <x:c r="J134" s="174" t="str">
+        <x:v>scripts/lib/qa-adaptive-action-proof.mjs; qa/guardian/desktop-journeys.json</x:v>
+      </x:c>
+      <x:c r="K134" s="174" t="str">
+        <x:v>0e52316</x:v>
+      </x:c>
+      <x:c r="L134" s="174" t="str">
+        <x:v>Add approved proof declarations to each new act journey and never accept Stagehand success alone.</x:v>
+      </x:c>
+      <x:c r="M134" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N134" s="174" t="str">
+        <x:v>Evidence retains normalized metadata only; response bodies and URL queries are not stored.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="150" customHeight="1">
+      <x:c r="A135" s="174" t="str">
+        <x:v>AL-130</x:v>
+      </x:c>
+      <x:c r="B135" s="176" t="n">
+        <x:v>46216.17</x:v>
+      </x:c>
+      <x:c r="C135" s="174" t="str">
+        <x:v>T-024</x:v>
+      </x:c>
+      <x:c r="D135" s="174" t="str">
+        <x:v>Validate, document, and publish AADP</x:v>
+      </x:c>
+      <x:c r="E135" s="174" t="str">
+        <x:v>Added focused tests and updated the PRD, README, implementation guide, and codebase guide, then committed and pushed the contract to the shared Browser-Base-QA main branch.</x:v>
+      </x:c>
+      <x:c r="F135" s="174" t="str">
+        <x:v>Node + GitHub</x:v>
+      </x:c>
+      <x:c r="G135" s="174" t="str">
+        <x:v>AADP checkpoint published</x:v>
+      </x:c>
+      <x:c r="H135" s="174" t="str">
+        <x:v>4/4 focused tests passed; 14/14 full tests passed; the tier-1 registry dry run selected 12 valid entries; syntax and diff checks passed; audit stayed below the moderate threshold.</x:v>
+      </x:c>
+      <x:c r="I135" s="174" t="str">
+        <x:v>Local deterministic validation</x:v>
+      </x:c>
+      <x:c r="J135" s="174" t="str">
+        <x:v>https://github.com/gicheru214/Browser-Base-QA</x:v>
+      </x:c>
+      <x:c r="K135" s="174" t="str">
+        <x:v>0e52316</x:v>
+      </x:c>
+      <x:c r="L135" s="174" t="str">
+        <x:v>Activate T-025 only with Browserbase configuration and an approved disposable QA tenant.</x:v>
+      </x:c>
+      <x:c r="M135" s="174" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="N135" s="174" t="str">
+        <x:v>The existing 19 low Stagehand transitive advisories remain; no live write-enabled journey was claimed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="136">
       <x:c r="B136" s="164"/>
@@ -11458,7 +11649,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2490f85433a94c93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raba764bb212d468f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15826,14 +16017,110 @@
         <x:v>1440x900 and 390x844 showed readiness, blockers, six metrics, five registry journeys, no horizontal overflow, and a working refresh.</x:v>
       </x:c>
     </x:row>
-    <x:row r="127">
-      <x:c r="I127" s="164"/>
-    </x:row>
-    <x:row r="128">
-      <x:c r="I128" s="164"/>
-    </x:row>
-    <x:row r="129">
-      <x:c r="I129" s="164"/>
+    <x:row r="127" ht="110" customHeight="1">
+      <x:c r="A127" s="174" t="str">
+        <x:v>QA-122</x:v>
+      </x:c>
+      <x:c r="B127" s="174" t="str">
+        <x:v>Contract</x:v>
+      </x:c>
+      <x:c r="C127" s="174" t="str">
+        <x:v>AADP validation and fail-closed policy</x:v>
+      </x:c>
+      <x:c r="D127" s="174" t="str">
+        <x:v>4 focused cases</x:v>
+      </x:c>
+      <x:c r="E127" s="174" t="str">
+        <x:v>Node test</x:v>
+      </x:c>
+      <x:c r="F127" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G127" s="174" t="str">
+        <x:v>T-024</x:v>
+      </x:c>
+      <x:c r="H127" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I127" s="176" t="n">
+        <x:v>46216.17</x:v>
+      </x:c>
+      <x:c r="J127" s="174" t="str">
+        <x:v>4/4 passed</x:v>
+      </x:c>
+      <x:c r="K127" s="174" t="str">
+        <x:v>Covered successful composite proof, console-error failure, missing-proof registry rejection, and write actions without response/API proof.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="110" customHeight="1">
+      <x:c r="A128" s="174" t="str">
+        <x:v>QA-123</x:v>
+      </x:c>
+      <x:c r="B128" s="174" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="C128" s="174" t="str">
+        <x:v>Master QA repository test suite after AADP</x:v>
+      </x:c>
+      <x:c r="D128" s="174" t="str">
+        <x:v>Full local suite</x:v>
+      </x:c>
+      <x:c r="E128" s="174" t="str">
+        <x:v>Node test</x:v>
+      </x:c>
+      <x:c r="F128" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G128" s="174" t="str">
+        <x:v>T-024</x:v>
+      </x:c>
+      <x:c r="H128" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I128" s="176" t="n">
+        <x:v>46216.17</x:v>
+      </x:c>
+      <x:c r="J128" s="174" t="str">
+        <x:v>14/14 passed</x:v>
+      </x:c>
+      <x:c r="K128" s="174" t="str">
+        <x:v>The new AADP tests and all prior policy, CLI, and dashboard contracts passed together.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="110" customHeight="1">
+      <x:c r="A129" s="174" t="str">
+        <x:v>QA-124</x:v>
+      </x:c>
+      <x:c r="B129" s="174" t="str">
+        <x:v>Registry</x:v>
+      </x:c>
+      <x:c r="C129" s="174" t="str">
+        <x:v>AADP registry and tier-1 dry-run validation</x:v>
+      </x:c>
+      <x:c r="D129" s="174" t="str">
+        <x:v>12 selected entries</x:v>
+      </x:c>
+      <x:c r="E129" s="174" t="str">
+        <x:v>Unified CLI dry run</x:v>
+      </x:c>
+      <x:c r="F129" s="174" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G129" s="174" t="str">
+        <x:v>T-024</x:v>
+      </x:c>
+      <x:c r="H129" s="174" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I129" s="176" t="n">
+        <x:v>46216.17</x:v>
+      </x:c>
+      <x:c r="J129" s="174" t="str">
+        <x:v>12/12 registry entries valid</x:v>
+      </x:c>
+      <x:c r="K129" s="174" t="str">
+        <x:v>The registry declares the AADP execution contract and validates before any Browserbase session is opened.</x:v>
+      </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="I130" s="164"/>
@@ -16076,7 +16363,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fea4dbefc734293"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae8902b72e7044c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17121,6 +17408,44 @@
       </x:c>
       <x:c r="L29" s="174" t="str">
         <x:v>This is a deliberate phase boundary, not a missing local feature; hosting decisions must precede remote access.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="180" customHeight="1">
+      <x:c r="A30" s="174" t="str">
+        <x:v>G-024</x:v>
+      </x:c>
+      <x:c r="B30" s="174" t="str">
+        <x:v>T-024</x:v>
+      </x:c>
+      <x:c r="C30" s="174" t="str">
+        <x:v>AADP Live Activation</x:v>
+      </x:c>
+      <x:c r="D30" s="174" t="str">
+        <x:v>AADP is enforced in the engine, but the registry currently contains observation and route-check flows rather than an approved live write-enabled Stagehand act with system-of-record proof.</x:v>
+      </x:c>
+      <x:c r="E30" s="174" t="str">
+        <x:v>The architecture prevents weak future act tests, but it has not yet demonstrated a real create/update flow end to end in an isolated QA tenant.</x:v>
+      </x:c>
+      <x:c r="F30" s="174" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="G30" s="174" t="str">
+        <x:v>Use T-025 to select a reversible workflow, provision an isolated tenant, declare allowlists and cleanup, prove the saved record by API, run repeated Browserbase sessions, and review retained evidence.</x:v>
+      </x:c>
+      <x:c r="H30" s="174" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="I30" s="174" t="str">
+        <x:v>T-025</x:v>
+      </x:c>
+      <x:c r="J30" s="174" t="str">
+        <x:v>Trevor + Codex</x:v>
+      </x:c>
+      <x:c r="K30" s="174" t="str">
+        <x:v>AADP engine, tests, and PRD published at 0e52316; live mutation intentionally not executed.</x:v>
+      </x:c>
+      <x:c r="L30" s="174" t="str">
+        <x:v>Do not point the first write journey at a customer tenant or treat a successful Stagehand act as proof of persistence.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17157,7 +17482,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13fb3d71db7244e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re75b2b86f6214432"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>